<commit_message>
Class sheet LỚP: free class and grade names, classes without a homeroom teacher
- Optional sheet LỚP (Lớp | Khối | Cơ sở 2) read into config.CLASSES; an empty
  sheet is the same as none (same rules code, same timetable).
- Grades are free names (Khối <tên>): all digits stay ints, other names are
  text; staff.grade_key sorts them, class_sort_key keeps the old order.
- A class with no homeroom teacher gets no homeroom share; the period-1 and
  homeroom-first rules skip it, HĐTN stays fixed; homeroom-only subjects
  there are an input error.
- LUẬT Khối/Lớp columns and Quản lý dạy khối accept grade and class names.
- Web UI: new step 3 Lớp (grade names, class table, take classes from
  homerooms); steps renumbered.
- Result codes unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WtuWVKdziZbvQ9VXgRdGv
</commit_message>
<xml_diff>
--- a/data/Input_Template_V8.xlsx
+++ b/data/Input_Template_V8.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NHÂN SỰ" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHƯƠNG TRÌNH HỌC" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHỨC VỤ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QUY ĐỊNH" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LUẬT" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HƯỚNG DẪN" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LỚP" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHỨC VỤ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QUY ĐỊNH" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LUẬT" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HƯỚNG DẪN" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -68,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -83,6 +84,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3114,6 +3118,959 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C300"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Lớp</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Khối</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cơ sở 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="6" t="n"/>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+    </row>
+    <row r="7" ht="25" customHeight="1">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+    </row>
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+    </row>
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="25" customHeight="1">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="5" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="5" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="5" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="5" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="5" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="5" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="5" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="5" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="5" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="5" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="5" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="5" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="5" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="5" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="5" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="5" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="5" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="5" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="5" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="5" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="5" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="5" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="5" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="5" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="5" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="5" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="5" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="5" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="5" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="5" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="5" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="5" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="5" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="5" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="5" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="5" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="5" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="5" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="5" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="5" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="5" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="5" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="5" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="5" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="5" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="5" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="5" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="5" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="5" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="5" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="5" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="5" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="5" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="5" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="5" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="5" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="5" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="5" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="5" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="5" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="5" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="5" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="5" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="5" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="5" t="n"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="5" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="5" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="5" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="5" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="5" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="5" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="5" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="5" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="5" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="5" t="n"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="5" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="5" t="n"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="5" t="n"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="5" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="5" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="5" t="n"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="5" t="n"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="5" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="5" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="5" t="n"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="5" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="5" t="n"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="5" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="5" t="n"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="5" t="n"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="5" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="5" t="n"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="5" t="n"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="5" t="n"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="5" t="n"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="5" t="n"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="5" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="5" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="5" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="5" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="5" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="5" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="5" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="5" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="5" t="n"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="5" t="n"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="5" t="n"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="5" t="n"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="5" t="n"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="5" t="n"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="5" t="n"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="5" t="n"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="5" t="n"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="5" t="n"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="5" t="n"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="5" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="5" t="n"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="5" t="n"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="5" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="5" t="n"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="5" t="n"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="5" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="5" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="5" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="5" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="5" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="5" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="5" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="5" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="5" t="n"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="5" t="n"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="5" t="n"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="5" t="n"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="5" t="n"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="5" t="n"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="5" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="5" t="n"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="5" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="5" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3178,7 +4135,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3481,7 +4438,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5290,13 +6247,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B64"/>
+  <dimension ref="A1:B65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -5359,7 +6316,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Chỉ ghi cho Chủ Nhiệm, dạng khối/số thứ tự (vd 1/1) hoặc khối rồi tên lớp (vd 1D15). Mỗi lớp một Chủ Nhiệm.</t>
+          <t>Chỉ ghi cho Chủ Nhiệm: một lớp của sheet LỚP; sheet LỚP trống thì ghi dạng khối/số thứ tự (vd 1/1) hoặc khối rồi tên lớp (vd 1D15). Mỗi lớp nhiều nhất một Chủ Nhiệm.</t>
         </is>
       </c>
     </row>
@@ -5407,7 +6364,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Dòng Chủ Nhiệm: ghi Có nếu lớp học ở cơ sở 2. Dòng khác: ghi Có nếu GV chỉ dạy ở cơ sở 2. Mỗi buổi, một GV chỉ dạy ở một cơ sở.</t>
+          <t>Dòng Chủ Nhiệm: ghi Có nếu lớp học ở cơ sở 2 (hoặc ghi ở sheet LỚP). Dòng khác: ghi Có nếu GV chỉ dạy ở cơ sở 2. Mỗi buổi, một GV chỉ dạy ở một cơ sở.</t>
         </is>
       </c>
     </row>
@@ -5443,7 +6400,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Mỗi môn một dòng: cột Môn học ghi tên môn (dùng đúng tên này ở sheet CHỨC VỤ, hoặc ở cột Chức Vụ của GV chuyên biệt chỉ dạy môn này), cột Khối k ghi số tiết/tuần của môn ở khối k (0 hoặc để trống: khối đó không học), các cột sau là quy định của môn.</t>
+          <t>Mỗi môn một dòng: cột Môn học ghi tên môn (dùng đúng tên này ở sheet CHỨC VỤ, hoặc ở cột Chức Vụ của GV chuyên biệt chỉ dạy môn này), cột Khối &lt;tên&gt; ghi số tiết/tuần của môn ở khối đó (0 hoặc để trống: khối đó không học), các cột sau là quy định của môn. Tên khối tùy ý, vd Khối 1, Khối Lá; thêm khối thì thêm cột.</t>
         </is>
       </c>
     </row>
@@ -5563,7 +6520,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Khối mà Quản Lý được dạy môn này, vd Kỹ năng sống: 4.</t>
+          <t>Khối mà Quản Lý được dạy môn này (tên khối như ở cột Khối &lt;tên&gt;), vd Kỹ năng sống: 4.</t>
         </is>
       </c>
     </row>
@@ -5738,334 +6695,346 @@
     <row r="37" ht="25" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>LUẬT</t>
+          <t>LỚP</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Mọi luật xếp TKB, mỗi dòng một luật, đọc như một câu: Với mỗi [cột Với mỗi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Mỗi luật trả lời một trong bốn câu hỏi: Ở đâu, Bao nhiêu, Đi cùng nhau, Ai dạy (các kiểu luật và phép đo xếp theo câu hỏi ở dưới). File mẫu ghi sẵn các luật có sẵn của chương trình: sửa số hoặc Điểm để chỉnh, đổi Bắt buộc, xóa dòng để bỏ luật (hoặc ghi Có ở cột Tạm tắt: chương trình bỏ qua dòng đó mà vẫn giữ lại, xóa chữ Có là dùng lại), thêm dòng để có luật mới. Cột Nhóm và Luật đọc là chỉ để đọc (chương trình ghi lại mỗi lần). Kiểu luật: một mẫu hoặc Tự ghép; cột kiểu luật không dùng để trống. Bắt buộc: Có (luật cứng) hoặc Không (ưu tiên); luật ưu tiên ghi Mức Thấp, Vừa, Cao, Rất cao (100, 400, 1500, 5000 điểm) hoặc ghi thẳng Điểm (điểm trừ mỗi lần không theo). Môn, Lớp, Khối, Ngày, Tiết ghi danh sách cách nhau bằng dấu phẩy hoặc khoảng, vd 3, 4 hoặc 3-5; Thứ 2, Thứ 4 hoặc T2-T4; 5-7. Buổi: Sáng hoặc Chiều. Giáo viên: chức vụ (Chủ Nhiệm, Bộ Môn, Quản Lý hoặc chức vụ GV chuyên biệt), 'trừ Chủ Nhiệm' là mọi giáo viên trừ chức vụ đó; hoặc một người: Mã GV (vd Bộ Môn 3, Chủ Nhiệm 1/1, đánh số theo thứ tự dòng của sheet NHÂN SỰ) hay họ tên (hai người trùng tên thì ghi Mã GV), vd giờ bận: Không xếp vào, Giáo viên Bộ Môn 3, Thứ 2, tiết 1 (để trống Môn); ép phân công: Chỉ giáo viên dạy, Môn Tiếng Anh, Lớp 3/1, Giáo viên Tiếng Anh 2. Câu đọc lại ghi Mã GV, không ghi họ tên. Nhãn, Trừ nhãn: tên các cột Có/Không của môn (vd Môn nặng) hoặc của giờ học (ngày, tiết, vd Luôn do GVCN dạy); nhiều nhãn giờ học là giờ có một trong các nhãn. Gồm môn tăng cường: Có thì Môn tính cả các môn tăng cường cùng nhóm. Không có sheet này thì chương trình dùng các luật có sẵn và sheet LUẬT RIÊNG (file của bản trước).</t>
+          <t>Không bắt buộc. Mỗi dòng một lớp: cột Lớp ghi tên lớp tùy ý (vd 1/1, 1A, Lá 2), cột Khối ghi tên khối như ở các cột Khối &lt;tên&gt; của sheet CHƯƠNG TRÌNH HỌC (vd 1 hoặc Lá; trống: các chữ số đầu tên lớp), cột Cơ sở 2 ghi Có nếu lớp học ở cơ sở 2. Có sheet này thì danh sách lớp lấy ở đây: Chủ Nhiệm ghi Lớp là một lớp của sheet, lớp không có Chủ Nhiệm vẫn được xếp (các môn chia cho GV khác; môn Chỉ GVCN dạy, tiết Luôn do GVCN dạy, tiết HĐTN cố định của GVCN không áp dụng cho lớp đó). Không có sheet này (hoặc sheet trống) thì lớp là lớp của các dòng Chủ Nhiệm, ghi dạng khối/số thứ tự (1/1) hoặc khối rồi tên lớp (1A).</t>
         </is>
       </c>
     </row>
     <row r="38" ht="25" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Không xếp vào</t>
+          <t>LUẬT</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Môn (của các khối ở cột Khối; để trống: mọi khối) không xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục không xếp vào tiết 1; Tin học không xếp vào Thứ 2. Ghi Giáo viên (chức vụ, Mã GV hoặc họ tên) thì chỉ xét tiết của người đó, để trống Môn là mọi môn: giờ bận, vd Bộ Môn 3 không dạy Thứ 2 tiết 1.</t>
+          <t>Mọi luật xếp TKB, mỗi dòng một luật, đọc như một câu: Với mỗi [cột Với mỗi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Mỗi luật trả lời một trong bốn câu hỏi: Ở đâu, Bao nhiêu, Đi cùng nhau, Ai dạy (các kiểu luật và phép đo xếp theo câu hỏi ở dưới). File mẫu ghi sẵn các luật có sẵn của chương trình: sửa số hoặc Điểm để chỉnh, đổi Bắt buộc, xóa dòng để bỏ luật (hoặc ghi Có ở cột Tạm tắt: chương trình bỏ qua dòng đó mà vẫn giữ lại, xóa chữ Có là dùng lại), thêm dòng để có luật mới. Cột Nhóm và Luật đọc là chỉ để đọc (chương trình ghi lại mỗi lần). Kiểu luật: một mẫu hoặc Tự ghép; cột kiểu luật không dùng để trống. Bắt buộc: Có (luật cứng) hoặc Không (ưu tiên); luật ưu tiên ghi Mức Thấp, Vừa, Cao, Rất cao (100, 400, 1500, 5000 điểm) hoặc ghi thẳng Điểm (điểm trừ mỗi lần không theo). Môn, Lớp, Khối, Ngày, Tiết ghi danh sách cách nhau bằng dấu phẩy hoặc khoảng, vd 3, 4 hoặc 3-5; Thứ 2, Thứ 4 hoặc T2-T4; 5-7. Buổi: Sáng hoặc Chiều. Giáo viên: chức vụ (Chủ Nhiệm, Bộ Môn, Quản Lý hoặc chức vụ GV chuyên biệt), 'trừ Chủ Nhiệm' là mọi giáo viên trừ chức vụ đó; hoặc một người: Mã GV (vd Bộ Môn 3, Chủ Nhiệm 1/1, đánh số theo thứ tự dòng của sheet NHÂN SỰ) hay họ tên (hai người trùng tên thì ghi Mã GV), vd giờ bận: Không xếp vào, Giáo viên Bộ Môn 3, Thứ 2, tiết 1 (để trống Môn); ép phân công: Chỉ giáo viên dạy, Môn Tiếng Anh, Lớp 3/1, Giáo viên Tiếng Anh 2. Câu đọc lại ghi Mã GV, không ghi họ tên. Nhãn, Trừ nhãn: tên các cột Có/Không của môn (vd Môn nặng) hoặc của giờ học (ngày, tiết, vd Luôn do GVCN dạy); nhiều nhãn giờ học là giờ có một trong các nhãn. Gồm môn tăng cường: Có thì Môn tính cả các môn tăng cường cùng nhóm. Không có sheet này thì chương trình dùng các luật có sẵn và sheet LUẬT RIÊNG (file của bản trước).</t>
         </is>
       </c>
     </row>
     <row r="39" ht="25" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Chỉ xếp vào</t>
+          <t>LUẬT: Ở đâu · Không xếp vào</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Môn chỉ xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục chỉ xếp vào buổi chiều. Ghi Giáo viên thì chỉ xét tiết của người đó (để trống Môn: mọi môn), vd Bộ Môn 3 chỉ dạy buổi sáng.</t>
+          <t>Môn (của các khối ở cột Khối; để trống: mọi khối) không xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục không xếp vào tiết 1; Tin học không xếp vào Thứ 2. Ghi Giáo viên (chức vụ, Mã GV hoặc họ tên) thì chỉ xét tiết của người đó, để trống Môn là mọi môn: giờ bận, vd Bộ Môn 3 không dạy Thứ 2 tiết 1.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="25" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Cố định vào</t>
+          <t>LUẬT: Ở đâu · Chỉ xếp vào</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Mỗi lớp (của các khối, lớp ghi ở dòng này) học đúng 1 tiết của Môn ở mỗi giờ ghi ở cột Ngày, Tiết, Buổi, vd Thể dục khối 1 cố định vào Thứ 3 tiết 3.</t>
+          <t>Môn chỉ xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục chỉ xếp vào buổi chiều. Ghi Giáo viên thì chỉ xét tiết của người đó (để trống Môn: mọi môn), vd Bộ Môn 3 chỉ dạy buổi sáng.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="25" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Giáo viên tối đa tiết mỗi ngày</t>
+          <t>LUẬT: Ở đâu · Cố định vào</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số tiết mỗi ngày.</t>
+          <t>Mỗi lớp (của các khối, lớp ghi ở dòng này) học đúng 1 tiết của Môn ở mỗi giờ ghi ở cột Ngày, Tiết, Buổi, vd Thể dục khối 1 cố định vào Thứ 3 tiết 3.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="25" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Giáo viên tối đa lớp mỗi ngày</t>
+          <t>LUẬT: Bao nhiêu · Giáo viên tối đa tiết mỗi ngày</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số lớp khác nhau mỗi ngày.</t>
+          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số tiết mỗi ngày.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="25" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Số lớp học cùng lúc tối đa</t>
+          <t>LUẬT: Bao nhiêu · Giáo viên tối đa lớp mỗi ngày</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Môn có tối đa Số lớp học cùng một giờ (cả trường, hoặc các khối ở cột Khối), vd phòng Tin học: 1, sân Thể dục: 2.</t>
+          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số lớp khác nhau mỗi ngày.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="25" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Học ít nhất số ngày</t>
+          <t>LUẬT: Bao nhiêu · Số lớp học cùng lúc tối đa</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Mỗi lớp học Môn ở ít nhất Số ngày khác nhau trong tuần, vd Tiếng Anh ít nhất 3 ngày.</t>
+          <t>Môn có tối đa Số lớp học cùng một giờ (cả trường, hoặc các khối ở cột Khối), vd phòng Tin học: 1, sân Thể dục: 2.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="25" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Học 2 tiết liền</t>
+          <t>LUẬT: Bao nhiêu · Học ít nhất số ngày</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Môn học thành cặp 2 tiết liền, cùng người dạy: mỗi buổi 0 hoặc 2 tiết của môn (tính chung môn tăng cường cùng nhóm), vd Tiếng Anh. Bắt buộc thì số tiết/tuần phải chẵn.</t>
+          <t>Mỗi lớp học Môn ở ít nhất Số ngày khác nhau trong tuần, vd Tiếng Anh ít nhất 3 ngày.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="25" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Học trước</t>
+          <t>LUẬT: Đi cùng nhau · Học 2 tiết liền</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Trong một buổi có cả hai môn thì Môn học trước Môn thứ hai, vd Tiếng Việt trước Toán.</t>
+          <t>Môn học thành cặp 2 tiết liền, cùng người dạy: mỗi buổi 0 hoặc 2 tiết của môn (tính chung môn tăng cường cùng nhóm), vd Tiếng Anh. Bắt buộc thì số tiết/tuần phải chẵn.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="25" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Chỉ giáo viên dạy</t>
+          <t>LUẬT: Đi cùng nhau · Học trước</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Các tiết của Môn (ở các khối, lớp, ngày, tiết ghi ở dòng này) chỉ do giáo viên ghi ở cột Giáo viên dạy: chức vụ, vd Tin học khối 3 chỉ GV Tin Học dạy; hoặc một người (Mã GV hay họ tên) để chọn ai dạy lớp nào, vd Tiếng Anh lớp 3/1 chỉ Tiếng Anh 2 dạy.</t>
+          <t>Trong một buổi có cả hai môn thì Môn học trước Môn thứ hai, vd Tiếng Việt trước Toán.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="25" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Buổi nghỉ của giáo viên</t>
+          <t>LUẬT: Ai dạy · Chỉ giáo viên dạy</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Giáo viên không dạy vào các buổi nghỉ ghi ở cột Buổi Nghỉ (sheet NHÂN SỰ) và nghỉ đủ số buổi ghi ở đó. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
+          <t>Các tiết của Môn (ở các khối, lớp, ngày, tiết ghi ở dòng này) chỉ do giáo viên ghi ở cột Giáo viên dạy: chức vụ, vd Tin học khối 3 chỉ GV Tin Học dạy; hoặc một người (Mã GV hay họ tên) để chọn ai dạy lớp nào, vd Tiếng Anh lớp 3/1 chỉ Tiếng Anh 2 dạy.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="25" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Giáo viên chỉ dạy cơ sở 2</t>
+          <t>LUẬT: Ai dạy · Buổi nghỉ của giáo viên</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Giáo viên không chủ nhiệm ghi Có ở cột Cơ sở 2 hoặc Thai Sản (sheet NHÂN SỰ) chỉ dạy các lớp ở cơ sở 2. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
+          <t>Giáo viên không dạy vào các buổi nghỉ ghi ở cột Buổi Nghỉ (sheet NHÂN SỰ) và nghỉ đủ số buổi ghi ở đó. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="25" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép</t>
+          <t>LUẬT: Ai dạy · Giáo viên chỉ dạy cơ sở 2</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Tự ghép câu luật: Với mỗi [phạm vi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Xem các phép đo ở dưới.</t>
+          <t>Giáo viên không chủ nhiệm ghi Có ở cột Cơ sở 2 hoặc Thai Sản (sheet NHÂN SỰ) chỉ dạy các lớp ở cơ sở 2. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="25" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Với mỗi</t>
+          <t>LUẬT: Tự ghép</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Chia các tiết thành từng nhóm theo các chiều, vd 'Lớp, Ngày': luật áp dụng cho mỗi lớp mỗi ngày. Các chiều: Lớp, Giáo viên, Môn, Nhóm môn, Khối, Ngày, Buổi, Giờ học, Cơ sở. Trống: cả trường cả tuần.</t>
+          <t>Tự ghép câu luật: Với mỗi [phạm vi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Xem các phép đo ở dưới.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="25" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Tự ghép, Phép đo Vị trí</t>
+          <t>LUẬT: Tự ghép, cột Với mỗi</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Các tiết chỉ xếp vào, hoặc không xếp vào, các ngày, tiết, buổi (hoặc giờ có nhãn) ghi ở dòng này. So sánh: Chỉ trong, Không trong.</t>
+          <t>Chia các tiết thành từng nhóm theo các chiều, vd 'Lớp, Ngày': luật áp dụng cho mỗi lớp mỗi ngày. Các chiều: Lớp, Giáo viên, Môn, Nhóm môn, Khối, Ngày, Buổi, Giờ học, Cơ sở. Trống: cả trường cả tuần.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="25" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số tiết</t>
+          <t>LUẬT: Ở đâu · Tự ghép, Phép đo Vị trí</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Đếm số tiết trong mỗi phạm vi, vd mỗi lớp mỗi ngày học tối đa 1 tiết Toán; mỗi giờ học có tối đa 1 tiết Tin học. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số.</t>
+          <t>Các tiết chỉ xếp vào, hoặc không xếp vào, các ngày, tiết, buổi (hoặc giờ có nhãn) ghi ở dòng này. So sánh: Chỉ trong, Không trong.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="25" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số khác nhau</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số tiết</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Đếm số lớp, ngày, cơ sở… khác nhau (cột Đếm theo), vd mỗi giáo viên mỗi ngày dạy tối đa 3 lớp; mỗi lớp học Tiếng Anh ít nhất 3 ngày. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số. Ghi cột Đếm theo.</t>
+          <t>Đếm số tiết trong mỗi phạm vi, vd mỗi lớp mỗi ngày học tối đa 1 tiết Toán; mỗi giờ học có tối đa 1 tiết Tin học. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="25" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Khoảng cách</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số khác nhau</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Số tiết trống xen giữa các tiết trong buổi (0: không có tiết trống); hoặc số tiết từ tiết đó đến cuối buổi (0: ở tiết cuối buổi). So sánh: Tiết trống tối đa, Cách cuối buổi tối đa. Ghi cột Số.</t>
+          <t>Đếm số lớp, ngày, cơ sở… khác nhau (cột Đếm theo), vd mỗi giáo viên mỗi ngày dạy tối đa 3 lớp; mỗi lớp học Tiếng Anh ít nhất 3 ngày. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số. Ghi cột Đếm theo.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="25" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Liền nhau</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Khoảng cách</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Các tiết trong một buổi (của mỗi lớp hoặc giáo viên) đứng liền nhau, không có tiết khác xen giữa.</t>
+          <t>Số tiết trống xen giữa các tiết trong buổi (0: không có tiết trống); hoặc số tiết từ tiết đó đến cuối buổi (0: ở tiết cuối buổi). So sánh: Tiết trống tối đa, Cách cuối buổi tối đa. Ghi cột Số.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="25" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Theo cặp 2 tiết</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Liền nhau</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Mỗi buổi học 0 hoặc 2 tiết, 2 tiết đó liền nhau (ưu tiên: hạn chế tiết lẻ đứng một mình).</t>
+          <t>Các tiết trong một buổi (của mỗi lớp hoặc giáo viên) đứng liền nhau, không có tiết khác xen giữa.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="25" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Thứ tự</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Theo cặp 2 tiết</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Trong một buổi (hoặc ngày, nếu Với mỗi có Ngày) tiết của Môn đứng trước (hoặc sau) tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm. So sánh: Trước, Sau.</t>
+          <t>Mỗi buổi học 0 hoặc 2 tiết, 2 tiết đó liền nhau (ưu tiên: hạn chế tiết lẻ đứng một mình).</t>
         </is>
       </c>
     </row>
     <row r="59" ht="25" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Đi kèm</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Thứ tự</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Buổi (hoặc ngày) có tiết của Môn thì cũng có tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm.</t>
+          <t>Trong một buổi (hoặc ngày, nếu Với mỗi có Ngày) tiết của Môn đứng trước (hoặc sau) tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm. So sánh: Trước, Sau.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="25" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Tự ghép, Phép đo Người dạy</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Đi kèm</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Các tiết do giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên) dạy; hoặc do cùng một người dạy; hoặc hai tiết liền nhau do cùng một người; hoặc tiết đầu tuần do giáo viên đó dạy, tiết của người khác không đứng trước. So sánh: Do, Cùng một người, Liền nhau cùng người, Tiết đầu tuần do.</t>
+          <t>Buổi (hoặc ngày) có tiết của Môn thì cũng có tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="25" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Số</t>
+          <t>LUẬT: Ai dạy · Tự ghép, Phép đo Người dạy</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Một số nguyên, hoặc (phép đo Số tiết) một ngưỡng theo dữ liệu: tải ngày, tải ngày + 1, số tiết/tuần chia số ngày (tải ngày: định mức của giáo viên chia theo số tiết của ngày).</t>
+          <t>Các tiết do giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên) dạy; hoặc do cùng một người dạy; hoặc hai tiết liền nhau do cùng một người; hoặc tiết đầu tuần do giáo viên đó dạy, tiết của người khác không đứng trước. So sánh: Do, Cùng một người, Liền nhau cùng người, Tiết đầu tuần do.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="25" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Áp dụng khi</t>
+          <t>LUẬT: Tự ghép, cột Số</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Chỉ áp dụng khi số tiết/tuần của các môn ở cột Môn (phạm vi có Môn, Nhóm môn: của từng môn, nhóm môn) ở khối đó thỏa điều kiện, vd '&gt;= 6, chẵn' (từ 6 tiết trở lên và chẵn) hoặc '&lt;= số ngày' (không quá số ngày học).</t>
+          <t>Một số nguyên, hoặc (phép đo Số tiết) một ngưỡng theo dữ liệu: tải ngày, tải ngày + 1, số tiết/tuần chia số ngày (tải ngày: định mức của giáo viên chia theo số tiết của ngày).</t>
         </is>
       </c>
     </row>
     <row r="63" ht="25" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: cấu trúc của TKB</t>
+          <t>LUẬT: Tự ghép, cột Áp dụng khi</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Cấu trúc của TKB (không phải luật, luôn có): mỗi lớp mỗi giờ học một tiết; mỗi lớp học đủ số tiết của chương trình học; giáo viên không dạy hai nơi cùng lúc, dạy không quá định mức (cộng số tiết bù tối đa ở chế độ bù giờ), Quản Lý dạy đúng định mức; giáo viên chỉ dạy các môn chức vụ được dạy (sheet CHƯƠNG TRÌNH HỌC, CHỨC VỤ).</t>
+          <t>Chỉ áp dụng khi số tiết/tuần của các môn ở cột Môn (phạm vi có Môn, Nhóm môn: của từng môn, nhóm môn) ở khối đó thỏa điều kiện, vd '&gt;= 6, chẵn' (từ 6 tiết trở lên và chẵn) hoặc '&lt;= số ngày' (không quá số ngày học).</t>
         </is>
       </c>
     </row>
     <row r="64" ht="25" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
+          <t>LUẬT: cấu trúc của TKB</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Cấu trúc của TKB (không phải luật, luôn có): mỗi lớp mỗi giờ học một tiết; mỗi lớp học đủ số tiết của chương trình học; giáo viên không dạy hai nơi cùng lúc, dạy không quá định mức (cộng số tiết bù tối đa ở chế độ bù giờ), Quản Lý dạy đúng định mức; giáo viên chỉ dạy các môn chức vụ được dạy (sheet CHƯƠNG TRÌNH HỌC, CHỨC VỤ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="25" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
           <t>Kiểu chữ</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>Các file kết quả chép kiểu chữ, cỡ chữ, viền của sheet NHÂN SỰ. Chỉ cần chữ và số: không cần công thức, màu nền, ghi chú trong ô hay danh sách thả xuống.</t>
         </is>

</xml_diff>

<commit_message>
Extra roles column: one person can hold several roles
Optional staff column "Chức Vụ Thêm" lists more roles (Bộ Môn or specialist
roles) a person also holds; who may teach is the union of the roles, in any
class. A homeroom teacher with extra roles takes only the priority subjects
(plus same-group ones) and uses the rest of the quota like a general teacher;
overtime and hires follow the subject's role. A homeroom teacher with extra
"Bộ Môn" is how a school drops "homeroom teachers only teach their class" per
person. Rule role names match extra roles. The web UI picks extra roles with
check boxes in the teacher dialog. Empty column: same codes as before.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WtuWVKdziZbvQ9VXgRdGv
</commit_message>
<xml_diff>
--- a/data/Input_Template_V8.xlsx
+++ b/data/Input_Template_V8.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I300"/>
+  <dimension ref="A1:J300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -464,6 +464,7 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -510,6 +511,11 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Buổi Nghỉ</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Chức Vụ Thêm</t>
         </is>
       </c>
     </row>
@@ -523,6 +529,7 @@
       <c r="G2" s="3" t="n"/>
       <c r="H2" s="4" t="n"/>
       <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
     </row>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -534,6 +541,7 @@
       <c r="G3" s="3" t="n"/>
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="2" t="n"/>
@@ -545,6 +553,7 @@
       <c r="G4" s="3" t="n"/>
       <c r="H4" s="4" t="n"/>
       <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
     </row>
     <row r="5" ht="25" customHeight="1">
       <c r="A5" s="2" t="n"/>
@@ -556,6 +565,7 @@
       <c r="G5" s="3" t="n"/>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
     </row>
     <row r="6" ht="25" customHeight="1">
       <c r="A6" s="2" t="n"/>
@@ -567,6 +577,7 @@
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
     </row>
     <row r="7" ht="25" customHeight="1">
       <c r="A7" s="2" t="n"/>
@@ -578,6 +589,7 @@
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="4" t="n"/>
       <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
     </row>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="2" t="n"/>
@@ -589,6 +601,7 @@
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
     </row>
     <row r="9" ht="25" customHeight="1">
       <c r="A9" s="2" t="n"/>
@@ -600,6 +613,7 @@
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
     </row>
     <row r="10" ht="25" customHeight="1">
       <c r="A10" s="2" t="n"/>
@@ -611,6 +625,7 @@
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="4" t="n"/>
       <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
     </row>
     <row r="11" ht="25" customHeight="1">
       <c r="A11" s="2" t="n"/>
@@ -622,6 +637,7 @@
       <c r="G11" s="3" t="n"/>
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="C12" s="5" t="n"/>
@@ -6253,7 +6269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B65"/>
+  <dimension ref="A1:B66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -6280,7 +6296,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên một dòng. Năm cột Thai Sản, Hợp Đồng, Cơ sở 2, Lớp Đang Dạy, Buổi Nghỉ không bắt buộc (để trống hoặc xóa cột).</t>
+          <t>Mỗi giáo viên một dòng. Sáu cột Thai Sản, Hợp Đồng, Cơ sở 2, Lớp Đang Dạy, Buổi Nghỉ, Chức Vụ Thêm không bắt buộc (để trống hoặc xóa cột).</t>
         </is>
       </c>
     </row>
@@ -6395,646 +6411,658 @@
     <row r="12" ht="25" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC</t>
+          <t>NHÂN SỰ: Chức Vụ Thêm</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Mỗi môn một dòng: cột Môn học ghi tên môn (dùng đúng tên này ở sheet CHỨC VỤ, hoặc ở cột Chức Vụ của GV chuyên biệt chỉ dạy môn này), cột Khối &lt;tên&gt; ghi số tiết/tuần của môn ở khối đó (0 hoặc để trống: khối đó không học), các cột sau là quy định của môn. Tên khối tùy ý, vd Khối 1, Khối Lá; thêm khối thì thêm cột.</t>
+          <t>Các chức vụ khác người này cũng giữ, cách nhau bằng dấu phẩy: Bộ Môn hoặc chức vụ GV chuyên biệt (vd Tiếng Anh). Người đó dạy được cả các môn của các chức vụ này, ở mọi lớp, trong định mức; vd Chủ Nhiệm ghi Bộ Môn thì dạy được cả các lớp khác. Chủ Nhiệm có chức vụ thêm dạy phần GVCN nhận trọn của lớp mình (không nhận thêm cho đủ định mức), phần định mức còn lại dùng cho chức vụ thêm. Mã GV theo chức vụ chính (cột Chức Vụ).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="25" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Quy ước các ô quy định</t>
+          <t>CHƯƠNG TRÌNH HỌC</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Mỗi quy định là một cột (bảng Quy định chung: một dòng). Mỗi ô chỉ ghi Có, Không hoặc một số nguyên dương; ô trống là Không. Riêng cột Tên trong TKB ghi chữ. Xóa một cột (một dòng của bảng chung, một bảng, hoặc cả sheet QUY ĐỊNH) thì quy định đó dùng giá trị mặc định của chương trình.</t>
+          <t>Mỗi môn một dòng: cột Môn học ghi tên môn (dùng đúng tên này ở sheet CHỨC VỤ, hoặc ở cột Chức Vụ của GV chuyên biệt chỉ dạy môn này), cột Khối &lt;tên&gt; ghi số tiết/tuần của môn ở khối đó (0 hoặc để trống: khối đó không học), các cột sau là quy định của môn. Tên khối tùy ý, vd Khối 1, Khối Lá; thêm khối thì thêm cột.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="25" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH</t>
+          <t>Quy ước các ô quy định</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Ba bảng cách nhau một dòng trống: Quy định | Giá trị; Ngày (mỗi dòng một ngày học, mỗi cột Buổi &lt;tên&gt; ghi số tiết của buổi đó); Tiết (đánh số liên tục trong ngày: sáng 4 tiết thì chiều từ tiết 5; ngày dài nhất có bao nhiêu tiết thì bấy nhiêu dòng).</t>
+          <t>Mỗi quy định là một cột (bảng Quy định chung: một dòng). Mỗi ô chỉ ghi Có, Không hoặc một số nguyên dương; ô trống là Không. Riêng cột Tên trong TKB ghi chữ. Xóa một cột (một dòng của bảng chung, một bảng, hoặc cả sheet QUY ĐỊNH) thì quy định đó dùng giá trị mặc định của chương trình.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="25" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Tên trong TKB</t>
+          <t>QUY ĐỊNH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Chữ ghi trong ô TKB (cột duy nhất ghi chữ); trống: ghi đúng tên môn.</t>
+          <t>Ba bảng cách nhau một dòng trống: Quy định | Giá trị; Ngày (mỗi dòng một ngày học, mỗi cột Buổi &lt;tên&gt; ghi số tiết của buổi đó); Tiết (đánh số liên tục trong ngày: sáng 4 tiết thì chiều từ tiết 5; ngày dài nhất có bao nhiêu tiết thì bấy nhiêu dòng).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="25" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Môn HĐTN</t>
+          <t>CHƯƠNG TRÌNH HỌC: Tên trong TKB</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Có ở một môn: môn chào cờ, sinh hoạt lớp, có tiết cố định ở bảng ngày của sheet QUY ĐỊNH.</t>
+          <t>Chữ ghi trong ô TKB (cột duy nhất ghi chữ); trống: ghi đúng tên môn.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="25" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận trọn</t>
+          <t>CHƯƠNG TRÌNH HỌC: Môn HĐTN</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>GVCN nhận hết các môn này của lớp mình; luật cứng: môn nào phải chia cho người khác thì tiết đầu tiên trong tuần do GVCN dạy.</t>
+          <t>Có ở một môn: môn chào cờ, sinh hoạt lớp, có tiết cố định ở bảng ngày của sheet QUY ĐỊNH.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="25" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN cắt bớt</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận trọn</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Số thứ tự 1, 2...: môn cắt trước khi các môn nhận trọn vượt định mức GVCN; mỗi môn GVCN giữ ít nhất 1 tiết.</t>
+          <t>GVCN nhận hết các môn này của lớp mình; luật cứng: môn nào phải chia cho người khác thì tiết đầu tiên trong tuần do GVCN dạy.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="25" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận thêm</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN cắt bớt</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Số thứ tự 1, 2...: môn GVCN nhận thêm trước cho đủ định mức (không nhận môn của GV chuyên biệt).</t>
+          <t>Số thứ tự 1, 2...: môn cắt trước khi các môn nhận trọn vượt định mức GVCN; mỗi môn GVCN giữ ít nhất 1 tiết.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Chỉ GVCN dạy</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận thêm</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: chỉ GVCN của lớp được dạy.</t>
+          <t>Số thứ tự 1, 2...: môn GVCN nhận thêm trước cho đủ định mức (không nhận môn của GV chuyên biệt).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Bộ Môn không dạy</t>
+          <t>CHƯƠNG TRÌNH HỌC: Chỉ GVCN dạy</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>GV bộ môn không dạy môn này; trường chưa có GV chuyên biệt của môn thì chương trình tuyển thêm. Ghi theo ngoại lệ để môn mới (ô trống) mặc nhiên bộ môn dạy được.</t>
+          <t>Luật cứng: chỉ GVCN của lớp được dạy.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Quản lý dạy khối</t>
+          <t>CHƯƠNG TRÌNH HỌC: Bộ Môn không dạy</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Khối mà Quản Lý được dạy môn này (tên khối như ở cột Khối &lt;tên&gt;), vd Kỹ năng sống: 4.</t>
+          <t>GV bộ môn không dạy môn này; trường chưa có GV chuyên biệt của môn thì chương trình tuyển thêm. Ghi theo ngoại lệ để môn mới (ô trống) mặc nhiên bộ môn dạy được.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="25" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN bù môn chuyên biệt</t>
+          <t>CHƯƠNG TRÌNH HỌC: Quản lý dạy khối</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Môn có GV chuyên biệt mà GVCN vẫn được dạy bù ở lớp mình (nhận sau cùng).</t>
+          <t>Khối mà Quản Lý được dạy môn này (tên khối như ở cột Khối &lt;tên&gt;), vd Kỹ năng sống: 4.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="25" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Nhóm môn</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN bù môn chuyên biệt</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Môn chính và các môn tăng cường của nó ghi cùng một số, vd Tiếng Việt và Tiếng Việt tăng cường: 1.</t>
+          <t>Môn có GV chuyên biệt mà GVCN vẫn được dạy bù ở lớp mình (nhận sau cùng).</t>
         </is>
       </c>
     </row>
     <row r="25" ht="25" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Môn tăng cường</t>
+          <t>CHƯƠNG TRÌNH HỌC: Nhóm môn</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Có ở môn tăng cường của nhóm; luật cứng: tiết tăng cường đứng sau mọi tiết môn chính trong ngày và ngày đó phải có tiết môn chính; cả nhóm tính chung cho giới hạn mỗi buổi và ghép cặp.</t>
+          <t>Môn chính và các môn tăng cường của nó ghi cùng một số, vd Tiếng Việt và Tiếng Việt tăng cường: 1.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="25" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Không ghép cặp</t>
+          <t>CHƯƠNG TRÌNH HỌC: Môn tăng cường</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Nhóm môn (ghi ở môn chính) không xếp thành cặp 2 tiết liền. Ghi theo ngoại lệ như cột Bộ Môn không dạy.</t>
+          <t>Có ở môn tăng cường của nhóm; luật cứng: tiết tăng cường đứng sau mọi tiết môn chính trong ngày và ngày đó phải có tiết môn chính; cả nhóm tính chung cho giới hạn mỗi buổi và ghép cặp.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="25" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Môn nặng</t>
+          <t>CHƯƠNG TRÌNH HỌC: Không ghép cặp</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu mềm: hạn chế xếp vào các tiết Hạn chế môn nặng (sheet QUY ĐỊNH).</t>
+          <t>Nhóm môn (ghi ở môn chính) không xếp thành cặp 2 tiết liền. Ghi theo ngoại lệ như cột Bộ Môn không dạy.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="25" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Ưu tiên buổi sáng</t>
+          <t>CHƯƠNG TRÌNH HỌC: Môn nặng</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu mềm: mỗi tiết ở buổi chiều bị trừ điểm, và môn được rải đều hơn trong tuần.</t>
+          <t>Mục tiêu mềm: hạn chế xếp vào các tiết Hạn chế môn nặng (sheet QUY ĐỊNH).</t>
         </is>
       </c>
     </row>
     <row r="29" ht="25" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Chủ Nhiệm được dạy bù</t>
+          <t>CHƯƠNG TRÌNH HỌC: Ưu tiên buổi sáng</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>GVCN chỉ bù ở lớp mình và bù trước bộ môn.</t>
+          <t>Mục tiêu mềm: mỗi tiết ở buổi chiều bị trừ điểm, và môn được rải đều hơn trong tuần.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="25" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Bộ Môn được dạy bù</t>
+          <t>QUY ĐỊNH: Chủ Nhiệm được dạy bù</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Bộ môn bù khi GVCN đã bù hết mức.</t>
+          <t>GVCN chỉ bù ở lớp mình và bù trước bộ môn.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="25" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Ngày, Buổi &lt;tên buổi&gt;</t>
+          <t>QUY ĐỊNH: Bộ Môn được dạy bù</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Bảng Ngày: mỗi dòng một ngày học, tên tùy ý (vd Thứ 2, Thứ 7, Chủ nhật), theo thứ tự trong tuần. Mỗi cột Buổi &lt;tên buổi&gt; (vd Buổi Sáng, Buổi Chiều, Buổi Tối) ghi số tiết của buổi đó trong ngày; ô trống là ngày đó không học buổi đó. Mỗi ngày một số tiết riêng được (vd chiều Thứ 5 có 4 tiết). Thêm buổi thì thêm cột, thêm ngày học thì thêm dòng; ngày không có tiết nào không phải ngày học. Tiết đánh số liên tục trong ngày theo thứ tự các cột buổi: sáng 4 tiết thì chiều bắt đầu từ tiết 5.</t>
+          <t>Bộ môn bù khi GVCN đã bù hết mức.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="25" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Tiết HĐTN cố định</t>
+          <t>QUY ĐỊNH: Ngày, Buổi &lt;tên buổi&gt;</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: tiết môn HĐTN cố định của ngày đó ở mọi lớp, vd Thứ 2: 1, Thứ 6: 4.</t>
+          <t>Bảng Ngày: mỗi dòng một ngày học, tên tùy ý (vd Thứ 2, Thứ 7, Chủ nhật), theo thứ tự trong tuần. Mỗi cột Buổi &lt;tên buổi&gt; (vd Buổi Sáng, Buổi Chiều, Buổi Tối) ghi số tiết của buổi đó trong ngày; ô trống là ngày đó không học buổi đó. Mỗi ngày một số tiết riêng được (vd chiều Thứ 5 có 4 tiết). Thêm buổi thì thêm cột, thêm ngày học thì thêm dòng; ngày không có tiết nào không phải ngày học. Tiết đánh số liên tục trong ngày theo thứ tự các cột buổi: sáng 4 tiết thì chiều bắt đầu từ tiết 5.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="25" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Xếp tiết HĐTN còn lại</t>
+          <t>QUY ĐỊNH: Tiết HĐTN cố định</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: các tiết HĐTN còn lại chỉ xếp vào các ngày này (mục tiêu mềm: gần cuối buổi).</t>
+          <t>Luật cứng: tiết môn HĐTN cố định của ngày đó ở mọi lớp, vd Thứ 2: 1, Thứ 6: 4.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="25" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Luôn do GVCN dạy</t>
+          <t>QUY ĐỊNH: Xếp tiết HĐTN còn lại</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: tiết này ở mọi ngày do GVCN của lớp dạy.</t>
+          <t>Luật cứng: các tiết HĐTN còn lại chỉ xếp vào các ngày này (mục tiêu mềm: gần cuối buổi).</t>
         </is>
       </c>
     </row>
     <row r="35" ht="25" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Hạn chế môn nặng</t>
+          <t>QUY ĐỊNH: Luôn do GVCN dạy</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu mềm: mỗi tiết môn nặng ở tiết này bị trừ điểm.</t>
+          <t>Luật cứng: tiết này ở mọi ngày do GVCN của lớp dạy.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="25" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>CHỨC VỤ</t>
+          <t>QUY ĐỊNH: Hạn chế môn nặng</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Không bắt buộc. Mỗi dòng một chức vụ GV chuyên biệt nhà trường tự đặt: cột Chức vụ ghi tên (không ghi số, không trùng Chủ Nhiệm, Bộ Môn, Quản Lý), cột Môn được dạy ghi các môn chức vụ đó dạy, cách nhau bằng dấu phẩy, đúng tên trong sheet CHƯƠNG TRÌNH HỌC, vd GV Nghệ thuật: Âm nhạc, Mỹ thuật. Ở sheet NHÂN SỰ, GV có Chức Vụ là tên đó chỉ dạy các môn này. Chức vụ không ghi ở đây mà trùng tên một môn (vd Tiếng Anh) thì chỉ dạy môn đó. Môn Bộ Môn không dạy mà chưa có GV nào dạy được thì chương trình tuyển thêm chức vụ đầu tiên ở đây dạy môn đó (không có thì chức vụ trùng tên môn).</t>
+          <t>Mục tiêu mềm: mỗi tiết môn nặng ở tiết này bị trừ điểm.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="25" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>LỚP</t>
+          <t>CHỨC VỤ</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Không bắt buộc. Mỗi dòng một lớp: cột Lớp ghi tên lớp tùy ý (vd 1/1, 1A, Lá 2), cột Khối ghi tên khối như ở các cột Khối &lt;tên&gt; của sheet CHƯƠNG TRÌNH HỌC (vd 1 hoặc Lá; trống: các chữ số đầu tên lớp), cột Cơ sở 2 ghi Có nếu lớp học ở cơ sở 2. Có sheet này thì danh sách lớp lấy ở đây: Chủ Nhiệm ghi Lớp là một lớp của sheet, lớp không có Chủ Nhiệm vẫn được xếp (các môn chia cho GV khác; môn Chỉ GVCN dạy, tiết Luôn do GVCN dạy, tiết HĐTN cố định của GVCN không áp dụng cho lớp đó). Không có sheet này (hoặc sheet trống) thì lớp là lớp của các dòng Chủ Nhiệm, ghi dạng khối/số thứ tự (1/1) hoặc khối rồi tên lớp (1A).</t>
+          <t>Không bắt buộc. Mỗi dòng một chức vụ GV chuyên biệt nhà trường tự đặt: cột Chức vụ ghi tên (không ghi số, không trùng Chủ Nhiệm, Bộ Môn, Quản Lý), cột Môn được dạy ghi các môn chức vụ đó dạy, cách nhau bằng dấu phẩy, đúng tên trong sheet CHƯƠNG TRÌNH HỌC, vd GV Nghệ thuật: Âm nhạc, Mỹ thuật. Ở sheet NHÂN SỰ, GV có Chức Vụ là tên đó chỉ dạy các môn này. Chức vụ không ghi ở đây mà trùng tên một môn (vd Tiếng Anh) thì chỉ dạy môn đó. Môn Bộ Môn không dạy mà chưa có GV nào dạy được thì chương trình tuyển thêm chức vụ đầu tiên ở đây dạy môn đó (không có thì chức vụ trùng tên môn).</t>
         </is>
       </c>
     </row>
     <row r="38" ht="25" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>LUẬT</t>
+          <t>LỚP</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Mọi luật xếp TKB, mỗi dòng một luật, đọc như một câu: Với mỗi [cột Với mỗi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Mỗi luật trả lời một trong bốn câu hỏi: Ở đâu, Bao nhiêu, Đi cùng nhau, Ai dạy (các kiểu luật và phép đo xếp theo câu hỏi ở dưới). File mẫu ghi sẵn các luật có sẵn của chương trình: sửa số hoặc Điểm để chỉnh, đổi Bắt buộc, xóa dòng để bỏ luật (hoặc ghi Có ở cột Tạm tắt: chương trình bỏ qua dòng đó mà vẫn giữ lại, xóa chữ Có là dùng lại), thêm dòng để có luật mới. Cột Nhóm và Luật đọc là chỉ để đọc (chương trình ghi lại mỗi lần). Kiểu luật: một mẫu hoặc Tự ghép; cột kiểu luật không dùng để trống. Bắt buộc: Có (luật cứng) hoặc Không (ưu tiên); luật ưu tiên ghi Mức Thấp, Vừa, Cao, Rất cao (100, 400, 1500, 5000 điểm) hoặc ghi thẳng Điểm (điểm trừ mỗi lần không theo). Môn, Lớp, Khối, Ngày, Tiết ghi danh sách cách nhau bằng dấu phẩy hoặc khoảng, vd 3, 4 hoặc 3-5; Thứ 2, Thứ 4 hoặc T2-T4; 5-7. Buổi: Sáng hoặc Chiều. Giáo viên: chức vụ (Chủ Nhiệm, Bộ Môn, Quản Lý hoặc chức vụ GV chuyên biệt), 'trừ Chủ Nhiệm' là mọi giáo viên trừ chức vụ đó; hoặc một người: Mã GV (vd Bộ Môn 3, Chủ Nhiệm 1/1, đánh số theo thứ tự dòng của sheet NHÂN SỰ) hay họ tên (hai người trùng tên thì ghi Mã GV), vd giờ bận: Không xếp vào, Giáo viên Bộ Môn 3, Thứ 2, tiết 1 (để trống Môn); ép phân công: Chỉ giáo viên dạy, Môn Tiếng Anh, Lớp 3/1, Giáo viên Tiếng Anh 2. Câu đọc lại ghi Mã GV, không ghi họ tên. Nhãn, Trừ nhãn: tên các cột Có/Không của môn (vd Môn nặng) hoặc của giờ học (ngày, tiết, vd Luôn do GVCN dạy); nhiều nhãn giờ học là giờ có một trong các nhãn. Gồm môn tăng cường: Có thì Môn tính cả các môn tăng cường cùng nhóm. Không có sheet này thì chương trình dùng các luật có sẵn và sheet LUẬT RIÊNG (file của bản trước).</t>
+          <t>Không bắt buộc. Mỗi dòng một lớp: cột Lớp ghi tên lớp tùy ý (vd 1/1, 1A, Lá 2), cột Khối ghi tên khối như ở các cột Khối &lt;tên&gt; của sheet CHƯƠNG TRÌNH HỌC (vd 1 hoặc Lá; trống: các chữ số đầu tên lớp), cột Cơ sở 2 ghi Có nếu lớp học ở cơ sở 2. Có sheet này thì danh sách lớp lấy ở đây: Chủ Nhiệm ghi Lớp là một lớp của sheet, lớp không có Chủ Nhiệm vẫn được xếp (các môn chia cho GV khác; môn Chỉ GVCN dạy, tiết Luôn do GVCN dạy, tiết HĐTN cố định của GVCN không áp dụng cho lớp đó). Không có sheet này (hoặc sheet trống) thì lớp là lớp của các dòng Chủ Nhiệm, ghi dạng khối/số thứ tự (1/1) hoặc khối rồi tên lớp (1A).</t>
         </is>
       </c>
     </row>
     <row r="39" ht="25" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Không xếp vào</t>
+          <t>LUẬT</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Môn (của các khối ở cột Khối; để trống: mọi khối) không xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục không xếp vào tiết 1; Tin học không xếp vào Thứ 2. Ghi Giáo viên (chức vụ, Mã GV hoặc họ tên) thì chỉ xét tiết của người đó, để trống Môn là mọi môn: giờ bận, vd Bộ Môn 3 không dạy Thứ 2 tiết 1.</t>
+          <t>Mọi luật xếp TKB, mỗi dòng một luật, đọc như một câu: Với mỗi [cột Với mỗi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Mỗi luật trả lời một trong bốn câu hỏi: Ở đâu, Bao nhiêu, Đi cùng nhau, Ai dạy (các kiểu luật và phép đo xếp theo câu hỏi ở dưới). File mẫu ghi sẵn các luật có sẵn của chương trình: sửa số hoặc Điểm để chỉnh, đổi Bắt buộc, xóa dòng để bỏ luật (hoặc ghi Có ở cột Tạm tắt: chương trình bỏ qua dòng đó mà vẫn giữ lại, xóa chữ Có là dùng lại), thêm dòng để có luật mới. Cột Nhóm và Luật đọc là chỉ để đọc (chương trình ghi lại mỗi lần). Kiểu luật: một mẫu hoặc Tự ghép; cột kiểu luật không dùng để trống. Bắt buộc: Có (luật cứng) hoặc Không (ưu tiên); luật ưu tiên ghi Mức Thấp, Vừa, Cao, Rất cao (100, 400, 1500, 5000 điểm) hoặc ghi thẳng Điểm (điểm trừ mỗi lần không theo). Môn, Lớp, Khối, Ngày, Tiết ghi danh sách cách nhau bằng dấu phẩy hoặc khoảng, vd 3, 4 hoặc 3-5; Thứ 2, Thứ 4 hoặc T2-T4; 5-7. Buổi: Sáng hoặc Chiều. Giáo viên: chức vụ (Chủ Nhiệm, Bộ Môn, Quản Lý hoặc chức vụ GV chuyên biệt), 'trừ Chủ Nhiệm' là mọi giáo viên trừ chức vụ đó; hoặc một người: Mã GV (vd Bộ Môn 3, Chủ Nhiệm 1/1, đánh số theo thứ tự dòng của sheet NHÂN SỰ) hay họ tên (hai người trùng tên thì ghi Mã GV), vd giờ bận: Không xếp vào, Giáo viên Bộ Môn 3, Thứ 2, tiết 1 (để trống Môn); ép phân công: Chỉ giáo viên dạy, Môn Tiếng Anh, Lớp 3/1, Giáo viên Tiếng Anh 2. Câu đọc lại ghi Mã GV, không ghi họ tên. Nhãn, Trừ nhãn: tên các cột Có/Không của môn (vd Môn nặng) hoặc của giờ học (ngày, tiết, vd Luôn do GVCN dạy); nhiều nhãn giờ học là giờ có một trong các nhãn. Gồm môn tăng cường: Có thì Môn tính cả các môn tăng cường cùng nhóm. Không có sheet này thì chương trình dùng các luật có sẵn và sheet LUẬT RIÊNG (file của bản trước).</t>
         </is>
       </c>
     </row>
     <row r="40" ht="25" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Chỉ xếp vào</t>
+          <t>LUẬT: Ở đâu · Không xếp vào</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Môn chỉ xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục chỉ xếp vào buổi chiều. Ghi Giáo viên thì chỉ xét tiết của người đó (để trống Môn: mọi môn), vd Bộ Môn 3 chỉ dạy buổi sáng.</t>
+          <t>Môn (của các khối ở cột Khối; để trống: mọi khối) không xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục không xếp vào tiết 1; Tin học không xếp vào Thứ 2. Ghi Giáo viên (chức vụ, Mã GV hoặc họ tên) thì chỉ xét tiết của người đó, để trống Môn là mọi môn: giờ bận, vd Bộ Môn 3 không dạy Thứ 2 tiết 1.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="25" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Cố định vào</t>
+          <t>LUẬT: Ở đâu · Chỉ xếp vào</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Mỗi lớp (của các khối, lớp ghi ở dòng này) học đúng 1 tiết của Môn ở mỗi giờ ghi ở cột Ngày, Tiết, Buổi, vd Thể dục khối 1 cố định vào Thứ 3 tiết 3.</t>
+          <t>Môn chỉ xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục chỉ xếp vào buổi chiều. Ghi Giáo viên thì chỉ xét tiết của người đó (để trống Môn: mọi môn), vd Bộ Môn 3 chỉ dạy buổi sáng.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="25" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Giáo viên tối đa tiết mỗi ngày</t>
+          <t>LUẬT: Ở đâu · Cố định vào</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số tiết mỗi ngày.</t>
+          <t>Mỗi lớp (của các khối, lớp ghi ở dòng này) học đúng 1 tiết của Môn ở mỗi giờ ghi ở cột Ngày, Tiết, Buổi, vd Thể dục khối 1 cố định vào Thứ 3 tiết 3.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="25" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Giáo viên tối đa lớp mỗi ngày</t>
+          <t>LUẬT: Bao nhiêu · Giáo viên tối đa tiết mỗi ngày</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số lớp khác nhau mỗi ngày.</t>
+          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số tiết mỗi ngày.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="25" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Số lớp học cùng lúc tối đa</t>
+          <t>LUẬT: Bao nhiêu · Giáo viên tối đa lớp mỗi ngày</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Môn có tối đa Số lớp học cùng một giờ (cả trường, hoặc các khối ở cột Khối), vd phòng Tin học: 1, sân Thể dục: 2.</t>
+          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số lớp khác nhau mỗi ngày.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="25" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Học ít nhất số ngày</t>
+          <t>LUẬT: Bao nhiêu · Số lớp học cùng lúc tối đa</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Mỗi lớp học Môn ở ít nhất Số ngày khác nhau trong tuần, vd Tiếng Anh ít nhất 3 ngày.</t>
+          <t>Môn có tối đa Số lớp học cùng một giờ (cả trường, hoặc các khối ở cột Khối), vd phòng Tin học: 1, sân Thể dục: 2.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="25" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Học 2 tiết liền</t>
+          <t>LUẬT: Bao nhiêu · Học ít nhất số ngày</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Môn học thành cặp 2 tiết liền, cùng người dạy: mỗi buổi 0 hoặc 2 tiết của môn (tính chung môn tăng cường cùng nhóm), vd Tiếng Anh. Bắt buộc thì số tiết/tuần phải chẵn.</t>
+          <t>Mỗi lớp học Môn ở ít nhất Số ngày khác nhau trong tuần, vd Tiếng Anh ít nhất 3 ngày.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="25" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Học trước</t>
+          <t>LUẬT: Đi cùng nhau · Học 2 tiết liền</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Trong một buổi có cả hai môn thì Môn học trước Môn thứ hai, vd Tiếng Việt trước Toán.</t>
+          <t>Môn học thành cặp 2 tiết liền, cùng người dạy: mỗi buổi 0 hoặc 2 tiết của môn (tính chung môn tăng cường cùng nhóm), vd Tiếng Anh. Bắt buộc thì số tiết/tuần phải chẵn.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="25" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Chỉ giáo viên dạy</t>
+          <t>LUẬT: Đi cùng nhau · Học trước</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Các tiết của Môn (ở các khối, lớp, ngày, tiết ghi ở dòng này) chỉ do giáo viên ghi ở cột Giáo viên dạy: chức vụ, vd Tin học khối 3 chỉ GV Tin Học dạy; hoặc một người (Mã GV hay họ tên) để chọn ai dạy lớp nào, vd Tiếng Anh lớp 3/1 chỉ Tiếng Anh 2 dạy.</t>
+          <t>Trong một buổi có cả hai môn thì Môn học trước Môn thứ hai, vd Tiếng Việt trước Toán.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="25" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Buổi nghỉ của giáo viên</t>
+          <t>LUẬT: Ai dạy · Chỉ giáo viên dạy</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Giáo viên không dạy vào các buổi nghỉ ghi ở cột Buổi Nghỉ (sheet NHÂN SỰ) và nghỉ đủ số buổi ghi ở đó. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
+          <t>Các tiết của Môn (ở các khối, lớp, ngày, tiết ghi ở dòng này) chỉ do giáo viên ghi ở cột Giáo viên dạy: chức vụ, vd Tin học khối 3 chỉ GV Tin Học dạy; hoặc một người (Mã GV hay họ tên) để chọn ai dạy lớp nào, vd Tiếng Anh lớp 3/1 chỉ Tiếng Anh 2 dạy.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="25" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Giáo viên chỉ dạy cơ sở 2</t>
+          <t>LUẬT: Ai dạy · Buổi nghỉ của giáo viên</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Giáo viên không chủ nhiệm ghi Có ở cột Cơ sở 2 hoặc Thai Sản (sheet NHÂN SỰ) chỉ dạy các lớp ở cơ sở 2. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
+          <t>Giáo viên không dạy vào các buổi nghỉ ghi ở cột Buổi Nghỉ (sheet NHÂN SỰ) và nghỉ đủ số buổi ghi ở đó. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="25" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép</t>
+          <t>LUẬT: Ai dạy · Giáo viên chỉ dạy cơ sở 2</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Tự ghép câu luật: Với mỗi [phạm vi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Xem các phép đo ở dưới.</t>
+          <t>Giáo viên không chủ nhiệm ghi Có ở cột Cơ sở 2 hoặc Thai Sản (sheet NHÂN SỰ) chỉ dạy các lớp ở cơ sở 2. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="25" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Với mỗi</t>
+          <t>LUẬT: Tự ghép</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Chia các tiết thành từng nhóm theo các chiều, vd 'Lớp, Ngày': luật áp dụng cho mỗi lớp mỗi ngày. Các chiều: Lớp, Giáo viên, Môn, Nhóm môn, Khối, Ngày, Buổi, Giờ học, Cơ sở. Trống: cả trường cả tuần.</t>
+          <t>Tự ghép câu luật: Với mỗi [phạm vi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Xem các phép đo ở dưới.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="25" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Tự ghép, Phép đo Vị trí</t>
+          <t>LUẬT: Tự ghép, cột Với mỗi</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Các tiết chỉ xếp vào, hoặc không xếp vào, các ngày, tiết, buổi (hoặc giờ có nhãn) ghi ở dòng này. So sánh: Chỉ trong, Không trong.</t>
+          <t>Chia các tiết thành từng nhóm theo các chiều, vd 'Lớp, Ngày': luật áp dụng cho mỗi lớp mỗi ngày. Các chiều: Lớp, Giáo viên, Môn, Nhóm môn, Khối, Ngày, Buổi, Giờ học, Cơ sở. Trống: cả trường cả tuần.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="25" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số tiết</t>
+          <t>LUẬT: Ở đâu · Tự ghép, Phép đo Vị trí</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Đếm số tiết trong mỗi phạm vi, vd mỗi lớp mỗi ngày học tối đa 1 tiết Toán; mỗi giờ học có tối đa 1 tiết Tin học. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số.</t>
+          <t>Các tiết chỉ xếp vào, hoặc không xếp vào, các ngày, tiết, buổi (hoặc giờ có nhãn) ghi ở dòng này. So sánh: Chỉ trong, Không trong.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="25" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số khác nhau</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số tiết</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Đếm số lớp, ngày, cơ sở… khác nhau (cột Đếm theo), vd mỗi giáo viên mỗi ngày dạy tối đa 3 lớp; mỗi lớp học Tiếng Anh ít nhất 3 ngày. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số. Ghi cột Đếm theo.</t>
+          <t>Đếm số tiết trong mỗi phạm vi, vd mỗi lớp mỗi ngày học tối đa 1 tiết Toán; mỗi giờ học có tối đa 1 tiết Tin học. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="25" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Khoảng cách</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số khác nhau</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Số tiết trống xen giữa các tiết trong buổi (0: không có tiết trống); hoặc số tiết từ tiết đó đến cuối buổi (0: ở tiết cuối buổi). So sánh: Tiết trống tối đa, Cách cuối buổi tối đa. Ghi cột Số.</t>
+          <t>Đếm số lớp, ngày, cơ sở… khác nhau (cột Đếm theo), vd mỗi giáo viên mỗi ngày dạy tối đa 3 lớp; mỗi lớp học Tiếng Anh ít nhất 3 ngày. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số. Ghi cột Đếm theo.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="25" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Liền nhau</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Khoảng cách</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Các tiết trong một buổi (của mỗi lớp hoặc giáo viên) đứng liền nhau, không có tiết khác xen giữa.</t>
+          <t>Số tiết trống xen giữa các tiết trong buổi (0: không có tiết trống); hoặc số tiết từ tiết đó đến cuối buổi (0: ở tiết cuối buổi). So sánh: Tiết trống tối đa, Cách cuối buổi tối đa. Ghi cột Số.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="25" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Theo cặp 2 tiết</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Liền nhau</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Mỗi buổi học 0 hoặc 2 tiết, 2 tiết đó liền nhau (ưu tiên: hạn chế tiết lẻ đứng một mình).</t>
+          <t>Các tiết trong một buổi (của mỗi lớp hoặc giáo viên) đứng liền nhau, không có tiết khác xen giữa.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="25" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Thứ tự</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Theo cặp 2 tiết</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Trong một buổi (hoặc ngày, nếu Với mỗi có Ngày) tiết của Môn đứng trước (hoặc sau) tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm. So sánh: Trước, Sau.</t>
+          <t>Mỗi buổi học 0 hoặc 2 tiết, 2 tiết đó liền nhau (ưu tiên: hạn chế tiết lẻ đứng một mình).</t>
         </is>
       </c>
     </row>
     <row r="60" ht="25" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Đi kèm</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Thứ tự</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Buổi (hoặc ngày) có tiết của Môn thì cũng có tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm.</t>
+          <t>Trong một buổi (hoặc ngày, nếu Với mỗi có Ngày) tiết của Môn đứng trước (hoặc sau) tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm. So sánh: Trước, Sau.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="25" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Tự ghép, Phép đo Người dạy</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Đi kèm</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Các tiết do giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên) dạy; hoặc do cùng một người dạy; hoặc hai tiết liền nhau do cùng một người; hoặc tiết đầu tuần do giáo viên đó dạy, tiết của người khác không đứng trước. So sánh: Do, Cùng một người, Liền nhau cùng người, Tiết đầu tuần do.</t>
+          <t>Buổi (hoặc ngày) có tiết của Môn thì cũng có tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="25" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Số</t>
+          <t>LUẬT: Ai dạy · Tự ghép, Phép đo Người dạy</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Một số nguyên, hoặc (phép đo Số tiết) một ngưỡng theo dữ liệu: tải ngày, tải ngày + 1, số tiết/tuần chia số ngày (tải ngày: định mức của giáo viên chia theo số tiết của ngày).</t>
+          <t>Các tiết do giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên) dạy; hoặc do cùng một người dạy; hoặc hai tiết liền nhau do cùng một người; hoặc tiết đầu tuần do giáo viên đó dạy, tiết của người khác không đứng trước. So sánh: Do, Cùng một người, Liền nhau cùng người, Tiết đầu tuần do.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="25" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Áp dụng khi</t>
+          <t>LUẬT: Tự ghép, cột Số</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Chỉ áp dụng khi số tiết/tuần của các môn ở cột Môn (phạm vi có Môn, Nhóm môn: của từng môn, nhóm môn) ở khối đó thỏa điều kiện, vd '&gt;= 6, chẵn' (từ 6 tiết trở lên và chẵn) hoặc '&lt;= số ngày' (không quá số ngày học).</t>
+          <t>Một số nguyên, hoặc (phép đo Số tiết) một ngưỡng theo dữ liệu: tải ngày, tải ngày + 1, số tiết/tuần chia số ngày (tải ngày: định mức của giáo viên chia theo số tiết của ngày).</t>
         </is>
       </c>
     </row>
     <row r="64" ht="25" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: cấu trúc của TKB</t>
+          <t>LUẬT: Tự ghép, cột Áp dụng khi</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Cấu trúc của TKB (không phải luật, luôn có): mỗi lớp mỗi giờ học một tiết; mỗi lớp học đủ số tiết của chương trình học; giáo viên không dạy hai nơi cùng lúc, dạy không quá định mức (cộng số tiết bù tối đa ở chế độ bù giờ), Quản Lý dạy đúng định mức; giáo viên chỉ dạy các môn chức vụ được dạy (sheet CHƯƠNG TRÌNH HỌC, CHỨC VỤ).</t>
+          <t>Chỉ áp dụng khi số tiết/tuần của các môn ở cột Môn (phạm vi có Môn, Nhóm môn: của từng môn, nhóm môn) ở khối đó thỏa điều kiện, vd '&gt;= 6, chẵn' (từ 6 tiết trở lên và chẵn) hoặc '&lt;= số ngày' (không quá số ngày học).</t>
         </is>
       </c>
     </row>
     <row r="65" ht="25" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
+          <t>LUẬT: cấu trúc của TKB</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Cấu trúc của TKB (không phải luật, luôn có): mỗi lớp mỗi giờ học một tiết; mỗi lớp học đủ số tiết của chương trình học; giáo viên không dạy hai nơi cùng lúc, dạy không quá định mức (cộng số tiết bù tối đa ở chế độ bù giờ), Quản Lý dạy đúng định mức; giáo viên chỉ dạy các môn chức vụ được dạy (sheet CHƯƠNG TRÌNH HỌC, CHỨC VỤ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="25" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
           <t>Kiểu chữ</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>Các file kết quả chép kiểu chữ, cỡ chữ, viền của sheet NHÂN SỰ. Chỉ cần chữ và số: không cần công thức, màu nền, ghi chú trong ô hay danh sách thả xuống.</t>
         </is>

</xml_diff>

<commit_message>
Staff and class tags usable in rules
Optional column "Nhãn" in NHÂN SỰ and in sheet LỚP holds free tags with no
meaning of their own. The rules' Giáo viên column matches staff tags and
the Lớp column expands class tags, so a rule can target a group of people
(part-time staff, a subject team) or of classes (bilingual classes). The
Thai Sản, Hợp Đồng and Cơ sở 2 columns also act as tags of the same name.
Class tags enter the rules code only when written; files without tags keep
their codes. The web UI has a Nhãn column in the class table and suggests
tags in the rule dialog.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WtuWVKdziZbvQ9VXgRdGv
</commit_message>
<xml_diff>
--- a/data/Input_Template_V8.xlsx
+++ b/data/Input_Template_V8.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J300"/>
+  <dimension ref="A1:K300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -465,6 +465,7 @@
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -516,6 +517,11 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Chức Vụ Thêm</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Nhãn</t>
         </is>
       </c>
     </row>
@@ -530,6 +536,7 @@
       <c r="H2" s="4" t="n"/>
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
     </row>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -542,6 +549,7 @@
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="2" t="n"/>
@@ -554,6 +562,7 @@
       <c r="H4" s="4" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
     </row>
     <row r="5" ht="25" customHeight="1">
       <c r="A5" s="2" t="n"/>
@@ -566,6 +575,7 @@
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
     </row>
     <row r="6" ht="25" customHeight="1">
       <c r="A6" s="2" t="n"/>
@@ -578,6 +588,7 @@
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
     </row>
     <row r="7" ht="25" customHeight="1">
       <c r="A7" s="2" t="n"/>
@@ -590,6 +601,7 @@
       <c r="H7" s="4" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
     </row>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="2" t="n"/>
@@ -602,6 +614,7 @@
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
     </row>
     <row r="9" ht="25" customHeight="1">
       <c r="A9" s="2" t="n"/>
@@ -614,6 +627,7 @@
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
     </row>
     <row r="10" ht="25" customHeight="1">
       <c r="A10" s="2" t="n"/>
@@ -626,6 +640,7 @@
       <c r="H10" s="4" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
     </row>
     <row r="11" ht="25" customHeight="1">
       <c r="A11" s="2" t="n"/>
@@ -638,6 +653,7 @@
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="C12" s="5" t="n"/>
@@ -3134,12 +3150,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C300"/>
+  <dimension ref="A1:D300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -3158,56 +3175,71 @@
           <t>Cơ sở 2</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Nhãn</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="6" t="n"/>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
     </row>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="6" t="n"/>
       <c r="B3" s="3" t="n"/>
       <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="6" t="n"/>
       <c r="B4" s="3" t="n"/>
       <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
     </row>
     <row r="5" ht="25" customHeight="1">
       <c r="A5" s="6" t="n"/>
       <c r="B5" s="3" t="n"/>
       <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
     </row>
     <row r="6" ht="25" customHeight="1">
       <c r="A6" s="6" t="n"/>
       <c r="B6" s="3" t="n"/>
       <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
     </row>
     <row r="7" ht="25" customHeight="1">
       <c r="A7" s="6" t="n"/>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
     </row>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="6" t="n"/>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
     </row>
     <row r="9" ht="25" customHeight="1">
       <c r="A9" s="6" t="n"/>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
     </row>
     <row r="10" ht="25" customHeight="1">
       <c r="A10" s="6" t="n"/>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
     </row>
     <row r="11" ht="25" customHeight="1">
       <c r="A11" s="6" t="n"/>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -6269,7 +6301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B66"/>
+  <dimension ref="A1:B67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -6296,7 +6328,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên một dòng. Sáu cột Thai Sản, Hợp Đồng, Cơ sở 2, Lớp Đang Dạy, Buổi Nghỉ, Chức Vụ Thêm không bắt buộc (để trống hoặc xóa cột).</t>
+          <t>Mỗi giáo viên một dòng. Bảy cột Thai Sản, Hợp Đồng, Cơ sở 2, Lớp Đang Dạy, Buổi Nghỉ, Chức Vụ Thêm, Nhãn không bắt buộc (để trống hoặc xóa cột).</t>
         </is>
       </c>
     </row>
@@ -6423,646 +6455,658 @@
     <row r="13" ht="25" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC</t>
+          <t>NHÂN SỰ: Nhãn</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Mỗi môn một dòng: cột Môn học ghi tên môn (dùng đúng tên này ở sheet CHỨC VỤ, hoặc ở cột Chức Vụ của GV chuyên biệt chỉ dạy môn này), cột Khối &lt;tên&gt; ghi số tiết/tuần của môn ở khối đó (0 hoặc để trống: khối đó không học), các cột sau là quy định của môn. Tên khối tùy ý, vd Khối 1, Khối Lá; thêm khối thì thêm cột.</t>
+          <t>Các nhãn tự đặt, cách nhau bằng dấu phẩy (vd Bán thời gian, Tổ Toán). Cột Giáo viên của sheet LUẬT ghi một nhãn là mọi GV có nhãn đó, vd luật Bán thời gian không dạy buổi chiều. Thai Sản, Hợp Đồng, Cơ sở 2 ghi Có cũng là nhãn cùng tên.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="25" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Quy ước các ô quy định</t>
+          <t>CHƯƠNG TRÌNH HỌC</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Mỗi quy định là một cột (bảng Quy định chung: một dòng). Mỗi ô chỉ ghi Có, Không hoặc một số nguyên dương; ô trống là Không. Riêng cột Tên trong TKB ghi chữ. Xóa một cột (một dòng của bảng chung, một bảng, hoặc cả sheet QUY ĐỊNH) thì quy định đó dùng giá trị mặc định của chương trình.</t>
+          <t>Mỗi môn một dòng: cột Môn học ghi tên môn (dùng đúng tên này ở sheet CHỨC VỤ, hoặc ở cột Chức Vụ của GV chuyên biệt chỉ dạy môn này), cột Khối &lt;tên&gt; ghi số tiết/tuần của môn ở khối đó (0 hoặc để trống: khối đó không học), các cột sau là quy định của môn. Tên khối tùy ý, vd Khối 1, Khối Lá; thêm khối thì thêm cột.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="25" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH</t>
+          <t>Quy ước các ô quy định</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Ba bảng cách nhau một dòng trống: Quy định | Giá trị; Ngày (mỗi dòng một ngày học, mỗi cột Buổi &lt;tên&gt; ghi số tiết của buổi đó); Tiết (đánh số liên tục trong ngày: sáng 4 tiết thì chiều từ tiết 5; ngày dài nhất có bao nhiêu tiết thì bấy nhiêu dòng).</t>
+          <t>Mỗi quy định là một cột (bảng Quy định chung: một dòng). Mỗi ô chỉ ghi Có, Không hoặc một số nguyên dương; ô trống là Không. Riêng cột Tên trong TKB ghi chữ. Xóa một cột (một dòng của bảng chung, một bảng, hoặc cả sheet QUY ĐỊNH) thì quy định đó dùng giá trị mặc định của chương trình.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="25" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Tên trong TKB</t>
+          <t>QUY ĐỊNH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Chữ ghi trong ô TKB (cột duy nhất ghi chữ); trống: ghi đúng tên môn.</t>
+          <t>Ba bảng cách nhau một dòng trống: Quy định | Giá trị; Ngày (mỗi dòng một ngày học, mỗi cột Buổi &lt;tên&gt; ghi số tiết của buổi đó); Tiết (đánh số liên tục trong ngày: sáng 4 tiết thì chiều từ tiết 5; ngày dài nhất có bao nhiêu tiết thì bấy nhiêu dòng).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="25" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Môn HĐTN</t>
+          <t>CHƯƠNG TRÌNH HỌC: Tên trong TKB</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Có ở một môn: môn chào cờ, sinh hoạt lớp, có tiết cố định ở bảng ngày của sheet QUY ĐỊNH.</t>
+          <t>Chữ ghi trong ô TKB (cột duy nhất ghi chữ); trống: ghi đúng tên môn.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="25" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận trọn</t>
+          <t>CHƯƠNG TRÌNH HỌC: Môn HĐTN</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>GVCN nhận hết các môn này của lớp mình; luật cứng: môn nào phải chia cho người khác thì tiết đầu tiên trong tuần do GVCN dạy.</t>
+          <t>Có ở một môn: môn chào cờ, sinh hoạt lớp, có tiết cố định ở bảng ngày của sheet QUY ĐỊNH.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="25" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN cắt bớt</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận trọn</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Số thứ tự 1, 2...: môn cắt trước khi các môn nhận trọn vượt định mức GVCN; mỗi môn GVCN giữ ít nhất 1 tiết.</t>
+          <t>GVCN nhận hết các môn này của lớp mình; luật cứng: môn nào phải chia cho người khác thì tiết đầu tiên trong tuần do GVCN dạy.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận thêm</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN cắt bớt</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Số thứ tự 1, 2...: môn GVCN nhận thêm trước cho đủ định mức (không nhận môn của GV chuyên biệt).</t>
+          <t>Số thứ tự 1, 2...: môn cắt trước khi các môn nhận trọn vượt định mức GVCN; mỗi môn GVCN giữ ít nhất 1 tiết.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Chỉ GVCN dạy</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận thêm</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: chỉ GVCN của lớp được dạy.</t>
+          <t>Số thứ tự 1, 2...: môn GVCN nhận thêm trước cho đủ định mức (không nhận môn của GV chuyên biệt).</t>
         </is>
       </c>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Bộ Môn không dạy</t>
+          <t>CHƯƠNG TRÌNH HỌC: Chỉ GVCN dạy</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>GV bộ môn không dạy môn này; trường chưa có GV chuyên biệt của môn thì chương trình tuyển thêm. Ghi theo ngoại lệ để môn mới (ô trống) mặc nhiên bộ môn dạy được.</t>
+          <t>Luật cứng: chỉ GVCN của lớp được dạy.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="25" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Quản lý dạy khối</t>
+          <t>CHƯƠNG TRÌNH HỌC: Bộ Môn không dạy</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Khối mà Quản Lý được dạy môn này (tên khối như ở cột Khối &lt;tên&gt;), vd Kỹ năng sống: 4.</t>
+          <t>GV bộ môn không dạy môn này; trường chưa có GV chuyên biệt của môn thì chương trình tuyển thêm. Ghi theo ngoại lệ để môn mới (ô trống) mặc nhiên bộ môn dạy được.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="25" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN bù môn chuyên biệt</t>
+          <t>CHƯƠNG TRÌNH HỌC: Quản lý dạy khối</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Môn có GV chuyên biệt mà GVCN vẫn được dạy bù ở lớp mình (nhận sau cùng).</t>
+          <t>Khối mà Quản Lý được dạy môn này (tên khối như ở cột Khối &lt;tên&gt;), vd Kỹ năng sống: 4.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="25" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Nhóm môn</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN bù môn chuyên biệt</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Môn chính và các môn tăng cường của nó ghi cùng một số, vd Tiếng Việt và Tiếng Việt tăng cường: 1.</t>
+          <t>Môn có GV chuyên biệt mà GVCN vẫn được dạy bù ở lớp mình (nhận sau cùng).</t>
         </is>
       </c>
     </row>
     <row r="26" ht="25" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Môn tăng cường</t>
+          <t>CHƯƠNG TRÌNH HỌC: Nhóm môn</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Có ở môn tăng cường của nhóm; luật cứng: tiết tăng cường đứng sau mọi tiết môn chính trong ngày và ngày đó phải có tiết môn chính; cả nhóm tính chung cho giới hạn mỗi buổi và ghép cặp.</t>
+          <t>Môn chính và các môn tăng cường của nó ghi cùng một số, vd Tiếng Việt và Tiếng Việt tăng cường: 1.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="25" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Không ghép cặp</t>
+          <t>CHƯƠNG TRÌNH HỌC: Môn tăng cường</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Nhóm môn (ghi ở môn chính) không xếp thành cặp 2 tiết liền. Ghi theo ngoại lệ như cột Bộ Môn không dạy.</t>
+          <t>Có ở môn tăng cường của nhóm; luật cứng: tiết tăng cường đứng sau mọi tiết môn chính trong ngày và ngày đó phải có tiết môn chính; cả nhóm tính chung cho giới hạn mỗi buổi và ghép cặp.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="25" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Môn nặng</t>
+          <t>CHƯƠNG TRÌNH HỌC: Không ghép cặp</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu mềm: hạn chế xếp vào các tiết Hạn chế môn nặng (sheet QUY ĐỊNH).</t>
+          <t>Nhóm môn (ghi ở môn chính) không xếp thành cặp 2 tiết liền. Ghi theo ngoại lệ như cột Bộ Môn không dạy.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="25" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Ưu tiên buổi sáng</t>
+          <t>CHƯƠNG TRÌNH HỌC: Môn nặng</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu mềm: mỗi tiết ở buổi chiều bị trừ điểm, và môn được rải đều hơn trong tuần.</t>
+          <t>Mục tiêu mềm: hạn chế xếp vào các tiết Hạn chế môn nặng (sheet QUY ĐỊNH).</t>
         </is>
       </c>
     </row>
     <row r="30" ht="25" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Chủ Nhiệm được dạy bù</t>
+          <t>CHƯƠNG TRÌNH HỌC: Ưu tiên buổi sáng</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>GVCN chỉ bù ở lớp mình và bù trước bộ môn.</t>
+          <t>Mục tiêu mềm: mỗi tiết ở buổi chiều bị trừ điểm, và môn được rải đều hơn trong tuần.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="25" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Bộ Môn được dạy bù</t>
+          <t>QUY ĐỊNH: Chủ Nhiệm được dạy bù</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Bộ môn bù khi GVCN đã bù hết mức.</t>
+          <t>GVCN chỉ bù ở lớp mình và bù trước bộ môn.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="25" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Ngày, Buổi &lt;tên buổi&gt;</t>
+          <t>QUY ĐỊNH: Bộ Môn được dạy bù</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Bảng Ngày: mỗi dòng một ngày học, tên tùy ý (vd Thứ 2, Thứ 7, Chủ nhật), theo thứ tự trong tuần. Mỗi cột Buổi &lt;tên buổi&gt; (vd Buổi Sáng, Buổi Chiều, Buổi Tối) ghi số tiết của buổi đó trong ngày; ô trống là ngày đó không học buổi đó. Mỗi ngày một số tiết riêng được (vd chiều Thứ 5 có 4 tiết). Thêm buổi thì thêm cột, thêm ngày học thì thêm dòng; ngày không có tiết nào không phải ngày học. Tiết đánh số liên tục trong ngày theo thứ tự các cột buổi: sáng 4 tiết thì chiều bắt đầu từ tiết 5.</t>
+          <t>Bộ môn bù khi GVCN đã bù hết mức.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="25" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Tiết HĐTN cố định</t>
+          <t>QUY ĐỊNH: Ngày, Buổi &lt;tên buổi&gt;</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: tiết môn HĐTN cố định của ngày đó ở mọi lớp, vd Thứ 2: 1, Thứ 6: 4.</t>
+          <t>Bảng Ngày: mỗi dòng một ngày học, tên tùy ý (vd Thứ 2, Thứ 7, Chủ nhật), theo thứ tự trong tuần. Mỗi cột Buổi &lt;tên buổi&gt; (vd Buổi Sáng, Buổi Chiều, Buổi Tối) ghi số tiết của buổi đó trong ngày; ô trống là ngày đó không học buổi đó. Mỗi ngày một số tiết riêng được (vd chiều Thứ 5 có 4 tiết). Thêm buổi thì thêm cột, thêm ngày học thì thêm dòng; ngày không có tiết nào không phải ngày học. Tiết đánh số liên tục trong ngày theo thứ tự các cột buổi: sáng 4 tiết thì chiều bắt đầu từ tiết 5.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="25" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Xếp tiết HĐTN còn lại</t>
+          <t>QUY ĐỊNH: Tiết HĐTN cố định</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: các tiết HĐTN còn lại chỉ xếp vào các ngày này (mục tiêu mềm: gần cuối buổi).</t>
+          <t>Luật cứng: tiết môn HĐTN cố định của ngày đó ở mọi lớp, vd Thứ 2: 1, Thứ 6: 4.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="25" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Luôn do GVCN dạy</t>
+          <t>QUY ĐỊNH: Xếp tiết HĐTN còn lại</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: tiết này ở mọi ngày do GVCN của lớp dạy.</t>
+          <t>Luật cứng: các tiết HĐTN còn lại chỉ xếp vào các ngày này (mục tiêu mềm: gần cuối buổi).</t>
         </is>
       </c>
     </row>
     <row r="36" ht="25" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Hạn chế môn nặng</t>
+          <t>QUY ĐỊNH: Luôn do GVCN dạy</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu mềm: mỗi tiết môn nặng ở tiết này bị trừ điểm.</t>
+          <t>Luật cứng: tiết này ở mọi ngày do GVCN của lớp dạy.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="25" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>CHỨC VỤ</t>
+          <t>QUY ĐỊNH: Hạn chế môn nặng</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Không bắt buộc. Mỗi dòng một chức vụ GV chuyên biệt nhà trường tự đặt: cột Chức vụ ghi tên (không ghi số, không trùng Chủ Nhiệm, Bộ Môn, Quản Lý), cột Môn được dạy ghi các môn chức vụ đó dạy, cách nhau bằng dấu phẩy, đúng tên trong sheet CHƯƠNG TRÌNH HỌC, vd GV Nghệ thuật: Âm nhạc, Mỹ thuật. Ở sheet NHÂN SỰ, GV có Chức Vụ là tên đó chỉ dạy các môn này. Chức vụ không ghi ở đây mà trùng tên một môn (vd Tiếng Anh) thì chỉ dạy môn đó. Môn Bộ Môn không dạy mà chưa có GV nào dạy được thì chương trình tuyển thêm chức vụ đầu tiên ở đây dạy môn đó (không có thì chức vụ trùng tên môn).</t>
+          <t>Mục tiêu mềm: mỗi tiết môn nặng ở tiết này bị trừ điểm.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="25" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>LỚP</t>
+          <t>CHỨC VỤ</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Không bắt buộc. Mỗi dòng một lớp: cột Lớp ghi tên lớp tùy ý (vd 1/1, 1A, Lá 2), cột Khối ghi tên khối như ở các cột Khối &lt;tên&gt; của sheet CHƯƠNG TRÌNH HỌC (vd 1 hoặc Lá; trống: các chữ số đầu tên lớp), cột Cơ sở 2 ghi Có nếu lớp học ở cơ sở 2. Có sheet này thì danh sách lớp lấy ở đây: Chủ Nhiệm ghi Lớp là một lớp của sheet, lớp không có Chủ Nhiệm vẫn được xếp (các môn chia cho GV khác; môn Chỉ GVCN dạy, tiết Luôn do GVCN dạy, tiết HĐTN cố định của GVCN không áp dụng cho lớp đó). Không có sheet này (hoặc sheet trống) thì lớp là lớp của các dòng Chủ Nhiệm, ghi dạng khối/số thứ tự (1/1) hoặc khối rồi tên lớp (1A).</t>
+          <t>Không bắt buộc. Mỗi dòng một chức vụ GV chuyên biệt nhà trường tự đặt: cột Chức vụ ghi tên (không ghi số, không trùng Chủ Nhiệm, Bộ Môn, Quản Lý), cột Môn được dạy ghi các môn chức vụ đó dạy, cách nhau bằng dấu phẩy, đúng tên trong sheet CHƯƠNG TRÌNH HỌC, vd GV Nghệ thuật: Âm nhạc, Mỹ thuật. Ở sheet NHÂN SỰ, GV có Chức Vụ là tên đó chỉ dạy các môn này. Chức vụ không ghi ở đây mà trùng tên một môn (vd Tiếng Anh) thì chỉ dạy môn đó. Môn Bộ Môn không dạy mà chưa có GV nào dạy được thì chương trình tuyển thêm chức vụ đầu tiên ở đây dạy môn đó (không có thì chức vụ trùng tên môn).</t>
         </is>
       </c>
     </row>
     <row r="39" ht="25" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>LUẬT</t>
+          <t>LỚP</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Mọi luật xếp TKB, mỗi dòng một luật, đọc như một câu: Với mỗi [cột Với mỗi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Mỗi luật trả lời một trong bốn câu hỏi: Ở đâu, Bao nhiêu, Đi cùng nhau, Ai dạy (các kiểu luật và phép đo xếp theo câu hỏi ở dưới). File mẫu ghi sẵn các luật có sẵn của chương trình: sửa số hoặc Điểm để chỉnh, đổi Bắt buộc, xóa dòng để bỏ luật (hoặc ghi Có ở cột Tạm tắt: chương trình bỏ qua dòng đó mà vẫn giữ lại, xóa chữ Có là dùng lại), thêm dòng để có luật mới. Cột Nhóm và Luật đọc là chỉ để đọc (chương trình ghi lại mỗi lần). Kiểu luật: một mẫu hoặc Tự ghép; cột kiểu luật không dùng để trống. Bắt buộc: Có (luật cứng) hoặc Không (ưu tiên); luật ưu tiên ghi Mức Thấp, Vừa, Cao, Rất cao (100, 400, 1500, 5000 điểm) hoặc ghi thẳng Điểm (điểm trừ mỗi lần không theo). Môn, Lớp, Khối, Ngày, Tiết ghi danh sách cách nhau bằng dấu phẩy hoặc khoảng, vd 3, 4 hoặc 3-5; Thứ 2, Thứ 4 hoặc T2-T4; 5-7. Buổi: Sáng hoặc Chiều. Giáo viên: chức vụ (Chủ Nhiệm, Bộ Môn, Quản Lý hoặc chức vụ GV chuyên biệt), 'trừ Chủ Nhiệm' là mọi giáo viên trừ chức vụ đó; hoặc một người: Mã GV (vd Bộ Môn 3, Chủ Nhiệm 1/1, đánh số theo thứ tự dòng của sheet NHÂN SỰ) hay họ tên (hai người trùng tên thì ghi Mã GV), vd giờ bận: Không xếp vào, Giáo viên Bộ Môn 3, Thứ 2, tiết 1 (để trống Môn); ép phân công: Chỉ giáo viên dạy, Môn Tiếng Anh, Lớp 3/1, Giáo viên Tiếng Anh 2. Câu đọc lại ghi Mã GV, không ghi họ tên. Nhãn, Trừ nhãn: tên các cột Có/Không của môn (vd Môn nặng) hoặc của giờ học (ngày, tiết, vd Luôn do GVCN dạy); nhiều nhãn giờ học là giờ có một trong các nhãn. Gồm môn tăng cường: Có thì Môn tính cả các môn tăng cường cùng nhóm. Không có sheet này thì chương trình dùng các luật có sẵn và sheet LUẬT RIÊNG (file của bản trước).</t>
+          <t>Không bắt buộc. Mỗi dòng một lớp: cột Lớp ghi tên lớp tùy ý (vd 1/1, 1A, Lá 2), cột Khối ghi tên khối như ở các cột Khối &lt;tên&gt; của sheet CHƯƠNG TRÌNH HỌC (vd 1 hoặc Lá; trống: các chữ số đầu tên lớp), cột Cơ sở 2 ghi Có nếu lớp học ở cơ sở 2, cột Nhãn ghi các nhãn tự đặt cách nhau dấu phẩy (vd Song ngữ; không trùng tên lớp): cột Lớp của sheet LUẬT ghi nhãn là mọi lớp có nhãn đó, lớp ghi Có ở cột Cơ sở 2 có nhãn Cơ sở 2. Có sheet này thì danh sách lớp lấy ở đây: Chủ Nhiệm ghi Lớp là một lớp của sheet, lớp không có Chủ Nhiệm vẫn được xếp (các môn chia cho GV khác; môn Chỉ GVCN dạy, tiết Luôn do GVCN dạy, tiết HĐTN cố định của GVCN không áp dụng cho lớp đó). Không có sheet này (hoặc sheet trống) thì lớp là lớp của các dòng Chủ Nhiệm, ghi dạng khối/số thứ tự (1/1) hoặc khối rồi tên lớp (1A).</t>
         </is>
       </c>
     </row>
     <row r="40" ht="25" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Không xếp vào</t>
+          <t>LUẬT</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Môn (của các khối ở cột Khối; để trống: mọi khối) không xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục không xếp vào tiết 1; Tin học không xếp vào Thứ 2. Ghi Giáo viên (chức vụ, Mã GV hoặc họ tên) thì chỉ xét tiết của người đó, để trống Môn là mọi môn: giờ bận, vd Bộ Môn 3 không dạy Thứ 2 tiết 1.</t>
+          <t>Mọi luật xếp TKB, mỗi dòng một luật, đọc như một câu: Với mỗi [cột Với mỗi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Mỗi luật trả lời một trong bốn câu hỏi: Ở đâu, Bao nhiêu, Đi cùng nhau, Ai dạy (các kiểu luật và phép đo xếp theo câu hỏi ở dưới). File mẫu ghi sẵn các luật có sẵn của chương trình: sửa số hoặc Điểm để chỉnh, đổi Bắt buộc, xóa dòng để bỏ luật (hoặc ghi Có ở cột Tạm tắt: chương trình bỏ qua dòng đó mà vẫn giữ lại, xóa chữ Có là dùng lại), thêm dòng để có luật mới. Cột Nhóm và Luật đọc là chỉ để đọc (chương trình ghi lại mỗi lần). Kiểu luật: một mẫu hoặc Tự ghép; cột kiểu luật không dùng để trống. Bắt buộc: Có (luật cứng) hoặc Không (ưu tiên); luật ưu tiên ghi Mức Thấp, Vừa, Cao, Rất cao (100, 400, 1500, 5000 điểm) hoặc ghi thẳng Điểm (điểm trừ mỗi lần không theo). Môn, Lớp, Khối, Ngày, Tiết ghi danh sách cách nhau bằng dấu phẩy hoặc khoảng, vd 3, 4 hoặc 3-5; Thứ 2, Thứ 4 hoặc T2-T4; 5-7. Buổi: Sáng hoặc Chiều. Giáo viên: chức vụ (Chủ Nhiệm, Bộ Môn, Quản Lý hoặc chức vụ GV chuyên biệt), 'trừ Chủ Nhiệm' là mọi giáo viên trừ chức vụ đó; hoặc một người: Mã GV (vd Bộ Môn 3, Chủ Nhiệm 1/1, đánh số theo thứ tự dòng của sheet NHÂN SỰ) hay họ tên (hai người trùng tên thì ghi Mã GV), vd giờ bận: Không xếp vào, Giáo viên Bộ Môn 3, Thứ 2, tiết 1 (để trống Môn); ép phân công: Chỉ giáo viên dạy, Môn Tiếng Anh, Lớp 3/1, Giáo viên Tiếng Anh 2. Câu đọc lại ghi Mã GV, không ghi họ tên. Nhãn, Trừ nhãn: tên các cột Có/Không của môn (vd Môn nặng) hoặc của giờ học (ngày, tiết, vd Luôn do GVCN dạy); nhiều nhãn giờ học là giờ có một trong các nhãn. Gồm môn tăng cường: Có thì Môn tính cả các môn tăng cường cùng nhóm. Không có sheet này thì chương trình dùng các luật có sẵn và sheet LUẬT RIÊNG (file của bản trước).</t>
         </is>
       </c>
     </row>
     <row r="41" ht="25" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Chỉ xếp vào</t>
+          <t>LUẬT: Ở đâu · Không xếp vào</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Môn chỉ xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục chỉ xếp vào buổi chiều. Ghi Giáo viên thì chỉ xét tiết của người đó (để trống Môn: mọi môn), vd Bộ Môn 3 chỉ dạy buổi sáng.</t>
+          <t>Môn (của các khối ở cột Khối; để trống: mọi khối) không xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục không xếp vào tiết 1; Tin học không xếp vào Thứ 2. Ghi Giáo viên (chức vụ, Mã GV hoặc họ tên) thì chỉ xét tiết của người đó, để trống Môn là mọi môn: giờ bận, vd Bộ Môn 3 không dạy Thứ 2 tiết 1.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="25" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Cố định vào</t>
+          <t>LUẬT: Ở đâu · Chỉ xếp vào</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Mỗi lớp (của các khối, lớp ghi ở dòng này) học đúng 1 tiết của Môn ở mỗi giờ ghi ở cột Ngày, Tiết, Buổi, vd Thể dục khối 1 cố định vào Thứ 3 tiết 3.</t>
+          <t>Môn chỉ xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục chỉ xếp vào buổi chiều. Ghi Giáo viên thì chỉ xét tiết của người đó (để trống Môn: mọi môn), vd Bộ Môn 3 chỉ dạy buổi sáng.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="25" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Giáo viên tối đa tiết mỗi ngày</t>
+          <t>LUẬT: Ở đâu · Cố định vào</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số tiết mỗi ngày.</t>
+          <t>Mỗi lớp (của các khối, lớp ghi ở dòng này) học đúng 1 tiết của Môn ở mỗi giờ ghi ở cột Ngày, Tiết, Buổi, vd Thể dục khối 1 cố định vào Thứ 3 tiết 3.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="25" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Giáo viên tối đa lớp mỗi ngày</t>
+          <t>LUẬT: Bao nhiêu · Giáo viên tối đa tiết mỗi ngày</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số lớp khác nhau mỗi ngày.</t>
+          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số tiết mỗi ngày.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="25" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Số lớp học cùng lúc tối đa</t>
+          <t>LUẬT: Bao nhiêu · Giáo viên tối đa lớp mỗi ngày</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Môn có tối đa Số lớp học cùng một giờ (cả trường, hoặc các khối ở cột Khối), vd phòng Tin học: 1, sân Thể dục: 2.</t>
+          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số lớp khác nhau mỗi ngày.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="25" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Học ít nhất số ngày</t>
+          <t>LUẬT: Bao nhiêu · Số lớp học cùng lúc tối đa</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Mỗi lớp học Môn ở ít nhất Số ngày khác nhau trong tuần, vd Tiếng Anh ít nhất 3 ngày.</t>
+          <t>Môn có tối đa Số lớp học cùng một giờ (cả trường, hoặc các khối ở cột Khối), vd phòng Tin học: 1, sân Thể dục: 2.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="25" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Học 2 tiết liền</t>
+          <t>LUẬT: Bao nhiêu · Học ít nhất số ngày</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Môn học thành cặp 2 tiết liền, cùng người dạy: mỗi buổi 0 hoặc 2 tiết của môn (tính chung môn tăng cường cùng nhóm), vd Tiếng Anh. Bắt buộc thì số tiết/tuần phải chẵn.</t>
+          <t>Mỗi lớp học Môn ở ít nhất Số ngày khác nhau trong tuần, vd Tiếng Anh ít nhất 3 ngày.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="25" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Học trước</t>
+          <t>LUẬT: Đi cùng nhau · Học 2 tiết liền</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Trong một buổi có cả hai môn thì Môn học trước Môn thứ hai, vd Tiếng Việt trước Toán.</t>
+          <t>Môn học thành cặp 2 tiết liền, cùng người dạy: mỗi buổi 0 hoặc 2 tiết của môn (tính chung môn tăng cường cùng nhóm), vd Tiếng Anh. Bắt buộc thì số tiết/tuần phải chẵn.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="25" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Chỉ giáo viên dạy</t>
+          <t>LUẬT: Đi cùng nhau · Học trước</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Các tiết của Môn (ở các khối, lớp, ngày, tiết ghi ở dòng này) chỉ do giáo viên ghi ở cột Giáo viên dạy: chức vụ, vd Tin học khối 3 chỉ GV Tin Học dạy; hoặc một người (Mã GV hay họ tên) để chọn ai dạy lớp nào, vd Tiếng Anh lớp 3/1 chỉ Tiếng Anh 2 dạy.</t>
+          <t>Trong một buổi có cả hai môn thì Môn học trước Môn thứ hai, vd Tiếng Việt trước Toán.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="25" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Buổi nghỉ của giáo viên</t>
+          <t>LUẬT: Ai dạy · Chỉ giáo viên dạy</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Giáo viên không dạy vào các buổi nghỉ ghi ở cột Buổi Nghỉ (sheet NHÂN SỰ) và nghỉ đủ số buổi ghi ở đó. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
+          <t>Các tiết của Môn (ở các khối, lớp, ngày, tiết ghi ở dòng này) chỉ do giáo viên ghi ở cột Giáo viên dạy: chức vụ, vd Tin học khối 3 chỉ GV Tin Học dạy; hoặc một người (Mã GV hay họ tên) để chọn ai dạy lớp nào, vd Tiếng Anh lớp 3/1 chỉ Tiếng Anh 2 dạy.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="25" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Giáo viên chỉ dạy cơ sở 2</t>
+          <t>LUẬT: Ai dạy · Buổi nghỉ của giáo viên</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Giáo viên không chủ nhiệm ghi Có ở cột Cơ sở 2 hoặc Thai Sản (sheet NHÂN SỰ) chỉ dạy các lớp ở cơ sở 2. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
+          <t>Giáo viên không dạy vào các buổi nghỉ ghi ở cột Buổi Nghỉ (sheet NHÂN SỰ) và nghỉ đủ số buổi ghi ở đó. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="25" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép</t>
+          <t>LUẬT: Ai dạy · Giáo viên chỉ dạy cơ sở 2</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Tự ghép câu luật: Với mỗi [phạm vi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Xem các phép đo ở dưới.</t>
+          <t>Giáo viên không chủ nhiệm ghi Có ở cột Cơ sở 2 hoặc Thai Sản (sheet NHÂN SỰ) chỉ dạy các lớp ở cơ sở 2. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="25" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Với mỗi</t>
+          <t>LUẬT: Tự ghép</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Chia các tiết thành từng nhóm theo các chiều, vd 'Lớp, Ngày': luật áp dụng cho mỗi lớp mỗi ngày. Các chiều: Lớp, Giáo viên, Môn, Nhóm môn, Khối, Ngày, Buổi, Giờ học, Cơ sở. Trống: cả trường cả tuần.</t>
+          <t>Tự ghép câu luật: Với mỗi [phạm vi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Xem các phép đo ở dưới.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="25" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Tự ghép, Phép đo Vị trí</t>
+          <t>LUẬT: Tự ghép, cột Với mỗi</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Các tiết chỉ xếp vào, hoặc không xếp vào, các ngày, tiết, buổi (hoặc giờ có nhãn) ghi ở dòng này. So sánh: Chỉ trong, Không trong.</t>
+          <t>Chia các tiết thành từng nhóm theo các chiều, vd 'Lớp, Ngày': luật áp dụng cho mỗi lớp mỗi ngày. Các chiều: Lớp, Giáo viên, Môn, Nhóm môn, Khối, Ngày, Buổi, Giờ học, Cơ sở. Trống: cả trường cả tuần.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="25" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số tiết</t>
+          <t>LUẬT: Ở đâu · Tự ghép, Phép đo Vị trí</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Đếm số tiết trong mỗi phạm vi, vd mỗi lớp mỗi ngày học tối đa 1 tiết Toán; mỗi giờ học có tối đa 1 tiết Tin học. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số.</t>
+          <t>Các tiết chỉ xếp vào, hoặc không xếp vào, các ngày, tiết, buổi (hoặc giờ có nhãn) ghi ở dòng này. So sánh: Chỉ trong, Không trong.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="25" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số khác nhau</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số tiết</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Đếm số lớp, ngày, cơ sở… khác nhau (cột Đếm theo), vd mỗi giáo viên mỗi ngày dạy tối đa 3 lớp; mỗi lớp học Tiếng Anh ít nhất 3 ngày. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số. Ghi cột Đếm theo.</t>
+          <t>Đếm số tiết trong mỗi phạm vi, vd mỗi lớp mỗi ngày học tối đa 1 tiết Toán; mỗi giờ học có tối đa 1 tiết Tin học. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="25" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Khoảng cách</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số khác nhau</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Số tiết trống xen giữa các tiết trong buổi (0: không có tiết trống); hoặc số tiết từ tiết đó đến cuối buổi (0: ở tiết cuối buổi). So sánh: Tiết trống tối đa, Cách cuối buổi tối đa. Ghi cột Số.</t>
+          <t>Đếm số lớp, ngày, cơ sở… khác nhau (cột Đếm theo), vd mỗi giáo viên mỗi ngày dạy tối đa 3 lớp; mỗi lớp học Tiếng Anh ít nhất 3 ngày. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số. Ghi cột Đếm theo.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="25" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Liền nhau</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Khoảng cách</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Các tiết trong một buổi (của mỗi lớp hoặc giáo viên) đứng liền nhau, không có tiết khác xen giữa.</t>
+          <t>Số tiết trống xen giữa các tiết trong buổi (0: không có tiết trống); hoặc số tiết từ tiết đó đến cuối buổi (0: ở tiết cuối buổi). So sánh: Tiết trống tối đa, Cách cuối buổi tối đa. Ghi cột Số.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="25" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Theo cặp 2 tiết</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Liền nhau</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Mỗi buổi học 0 hoặc 2 tiết, 2 tiết đó liền nhau (ưu tiên: hạn chế tiết lẻ đứng một mình).</t>
+          <t>Các tiết trong một buổi (của mỗi lớp hoặc giáo viên) đứng liền nhau, không có tiết khác xen giữa.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="25" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Thứ tự</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Theo cặp 2 tiết</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Trong một buổi (hoặc ngày, nếu Với mỗi có Ngày) tiết của Môn đứng trước (hoặc sau) tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm. So sánh: Trước, Sau.</t>
+          <t>Mỗi buổi học 0 hoặc 2 tiết, 2 tiết đó liền nhau (ưu tiên: hạn chế tiết lẻ đứng một mình).</t>
         </is>
       </c>
     </row>
     <row r="61" ht="25" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Đi kèm</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Thứ tự</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Buổi (hoặc ngày) có tiết của Môn thì cũng có tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm.</t>
+          <t>Trong một buổi (hoặc ngày, nếu Với mỗi có Ngày) tiết của Môn đứng trước (hoặc sau) tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm. So sánh: Trước, Sau.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="25" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Tự ghép, Phép đo Người dạy</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Đi kèm</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Các tiết do giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên) dạy; hoặc do cùng một người dạy; hoặc hai tiết liền nhau do cùng một người; hoặc tiết đầu tuần do giáo viên đó dạy, tiết của người khác không đứng trước. So sánh: Do, Cùng một người, Liền nhau cùng người, Tiết đầu tuần do.</t>
+          <t>Buổi (hoặc ngày) có tiết của Môn thì cũng có tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="25" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Số</t>
+          <t>LUẬT: Ai dạy · Tự ghép, Phép đo Người dạy</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Một số nguyên, hoặc (phép đo Số tiết) một ngưỡng theo dữ liệu: tải ngày, tải ngày + 1, số tiết/tuần chia số ngày (tải ngày: định mức của giáo viên chia theo số tiết của ngày).</t>
+          <t>Các tiết do giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên) dạy; hoặc do cùng một người dạy; hoặc hai tiết liền nhau do cùng một người; hoặc tiết đầu tuần do giáo viên đó dạy, tiết của người khác không đứng trước. So sánh: Do, Cùng một người, Liền nhau cùng người, Tiết đầu tuần do.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="25" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Áp dụng khi</t>
+          <t>LUẬT: Tự ghép, cột Số</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Chỉ áp dụng khi số tiết/tuần của các môn ở cột Môn (phạm vi có Môn, Nhóm môn: của từng môn, nhóm môn) ở khối đó thỏa điều kiện, vd '&gt;= 6, chẵn' (từ 6 tiết trở lên và chẵn) hoặc '&lt;= số ngày' (không quá số ngày học).</t>
+          <t>Một số nguyên, hoặc (phép đo Số tiết) một ngưỡng theo dữ liệu: tải ngày, tải ngày + 1, số tiết/tuần chia số ngày (tải ngày: định mức của giáo viên chia theo số tiết của ngày).</t>
         </is>
       </c>
     </row>
     <row r="65" ht="25" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: cấu trúc của TKB</t>
+          <t>LUẬT: Tự ghép, cột Áp dụng khi</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Cấu trúc của TKB (không phải luật, luôn có): mỗi lớp mỗi giờ học một tiết; mỗi lớp học đủ số tiết của chương trình học; giáo viên không dạy hai nơi cùng lúc, dạy không quá định mức (cộng số tiết bù tối đa ở chế độ bù giờ), Quản Lý dạy đúng định mức; giáo viên chỉ dạy các môn chức vụ được dạy (sheet CHƯƠNG TRÌNH HỌC, CHỨC VỤ).</t>
+          <t>Chỉ áp dụng khi số tiết/tuần của các môn ở cột Môn (phạm vi có Môn, Nhóm môn: của từng môn, nhóm môn) ở khối đó thỏa điều kiện, vd '&gt;= 6, chẵn' (từ 6 tiết trở lên và chẵn) hoặc '&lt;= số ngày' (không quá số ngày học).</t>
         </is>
       </c>
     </row>
     <row r="66" ht="25" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
+          <t>LUẬT: cấu trúc của TKB</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Cấu trúc của TKB (không phải luật, luôn có): mỗi lớp mỗi giờ học một tiết; mỗi lớp học đủ số tiết của chương trình học; giáo viên không dạy hai nơi cùng lúc, dạy không quá định mức (cộng số tiết bù tối đa ở chế độ bù giờ), Quản Lý dạy đúng định mức; giáo viên chỉ dạy các môn chức vụ được dạy (sheet CHƯƠNG TRÌNH HỌC, CHỨC VỤ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="25" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
           <t>Kiểu chữ</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>Các file kết quả chép kiểu chữ, cỡ chữ, viền của sheet NHÂN SỰ. Chỉ cần chữ và số: không cần công thức, màu nền, ghi chú trong ô hay danh sách thả xuống.</t>
         </is>

</xml_diff>

<commit_message>
Any number of campuses with free names
Sheet LỚP gets a "Cơ sở" column holding a campus name; blank means
"Cơ sở 1" and the old Có/Không "Cơ sở 2" column (and the homeroom row's
flag) still mean "Cơ sở 2". The hard rule "one campus per session" and the
soft penalty for changing campus within a day now work for any number of
campuses; with two campuses the model keeps its old variables, so codes
are unchanged. The timetable is split into one file per campus, the
statistics and messages name the campuses, and each campus name is a
class tag usable in rules. The web UI edits the campus name per class.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WtuWVKdziZbvQ9VXgRdGv
</commit_message>
<xml_diff>
--- a/data/Input_Template_V8.xlsx
+++ b/data/Input_Template_V8.xlsx
@@ -3155,7 +3155,7 @@
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Cơ sở 2</t>
+          <t>Cơ sở</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -5554,7 +5554,7 @@
       <c r="W17" s="3" t="n"/>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>Hạn chế để một giáo viên dạy ở cả hai cơ sở trong cùng một ngày (ưu tiên rất cao)</t>
+          <t>Hạn chế để một giáo viên đổi cơ sở trong cùng một ngày (dạy ở hai cơ sở trở lên) (ưu tiên rất cao)</t>
         </is>
       </c>
     </row>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Không bắt buộc. Mỗi dòng một lớp: cột Lớp ghi tên lớp tùy ý (vd 1/1, 1A, Lá 2), cột Khối ghi tên khối như ở các cột Khối &lt;tên&gt; của sheet CHƯƠNG TRÌNH HỌC (vd 1 hoặc Lá; trống: các chữ số đầu tên lớp), cột Cơ sở 2 ghi Có nếu lớp học ở cơ sở 2, cột Nhãn ghi các nhãn tự đặt cách nhau dấu phẩy (vd Song ngữ; không trùng tên lớp): cột Lớp của sheet LUẬT ghi nhãn là mọi lớp có nhãn đó, lớp ghi Có ở cột Cơ sở 2 có nhãn Cơ sở 2. Có sheet này thì danh sách lớp lấy ở đây: Chủ Nhiệm ghi Lớp là một lớp của sheet, lớp không có Chủ Nhiệm vẫn được xếp (các môn chia cho GV khác; môn Chỉ GVCN dạy, tiết Luôn do GVCN dạy, tiết HĐTN cố định của GVCN không áp dụng cho lớp đó). Không có sheet này (hoặc sheet trống) thì lớp là lớp của các dòng Chủ Nhiệm, ghi dạng khối/số thứ tự (1/1) hoặc khối rồi tên lớp (1A).</t>
+          <t>Không bắt buộc. Mỗi dòng một lớp: cột Lớp ghi tên lớp tùy ý (vd 1/1, 1A, Lá 2), cột Khối ghi tên khối như ở các cột Khối &lt;tên&gt; của sheet CHƯƠNG TRÌNH HỌC (vd 1 hoặc Lá; trống: các chữ số đầu tên lớp), cột Cơ sở ghi tên cơ sở (điểm trường) lớp học, tùy ý, bao nhiêu cơ sở cũng được (trống: Cơ sở 1), cột Nhãn ghi các nhãn tự đặt cách nhau dấu phẩy (vd Song ngữ; không trùng tên lớp): cột Lớp của sheet LUẬT ghi nhãn hay tên cơ sở là mọi lớp có nhãn đó, ở cơ sở đó. Có sheet này thì danh sách lớp lấy ở đây: Chủ Nhiệm ghi Lớp là một lớp của sheet, lớp không có Chủ Nhiệm vẫn được xếp (các môn chia cho GV khác; môn Chỉ GVCN dạy, tiết Luôn do GVCN dạy, tiết HĐTN cố định của GVCN không áp dụng cho lớp đó). Không có sheet này (hoặc sheet trống) thì lớp là lớp của các dòng Chủ Nhiệm, ghi dạng khối/số thứ tự (1/1) hoặc khối rồi tên lớp (1A).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Overtime order set per person
Optional staff column "Thứ Tự Bù" gives who teaches overtime first
(1 = first, equal numbers share). Blank keeps the old order by role and
the Hợp Đồng column (homeroom contract 1, homeroom 2, general contract 3,
general 4) with the same four prices, so codes are unchanged; other
numbers spread over the same price range. The checker's "homeroom teacher
first in their own class" rule now applies only when the homeroom teacher
ranks first. A value on someone who cannot teach overtime gives a warning.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WtuWVKdziZbvQ9VXgRdGv
</commit_message>
<xml_diff>
--- a/data/Input_Template_V8.xlsx
+++ b/data/Input_Template_V8.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K300"/>
+  <dimension ref="A1:L300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -466,6 +466,7 @@
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -522,6 +523,11 @@
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Nhãn</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Thứ Tự Bù</t>
         </is>
       </c>
     </row>
@@ -537,6 +543,7 @@
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
       <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
     </row>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -550,6 +557,7 @@
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="2" t="n"/>
@@ -563,6 +571,7 @@
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
       <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
     </row>
     <row r="5" ht="25" customHeight="1">
       <c r="A5" s="2" t="n"/>
@@ -576,6 +585,7 @@
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
       <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
     </row>
     <row r="6" ht="25" customHeight="1">
       <c r="A6" s="2" t="n"/>
@@ -589,6 +599,7 @@
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
     </row>
     <row r="7" ht="25" customHeight="1">
       <c r="A7" s="2" t="n"/>
@@ -602,6 +613,7 @@
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
       <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
     </row>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="2" t="n"/>
@@ -615,6 +627,7 @@
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
       <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
     </row>
     <row r="9" ht="25" customHeight="1">
       <c r="A9" s="2" t="n"/>
@@ -628,6 +641,7 @@
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
     </row>
     <row r="10" ht="25" customHeight="1">
       <c r="A10" s="2" t="n"/>
@@ -641,6 +655,7 @@
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
       <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
     </row>
     <row r="11" ht="25" customHeight="1">
       <c r="A11" s="2" t="n"/>
@@ -654,6 +669,7 @@
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
       <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="C12" s="5" t="n"/>
@@ -6301,7 +6317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B67"/>
+  <dimension ref="A1:B68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -6328,7 +6344,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên một dòng. Bảy cột Thai Sản, Hợp Đồng, Cơ sở 2, Lớp Đang Dạy, Buổi Nghỉ, Chức Vụ Thêm, Nhãn không bắt buộc (để trống hoặc xóa cột).</t>
+          <t>Mỗi giáo viên một dòng. Tám cột Thai Sản, Hợp Đồng, Cơ sở 2, Lớp Đang Dạy, Buổi Nghỉ, Chức Vụ Thêm, Nhãn, Thứ Tự Bù không bắt buộc (để trống hoặc xóa cột).</t>
         </is>
       </c>
     </row>
@@ -6467,646 +6483,658 @@
     <row r="14" ht="25" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC</t>
+          <t>NHÂN SỰ: Thứ Tự Bù</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Mỗi môn một dòng: cột Môn học ghi tên môn (dùng đúng tên này ở sheet CHỨC VỤ, hoặc ở cột Chức Vụ của GV chuyên biệt chỉ dạy môn này), cột Khối &lt;tên&gt; ghi số tiết/tuần của môn ở khối đó (0 hoặc để trống: khối đó không học), các cột sau là quy định của môn. Tên khối tùy ý, vd Khối 1, Khối Lá; thêm khối thì thêm cột.</t>
+          <t>Ai dạy bù trước khi phải bù giờ: số nguyên dương, 1 là bù trước nhất; người cùng số bù ngang nhau. Để trống: GVCN hợp đồng 1, GVCN 2, bộ môn hợp đồng 3, bộ môn 4. Chỉ có tác dụng với người được dạy bù (sheet QUY ĐỊNH, không thai sản).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="25" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Quy ước các ô quy định</t>
+          <t>CHƯƠNG TRÌNH HỌC</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Mỗi quy định là một cột (bảng Quy định chung: một dòng). Mỗi ô chỉ ghi Có, Không hoặc một số nguyên dương; ô trống là Không. Riêng cột Tên trong TKB ghi chữ. Xóa một cột (một dòng của bảng chung, một bảng, hoặc cả sheet QUY ĐỊNH) thì quy định đó dùng giá trị mặc định của chương trình.</t>
+          <t>Mỗi môn một dòng: cột Môn học ghi tên môn (dùng đúng tên này ở sheet CHỨC VỤ, hoặc ở cột Chức Vụ của GV chuyên biệt chỉ dạy môn này), cột Khối &lt;tên&gt; ghi số tiết/tuần của môn ở khối đó (0 hoặc để trống: khối đó không học), các cột sau là quy định của môn. Tên khối tùy ý, vd Khối 1, Khối Lá; thêm khối thì thêm cột.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="25" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH</t>
+          <t>Quy ước các ô quy định</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Ba bảng cách nhau một dòng trống: Quy định | Giá trị; Ngày (mỗi dòng một ngày học, mỗi cột Buổi &lt;tên&gt; ghi số tiết của buổi đó); Tiết (đánh số liên tục trong ngày: sáng 4 tiết thì chiều từ tiết 5; ngày dài nhất có bao nhiêu tiết thì bấy nhiêu dòng).</t>
+          <t>Mỗi quy định là một cột (bảng Quy định chung: một dòng). Mỗi ô chỉ ghi Có, Không hoặc một số nguyên dương; ô trống là Không. Riêng cột Tên trong TKB ghi chữ. Xóa một cột (một dòng của bảng chung, một bảng, hoặc cả sheet QUY ĐỊNH) thì quy định đó dùng giá trị mặc định của chương trình.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="25" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Tên trong TKB</t>
+          <t>QUY ĐỊNH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Chữ ghi trong ô TKB (cột duy nhất ghi chữ); trống: ghi đúng tên môn.</t>
+          <t>Ba bảng cách nhau một dòng trống: Quy định | Giá trị; Ngày (mỗi dòng một ngày học, mỗi cột Buổi &lt;tên&gt; ghi số tiết của buổi đó); Tiết (đánh số liên tục trong ngày: sáng 4 tiết thì chiều từ tiết 5; ngày dài nhất có bao nhiêu tiết thì bấy nhiêu dòng).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="25" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Môn HĐTN</t>
+          <t>CHƯƠNG TRÌNH HỌC: Tên trong TKB</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Có ở một môn: môn chào cờ, sinh hoạt lớp, có tiết cố định ở bảng ngày của sheet QUY ĐỊNH.</t>
+          <t>Chữ ghi trong ô TKB (cột duy nhất ghi chữ); trống: ghi đúng tên môn.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="25" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận trọn</t>
+          <t>CHƯƠNG TRÌNH HỌC: Môn HĐTN</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>GVCN nhận hết các môn này của lớp mình; luật cứng: môn nào phải chia cho người khác thì tiết đầu tiên trong tuần do GVCN dạy.</t>
+          <t>Có ở một môn: môn chào cờ, sinh hoạt lớp, có tiết cố định ở bảng ngày của sheet QUY ĐỊNH.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN cắt bớt</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận trọn</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Số thứ tự 1, 2...: môn cắt trước khi các môn nhận trọn vượt định mức GVCN; mỗi môn GVCN giữ ít nhất 1 tiết.</t>
+          <t>GVCN nhận hết các môn này của lớp mình; luật cứng: môn nào phải chia cho người khác thì tiết đầu tiên trong tuần do GVCN dạy.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận thêm</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN cắt bớt</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Số thứ tự 1, 2...: môn GVCN nhận thêm trước cho đủ định mức (không nhận môn của GV chuyên biệt).</t>
+          <t>Số thứ tự 1, 2...: môn cắt trước khi các môn nhận trọn vượt định mức GVCN; mỗi môn GVCN giữ ít nhất 1 tiết.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Chỉ GVCN dạy</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận thêm</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: chỉ GVCN của lớp được dạy.</t>
+          <t>Số thứ tự 1, 2...: môn GVCN nhận thêm trước cho đủ định mức (không nhận môn của GV chuyên biệt).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="25" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Bộ Môn không dạy</t>
+          <t>CHƯƠNG TRÌNH HỌC: Chỉ GVCN dạy</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>GV bộ môn không dạy môn này; trường chưa có GV chuyên biệt của môn thì chương trình tuyển thêm. Ghi theo ngoại lệ để môn mới (ô trống) mặc nhiên bộ môn dạy được.</t>
+          <t>Luật cứng: chỉ GVCN của lớp được dạy.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="25" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Quản lý dạy khối</t>
+          <t>CHƯƠNG TRÌNH HỌC: Bộ Môn không dạy</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Khối mà Quản Lý được dạy môn này (tên khối như ở cột Khối &lt;tên&gt;), vd Kỹ năng sống: 4.</t>
+          <t>GV bộ môn không dạy môn này; trường chưa có GV chuyên biệt của môn thì chương trình tuyển thêm. Ghi theo ngoại lệ để môn mới (ô trống) mặc nhiên bộ môn dạy được.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="25" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN bù môn chuyên biệt</t>
+          <t>CHƯƠNG TRÌNH HỌC: Quản lý dạy khối</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Môn có GV chuyên biệt mà GVCN vẫn được dạy bù ở lớp mình (nhận sau cùng).</t>
+          <t>Khối mà Quản Lý được dạy môn này (tên khối như ở cột Khối &lt;tên&gt;), vd Kỹ năng sống: 4.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="25" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Nhóm môn</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN bù môn chuyên biệt</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Môn chính và các môn tăng cường của nó ghi cùng một số, vd Tiếng Việt và Tiếng Việt tăng cường: 1.</t>
+          <t>Môn có GV chuyên biệt mà GVCN vẫn được dạy bù ở lớp mình (nhận sau cùng).</t>
         </is>
       </c>
     </row>
     <row r="27" ht="25" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Môn tăng cường</t>
+          <t>CHƯƠNG TRÌNH HỌC: Nhóm môn</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Có ở môn tăng cường của nhóm; luật cứng: tiết tăng cường đứng sau mọi tiết môn chính trong ngày và ngày đó phải có tiết môn chính; cả nhóm tính chung cho giới hạn mỗi buổi và ghép cặp.</t>
+          <t>Môn chính và các môn tăng cường của nó ghi cùng một số, vd Tiếng Việt và Tiếng Việt tăng cường: 1.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="25" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Không ghép cặp</t>
+          <t>CHƯƠNG TRÌNH HỌC: Môn tăng cường</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Nhóm môn (ghi ở môn chính) không xếp thành cặp 2 tiết liền. Ghi theo ngoại lệ như cột Bộ Môn không dạy.</t>
+          <t>Có ở môn tăng cường của nhóm; luật cứng: tiết tăng cường đứng sau mọi tiết môn chính trong ngày và ngày đó phải có tiết môn chính; cả nhóm tính chung cho giới hạn mỗi buổi và ghép cặp.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="25" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Môn nặng</t>
+          <t>CHƯƠNG TRÌNH HỌC: Không ghép cặp</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu mềm: hạn chế xếp vào các tiết Hạn chế môn nặng (sheet QUY ĐỊNH).</t>
+          <t>Nhóm môn (ghi ở môn chính) không xếp thành cặp 2 tiết liền. Ghi theo ngoại lệ như cột Bộ Môn không dạy.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="25" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Ưu tiên buổi sáng</t>
+          <t>CHƯƠNG TRÌNH HỌC: Môn nặng</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu mềm: mỗi tiết ở buổi chiều bị trừ điểm, và môn được rải đều hơn trong tuần.</t>
+          <t>Mục tiêu mềm: hạn chế xếp vào các tiết Hạn chế môn nặng (sheet QUY ĐỊNH).</t>
         </is>
       </c>
     </row>
     <row r="31" ht="25" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Chủ Nhiệm được dạy bù</t>
+          <t>CHƯƠNG TRÌNH HỌC: Ưu tiên buổi sáng</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>GVCN chỉ bù ở lớp mình và bù trước bộ môn.</t>
+          <t>Mục tiêu mềm: mỗi tiết ở buổi chiều bị trừ điểm, và môn được rải đều hơn trong tuần.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="25" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Bộ Môn được dạy bù</t>
+          <t>QUY ĐỊNH: Chủ Nhiệm được dạy bù</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Bộ môn bù khi GVCN đã bù hết mức.</t>
+          <t>GVCN chỉ bù ở lớp mình và bù trước bộ môn.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="25" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Ngày, Buổi &lt;tên buổi&gt;</t>
+          <t>QUY ĐỊNH: Bộ Môn được dạy bù</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Bảng Ngày: mỗi dòng một ngày học, tên tùy ý (vd Thứ 2, Thứ 7, Chủ nhật), theo thứ tự trong tuần. Mỗi cột Buổi &lt;tên buổi&gt; (vd Buổi Sáng, Buổi Chiều, Buổi Tối) ghi số tiết của buổi đó trong ngày; ô trống là ngày đó không học buổi đó. Mỗi ngày một số tiết riêng được (vd chiều Thứ 5 có 4 tiết). Thêm buổi thì thêm cột, thêm ngày học thì thêm dòng; ngày không có tiết nào không phải ngày học. Tiết đánh số liên tục trong ngày theo thứ tự các cột buổi: sáng 4 tiết thì chiều bắt đầu từ tiết 5.</t>
+          <t>Bộ môn bù khi GVCN đã bù hết mức.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="25" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Tiết HĐTN cố định</t>
+          <t>QUY ĐỊNH: Ngày, Buổi &lt;tên buổi&gt;</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: tiết môn HĐTN cố định của ngày đó ở mọi lớp, vd Thứ 2: 1, Thứ 6: 4.</t>
+          <t>Bảng Ngày: mỗi dòng một ngày học, tên tùy ý (vd Thứ 2, Thứ 7, Chủ nhật), theo thứ tự trong tuần. Mỗi cột Buổi &lt;tên buổi&gt; (vd Buổi Sáng, Buổi Chiều, Buổi Tối) ghi số tiết của buổi đó trong ngày; ô trống là ngày đó không học buổi đó. Mỗi ngày một số tiết riêng được (vd chiều Thứ 5 có 4 tiết). Thêm buổi thì thêm cột, thêm ngày học thì thêm dòng; ngày không có tiết nào không phải ngày học. Tiết đánh số liên tục trong ngày theo thứ tự các cột buổi: sáng 4 tiết thì chiều bắt đầu từ tiết 5.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="25" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Xếp tiết HĐTN còn lại</t>
+          <t>QUY ĐỊNH: Tiết HĐTN cố định</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: các tiết HĐTN còn lại chỉ xếp vào các ngày này (mục tiêu mềm: gần cuối buổi).</t>
+          <t>Luật cứng: tiết môn HĐTN cố định của ngày đó ở mọi lớp, vd Thứ 2: 1, Thứ 6: 4.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="25" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Luôn do GVCN dạy</t>
+          <t>QUY ĐỊNH: Xếp tiết HĐTN còn lại</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: tiết này ở mọi ngày do GVCN của lớp dạy.</t>
+          <t>Luật cứng: các tiết HĐTN còn lại chỉ xếp vào các ngày này (mục tiêu mềm: gần cuối buổi).</t>
         </is>
       </c>
     </row>
     <row r="37" ht="25" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Hạn chế môn nặng</t>
+          <t>QUY ĐỊNH: Luôn do GVCN dạy</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu mềm: mỗi tiết môn nặng ở tiết này bị trừ điểm.</t>
+          <t>Luật cứng: tiết này ở mọi ngày do GVCN của lớp dạy.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="25" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>CHỨC VỤ</t>
+          <t>QUY ĐỊNH: Hạn chế môn nặng</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Không bắt buộc. Mỗi dòng một chức vụ GV chuyên biệt nhà trường tự đặt: cột Chức vụ ghi tên (không ghi số, không trùng Chủ Nhiệm, Bộ Môn, Quản Lý), cột Môn được dạy ghi các môn chức vụ đó dạy, cách nhau bằng dấu phẩy, đúng tên trong sheet CHƯƠNG TRÌNH HỌC, vd GV Nghệ thuật: Âm nhạc, Mỹ thuật. Ở sheet NHÂN SỰ, GV có Chức Vụ là tên đó chỉ dạy các môn này. Chức vụ không ghi ở đây mà trùng tên một môn (vd Tiếng Anh) thì chỉ dạy môn đó. Môn Bộ Môn không dạy mà chưa có GV nào dạy được thì chương trình tuyển thêm chức vụ đầu tiên ở đây dạy môn đó (không có thì chức vụ trùng tên môn).</t>
+          <t>Mục tiêu mềm: mỗi tiết môn nặng ở tiết này bị trừ điểm.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="25" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>LỚP</t>
+          <t>CHỨC VỤ</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Không bắt buộc. Mỗi dòng một lớp: cột Lớp ghi tên lớp tùy ý (vd 1/1, 1A, Lá 2), cột Khối ghi tên khối như ở các cột Khối &lt;tên&gt; của sheet CHƯƠNG TRÌNH HỌC (vd 1 hoặc Lá; trống: các chữ số đầu tên lớp), cột Cơ sở ghi tên cơ sở (điểm trường) lớp học, tùy ý, bao nhiêu cơ sở cũng được (trống: Cơ sở 1), cột Nhãn ghi các nhãn tự đặt cách nhau dấu phẩy (vd Song ngữ; không trùng tên lớp): cột Lớp của sheet LUẬT ghi nhãn hay tên cơ sở là mọi lớp có nhãn đó, ở cơ sở đó. Có sheet này thì danh sách lớp lấy ở đây: Chủ Nhiệm ghi Lớp là một lớp của sheet, lớp không có Chủ Nhiệm vẫn được xếp (các môn chia cho GV khác; môn Chỉ GVCN dạy, tiết Luôn do GVCN dạy, tiết HĐTN cố định của GVCN không áp dụng cho lớp đó). Không có sheet này (hoặc sheet trống) thì lớp là lớp của các dòng Chủ Nhiệm, ghi dạng khối/số thứ tự (1/1) hoặc khối rồi tên lớp (1A).</t>
+          <t>Không bắt buộc. Mỗi dòng một chức vụ GV chuyên biệt nhà trường tự đặt: cột Chức vụ ghi tên (không ghi số, không trùng Chủ Nhiệm, Bộ Môn, Quản Lý), cột Môn được dạy ghi các môn chức vụ đó dạy, cách nhau bằng dấu phẩy, đúng tên trong sheet CHƯƠNG TRÌNH HỌC, vd GV Nghệ thuật: Âm nhạc, Mỹ thuật. Ở sheet NHÂN SỰ, GV có Chức Vụ là tên đó chỉ dạy các môn này. Chức vụ không ghi ở đây mà trùng tên một môn (vd Tiếng Anh) thì chỉ dạy môn đó. Môn Bộ Môn không dạy mà chưa có GV nào dạy được thì chương trình tuyển thêm chức vụ đầu tiên ở đây dạy môn đó (không có thì chức vụ trùng tên môn).</t>
         </is>
       </c>
     </row>
     <row r="40" ht="25" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>LUẬT</t>
+          <t>LỚP</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Mọi luật xếp TKB, mỗi dòng một luật, đọc như một câu: Với mỗi [cột Với mỗi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Mỗi luật trả lời một trong bốn câu hỏi: Ở đâu, Bao nhiêu, Đi cùng nhau, Ai dạy (các kiểu luật và phép đo xếp theo câu hỏi ở dưới). File mẫu ghi sẵn các luật có sẵn của chương trình: sửa số hoặc Điểm để chỉnh, đổi Bắt buộc, xóa dòng để bỏ luật (hoặc ghi Có ở cột Tạm tắt: chương trình bỏ qua dòng đó mà vẫn giữ lại, xóa chữ Có là dùng lại), thêm dòng để có luật mới. Cột Nhóm và Luật đọc là chỉ để đọc (chương trình ghi lại mỗi lần). Kiểu luật: một mẫu hoặc Tự ghép; cột kiểu luật không dùng để trống. Bắt buộc: Có (luật cứng) hoặc Không (ưu tiên); luật ưu tiên ghi Mức Thấp, Vừa, Cao, Rất cao (100, 400, 1500, 5000 điểm) hoặc ghi thẳng Điểm (điểm trừ mỗi lần không theo). Môn, Lớp, Khối, Ngày, Tiết ghi danh sách cách nhau bằng dấu phẩy hoặc khoảng, vd 3, 4 hoặc 3-5; Thứ 2, Thứ 4 hoặc T2-T4; 5-7. Buổi: Sáng hoặc Chiều. Giáo viên: chức vụ (Chủ Nhiệm, Bộ Môn, Quản Lý hoặc chức vụ GV chuyên biệt), 'trừ Chủ Nhiệm' là mọi giáo viên trừ chức vụ đó; hoặc một người: Mã GV (vd Bộ Môn 3, Chủ Nhiệm 1/1, đánh số theo thứ tự dòng của sheet NHÂN SỰ) hay họ tên (hai người trùng tên thì ghi Mã GV), vd giờ bận: Không xếp vào, Giáo viên Bộ Môn 3, Thứ 2, tiết 1 (để trống Môn); ép phân công: Chỉ giáo viên dạy, Môn Tiếng Anh, Lớp 3/1, Giáo viên Tiếng Anh 2. Câu đọc lại ghi Mã GV, không ghi họ tên. Nhãn, Trừ nhãn: tên các cột Có/Không của môn (vd Môn nặng) hoặc của giờ học (ngày, tiết, vd Luôn do GVCN dạy); nhiều nhãn giờ học là giờ có một trong các nhãn. Gồm môn tăng cường: Có thì Môn tính cả các môn tăng cường cùng nhóm. Không có sheet này thì chương trình dùng các luật có sẵn và sheet LUẬT RIÊNG (file của bản trước).</t>
+          <t>Không bắt buộc. Mỗi dòng một lớp: cột Lớp ghi tên lớp tùy ý (vd 1/1, 1A, Lá 2), cột Khối ghi tên khối như ở các cột Khối &lt;tên&gt; của sheet CHƯƠNG TRÌNH HỌC (vd 1 hoặc Lá; trống: các chữ số đầu tên lớp), cột Cơ sở ghi tên cơ sở (điểm trường) lớp học, tùy ý, bao nhiêu cơ sở cũng được (trống: Cơ sở 1), cột Nhãn ghi các nhãn tự đặt cách nhau dấu phẩy (vd Song ngữ; không trùng tên lớp): cột Lớp của sheet LUẬT ghi nhãn hay tên cơ sở là mọi lớp có nhãn đó, ở cơ sở đó. Có sheet này thì danh sách lớp lấy ở đây: Chủ Nhiệm ghi Lớp là một lớp của sheet, lớp không có Chủ Nhiệm vẫn được xếp (các môn chia cho GV khác; môn Chỉ GVCN dạy, tiết Luôn do GVCN dạy, tiết HĐTN cố định của GVCN không áp dụng cho lớp đó). Không có sheet này (hoặc sheet trống) thì lớp là lớp của các dòng Chủ Nhiệm, ghi dạng khối/số thứ tự (1/1) hoặc khối rồi tên lớp (1A).</t>
         </is>
       </c>
     </row>
     <row r="41" ht="25" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Không xếp vào</t>
+          <t>LUẬT</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Môn (của các khối ở cột Khối; để trống: mọi khối) không xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục không xếp vào tiết 1; Tin học không xếp vào Thứ 2. Ghi Giáo viên (chức vụ, Mã GV hoặc họ tên) thì chỉ xét tiết của người đó, để trống Môn là mọi môn: giờ bận, vd Bộ Môn 3 không dạy Thứ 2 tiết 1.</t>
+          <t>Mọi luật xếp TKB, mỗi dòng một luật, đọc như một câu: Với mỗi [cột Với mỗi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Mỗi luật trả lời một trong bốn câu hỏi: Ở đâu, Bao nhiêu, Đi cùng nhau, Ai dạy (các kiểu luật và phép đo xếp theo câu hỏi ở dưới). File mẫu ghi sẵn các luật có sẵn của chương trình: sửa số hoặc Điểm để chỉnh, đổi Bắt buộc, xóa dòng để bỏ luật (hoặc ghi Có ở cột Tạm tắt: chương trình bỏ qua dòng đó mà vẫn giữ lại, xóa chữ Có là dùng lại), thêm dòng để có luật mới. Cột Nhóm và Luật đọc là chỉ để đọc (chương trình ghi lại mỗi lần). Kiểu luật: một mẫu hoặc Tự ghép; cột kiểu luật không dùng để trống. Bắt buộc: Có (luật cứng) hoặc Không (ưu tiên); luật ưu tiên ghi Mức Thấp, Vừa, Cao, Rất cao (100, 400, 1500, 5000 điểm) hoặc ghi thẳng Điểm (điểm trừ mỗi lần không theo). Môn, Lớp, Khối, Ngày, Tiết ghi danh sách cách nhau bằng dấu phẩy hoặc khoảng, vd 3, 4 hoặc 3-5; Thứ 2, Thứ 4 hoặc T2-T4; 5-7. Buổi: Sáng hoặc Chiều. Giáo viên: chức vụ (Chủ Nhiệm, Bộ Môn, Quản Lý hoặc chức vụ GV chuyên biệt), 'trừ Chủ Nhiệm' là mọi giáo viên trừ chức vụ đó; hoặc một người: Mã GV (vd Bộ Môn 3, Chủ Nhiệm 1/1, đánh số theo thứ tự dòng của sheet NHÂN SỰ) hay họ tên (hai người trùng tên thì ghi Mã GV), vd giờ bận: Không xếp vào, Giáo viên Bộ Môn 3, Thứ 2, tiết 1 (để trống Môn); ép phân công: Chỉ giáo viên dạy, Môn Tiếng Anh, Lớp 3/1, Giáo viên Tiếng Anh 2. Câu đọc lại ghi Mã GV, không ghi họ tên. Nhãn, Trừ nhãn: tên các cột Có/Không của môn (vd Môn nặng) hoặc của giờ học (ngày, tiết, vd Luôn do GVCN dạy); nhiều nhãn giờ học là giờ có một trong các nhãn. Gồm môn tăng cường: Có thì Môn tính cả các môn tăng cường cùng nhóm. Không có sheet này thì chương trình dùng các luật có sẵn và sheet LUẬT RIÊNG (file của bản trước).</t>
         </is>
       </c>
     </row>
     <row r="42" ht="25" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Chỉ xếp vào</t>
+          <t>LUẬT: Ở đâu · Không xếp vào</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Môn chỉ xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục chỉ xếp vào buổi chiều. Ghi Giáo viên thì chỉ xét tiết của người đó (để trống Môn: mọi môn), vd Bộ Môn 3 chỉ dạy buổi sáng.</t>
+          <t>Môn (của các khối ở cột Khối; để trống: mọi khối) không xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục không xếp vào tiết 1; Tin học không xếp vào Thứ 2. Ghi Giáo viên (chức vụ, Mã GV hoặc họ tên) thì chỉ xét tiết của người đó, để trống Môn là mọi môn: giờ bận, vd Bộ Môn 3 không dạy Thứ 2 tiết 1.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="25" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Cố định vào</t>
+          <t>LUẬT: Ở đâu · Chỉ xếp vào</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Mỗi lớp (của các khối, lớp ghi ở dòng này) học đúng 1 tiết của Môn ở mỗi giờ ghi ở cột Ngày, Tiết, Buổi, vd Thể dục khối 1 cố định vào Thứ 3 tiết 3.</t>
+          <t>Môn chỉ xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục chỉ xếp vào buổi chiều. Ghi Giáo viên thì chỉ xét tiết của người đó (để trống Môn: mọi môn), vd Bộ Môn 3 chỉ dạy buổi sáng.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="25" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Giáo viên tối đa tiết mỗi ngày</t>
+          <t>LUẬT: Ở đâu · Cố định vào</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số tiết mỗi ngày.</t>
+          <t>Mỗi lớp (của các khối, lớp ghi ở dòng này) học đúng 1 tiết của Môn ở mỗi giờ ghi ở cột Ngày, Tiết, Buổi, vd Thể dục khối 1 cố định vào Thứ 3 tiết 3.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="25" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Giáo viên tối đa lớp mỗi ngày</t>
+          <t>LUẬT: Bao nhiêu · Giáo viên tối đa tiết mỗi ngày</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số lớp khác nhau mỗi ngày.</t>
+          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số tiết mỗi ngày.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="25" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Số lớp học cùng lúc tối đa</t>
+          <t>LUẬT: Bao nhiêu · Giáo viên tối đa lớp mỗi ngày</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Môn có tối đa Số lớp học cùng một giờ (cả trường, hoặc các khối ở cột Khối), vd phòng Tin học: 1, sân Thể dục: 2.</t>
+          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số lớp khác nhau mỗi ngày.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="25" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Học ít nhất số ngày</t>
+          <t>LUẬT: Bao nhiêu · Số lớp học cùng lúc tối đa</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Mỗi lớp học Môn ở ít nhất Số ngày khác nhau trong tuần, vd Tiếng Anh ít nhất 3 ngày.</t>
+          <t>Môn có tối đa Số lớp học cùng một giờ (cả trường, hoặc các khối ở cột Khối), vd phòng Tin học: 1, sân Thể dục: 2.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="25" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Học 2 tiết liền</t>
+          <t>LUẬT: Bao nhiêu · Học ít nhất số ngày</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Môn học thành cặp 2 tiết liền, cùng người dạy: mỗi buổi 0 hoặc 2 tiết của môn (tính chung môn tăng cường cùng nhóm), vd Tiếng Anh. Bắt buộc thì số tiết/tuần phải chẵn.</t>
+          <t>Mỗi lớp học Môn ở ít nhất Số ngày khác nhau trong tuần, vd Tiếng Anh ít nhất 3 ngày.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="25" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Học trước</t>
+          <t>LUẬT: Đi cùng nhau · Học 2 tiết liền</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Trong một buổi có cả hai môn thì Môn học trước Môn thứ hai, vd Tiếng Việt trước Toán.</t>
+          <t>Môn học thành cặp 2 tiết liền, cùng người dạy: mỗi buổi 0 hoặc 2 tiết của môn (tính chung môn tăng cường cùng nhóm), vd Tiếng Anh. Bắt buộc thì số tiết/tuần phải chẵn.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="25" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Chỉ giáo viên dạy</t>
+          <t>LUẬT: Đi cùng nhau · Học trước</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Các tiết của Môn (ở các khối, lớp, ngày, tiết ghi ở dòng này) chỉ do giáo viên ghi ở cột Giáo viên dạy: chức vụ, vd Tin học khối 3 chỉ GV Tin Học dạy; hoặc một người (Mã GV hay họ tên) để chọn ai dạy lớp nào, vd Tiếng Anh lớp 3/1 chỉ Tiếng Anh 2 dạy.</t>
+          <t>Trong một buổi có cả hai môn thì Môn học trước Môn thứ hai, vd Tiếng Việt trước Toán.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="25" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Buổi nghỉ của giáo viên</t>
+          <t>LUẬT: Ai dạy · Chỉ giáo viên dạy</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Giáo viên không dạy vào các buổi nghỉ ghi ở cột Buổi Nghỉ (sheet NHÂN SỰ) và nghỉ đủ số buổi ghi ở đó. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
+          <t>Các tiết của Môn (ở các khối, lớp, ngày, tiết ghi ở dòng này) chỉ do giáo viên ghi ở cột Giáo viên dạy: chức vụ, vd Tin học khối 3 chỉ GV Tin Học dạy; hoặc một người (Mã GV hay họ tên) để chọn ai dạy lớp nào, vd Tiếng Anh lớp 3/1 chỉ Tiếng Anh 2 dạy.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="25" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Giáo viên chỉ dạy cơ sở 2</t>
+          <t>LUẬT: Ai dạy · Buổi nghỉ của giáo viên</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Giáo viên không chủ nhiệm ghi Có ở cột Cơ sở 2 hoặc Thai Sản (sheet NHÂN SỰ) chỉ dạy các lớp ở cơ sở 2. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
+          <t>Giáo viên không dạy vào các buổi nghỉ ghi ở cột Buổi Nghỉ (sheet NHÂN SỰ) và nghỉ đủ số buổi ghi ở đó. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="25" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép</t>
+          <t>LUẬT: Ai dạy · Giáo viên chỉ dạy cơ sở 2</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Tự ghép câu luật: Với mỗi [phạm vi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Xem các phép đo ở dưới.</t>
+          <t>Giáo viên không chủ nhiệm ghi Có ở cột Cơ sở 2 hoặc Thai Sản (sheet NHÂN SỰ) chỉ dạy các lớp ở cơ sở 2. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="25" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Với mỗi</t>
+          <t>LUẬT: Tự ghép</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Chia các tiết thành từng nhóm theo các chiều, vd 'Lớp, Ngày': luật áp dụng cho mỗi lớp mỗi ngày. Các chiều: Lớp, Giáo viên, Môn, Nhóm môn, Khối, Ngày, Buổi, Giờ học, Cơ sở. Trống: cả trường cả tuần.</t>
+          <t>Tự ghép câu luật: Với mỗi [phạm vi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Xem các phép đo ở dưới.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="25" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Tự ghép, Phép đo Vị trí</t>
+          <t>LUẬT: Tự ghép, cột Với mỗi</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Các tiết chỉ xếp vào, hoặc không xếp vào, các ngày, tiết, buổi (hoặc giờ có nhãn) ghi ở dòng này. So sánh: Chỉ trong, Không trong.</t>
+          <t>Chia các tiết thành từng nhóm theo các chiều, vd 'Lớp, Ngày': luật áp dụng cho mỗi lớp mỗi ngày. Các chiều: Lớp, Giáo viên, Môn, Nhóm môn, Khối, Ngày, Buổi, Giờ học, Cơ sở. Trống: cả trường cả tuần.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="25" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số tiết</t>
+          <t>LUẬT: Ở đâu · Tự ghép, Phép đo Vị trí</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Đếm số tiết trong mỗi phạm vi, vd mỗi lớp mỗi ngày học tối đa 1 tiết Toán; mỗi giờ học có tối đa 1 tiết Tin học. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số.</t>
+          <t>Các tiết chỉ xếp vào, hoặc không xếp vào, các ngày, tiết, buổi (hoặc giờ có nhãn) ghi ở dòng này. So sánh: Chỉ trong, Không trong.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="25" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số khác nhau</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số tiết</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Đếm số lớp, ngày, cơ sở… khác nhau (cột Đếm theo), vd mỗi giáo viên mỗi ngày dạy tối đa 3 lớp; mỗi lớp học Tiếng Anh ít nhất 3 ngày. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số. Ghi cột Đếm theo.</t>
+          <t>Đếm số tiết trong mỗi phạm vi, vd mỗi lớp mỗi ngày học tối đa 1 tiết Toán; mỗi giờ học có tối đa 1 tiết Tin học. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="25" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Khoảng cách</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số khác nhau</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Số tiết trống xen giữa các tiết trong buổi (0: không có tiết trống); hoặc số tiết từ tiết đó đến cuối buổi (0: ở tiết cuối buổi). So sánh: Tiết trống tối đa, Cách cuối buổi tối đa. Ghi cột Số.</t>
+          <t>Đếm số lớp, ngày, cơ sở… khác nhau (cột Đếm theo), vd mỗi giáo viên mỗi ngày dạy tối đa 3 lớp; mỗi lớp học Tiếng Anh ít nhất 3 ngày. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số. Ghi cột Đếm theo.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="25" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Liền nhau</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Khoảng cách</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Các tiết trong một buổi (của mỗi lớp hoặc giáo viên) đứng liền nhau, không có tiết khác xen giữa.</t>
+          <t>Số tiết trống xen giữa các tiết trong buổi (0: không có tiết trống); hoặc số tiết từ tiết đó đến cuối buổi (0: ở tiết cuối buổi). So sánh: Tiết trống tối đa, Cách cuối buổi tối đa. Ghi cột Số.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="25" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Theo cặp 2 tiết</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Liền nhau</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Mỗi buổi học 0 hoặc 2 tiết, 2 tiết đó liền nhau (ưu tiên: hạn chế tiết lẻ đứng một mình).</t>
+          <t>Các tiết trong một buổi (của mỗi lớp hoặc giáo viên) đứng liền nhau, không có tiết khác xen giữa.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="25" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Thứ tự</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Theo cặp 2 tiết</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Trong một buổi (hoặc ngày, nếu Với mỗi có Ngày) tiết của Môn đứng trước (hoặc sau) tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm. So sánh: Trước, Sau.</t>
+          <t>Mỗi buổi học 0 hoặc 2 tiết, 2 tiết đó liền nhau (ưu tiên: hạn chế tiết lẻ đứng một mình).</t>
         </is>
       </c>
     </row>
     <row r="62" ht="25" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Đi kèm</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Thứ tự</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Buổi (hoặc ngày) có tiết của Môn thì cũng có tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm.</t>
+          <t>Trong một buổi (hoặc ngày, nếu Với mỗi có Ngày) tiết của Môn đứng trước (hoặc sau) tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm. So sánh: Trước, Sau.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="25" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Tự ghép, Phép đo Người dạy</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Đi kèm</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Các tiết do giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên) dạy; hoặc do cùng một người dạy; hoặc hai tiết liền nhau do cùng một người; hoặc tiết đầu tuần do giáo viên đó dạy, tiết của người khác không đứng trước. So sánh: Do, Cùng một người, Liền nhau cùng người, Tiết đầu tuần do.</t>
+          <t>Buổi (hoặc ngày) có tiết của Môn thì cũng có tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="25" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Số</t>
+          <t>LUẬT: Ai dạy · Tự ghép, Phép đo Người dạy</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Một số nguyên, hoặc (phép đo Số tiết) một ngưỡng theo dữ liệu: tải ngày, tải ngày + 1, số tiết/tuần chia số ngày (tải ngày: định mức của giáo viên chia theo số tiết của ngày).</t>
+          <t>Các tiết do giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên) dạy; hoặc do cùng một người dạy; hoặc hai tiết liền nhau do cùng một người; hoặc tiết đầu tuần do giáo viên đó dạy, tiết của người khác không đứng trước. So sánh: Do, Cùng một người, Liền nhau cùng người, Tiết đầu tuần do.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="25" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Áp dụng khi</t>
+          <t>LUẬT: Tự ghép, cột Số</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Chỉ áp dụng khi số tiết/tuần của các môn ở cột Môn (phạm vi có Môn, Nhóm môn: của từng môn, nhóm môn) ở khối đó thỏa điều kiện, vd '&gt;= 6, chẵn' (từ 6 tiết trở lên và chẵn) hoặc '&lt;= số ngày' (không quá số ngày học).</t>
+          <t>Một số nguyên, hoặc (phép đo Số tiết) một ngưỡng theo dữ liệu: tải ngày, tải ngày + 1, số tiết/tuần chia số ngày (tải ngày: định mức của giáo viên chia theo số tiết của ngày).</t>
         </is>
       </c>
     </row>
     <row r="66" ht="25" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: cấu trúc của TKB</t>
+          <t>LUẬT: Tự ghép, cột Áp dụng khi</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Cấu trúc của TKB (không phải luật, luôn có): mỗi lớp mỗi giờ học một tiết; mỗi lớp học đủ số tiết của chương trình học; giáo viên không dạy hai nơi cùng lúc, dạy không quá định mức (cộng số tiết bù tối đa ở chế độ bù giờ), Quản Lý dạy đúng định mức; giáo viên chỉ dạy các môn chức vụ được dạy (sheet CHƯƠNG TRÌNH HỌC, CHỨC VỤ).</t>
+          <t>Chỉ áp dụng khi số tiết/tuần của các môn ở cột Môn (phạm vi có Môn, Nhóm môn: của từng môn, nhóm môn) ở khối đó thỏa điều kiện, vd '&gt;= 6, chẵn' (từ 6 tiết trở lên và chẵn) hoặc '&lt;= số ngày' (không quá số ngày học).</t>
         </is>
       </c>
     </row>
     <row r="67" ht="25" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
+          <t>LUẬT: cấu trúc của TKB</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Cấu trúc của TKB (không phải luật, luôn có): mỗi lớp mỗi giờ học một tiết; mỗi lớp học đủ số tiết của chương trình học; giáo viên không dạy hai nơi cùng lúc, dạy không quá định mức (cộng số tiết bù tối đa ở chế độ bù giờ), Quản Lý dạy đúng định mức; giáo viên chỉ dạy các môn chức vụ được dạy (sheet CHƯƠNG TRÌNH HỌC, CHỨC VỤ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="25" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
           <t>Kiểu chữ</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>Các file kết quả chép kiểu chữ, cỡ chữ, viền của sheet NHÂN SỰ. Chỉ cần chữ và số: không cần công thức, màu nền, ghi chú trong ô hay danh sách thả xuống.</t>
         </is>

</xml_diff>

<commit_message>
Read hand-filled Excel files leniently and explain mistakes clearly
- Sheet and column names match without accents, case, spaces or punctuation;
  common header aliases (Họ tên, Số tiết, Định mức, STT); two-row headers with
  vertically merged cells; near-miss sheet and column names are warned about.
- Yes/no cells accept ✓, v, Đúng, ko...; roles accept GVCN, GV bộ môn, CBQL;
  Lớp Đang Dạy accepts ";", "+", "&" and "và".
- Merged data cells are spread to every row with a warning; hidden rows warn.
- Clear errors: quota above the week's periods, duplicate names (Mã GV only),
  "Tổng" rows skipped, name suggestions for roles and LUẬT subjects, non-.xlsx
  files explained without a traceback.
- Template gets a "Bắt đầu nhanh" guide; page wording without jargon; import
  dialog no longer says "0 ngày học".

Result codes are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WtuWVKdziZbvQ9VXgRdGv
</commit_message>
<xml_diff>
--- a/data/Input_Template_V8.xlsx
+++ b/data/Input_Template_V8.xlsx
@@ -7303,7 +7303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B72"/>
+  <dimension ref="A1:B76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -7325,850 +7325,898 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ</t>
+          <t>BẮT ĐẦU NHANH</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên một dòng. Tám cột Thai Sản, Hợp Đồng, Cơ sở 2, Lớp Đang Dạy, Buổi Nghỉ, Chức Vụ Thêm, Nhãn, Thứ Tự Bù không bắt buộc (để trống hoặc xóa cột).</t>
+          <t>Chỉ cần điền hai sheet: NHÂN SỰ (bốn cột đầu: Họ và Tên, Chức Vụ, Lớp, Số Tiết/Tuần) và CHƯƠNG TRÌNH HỌC (số tiết/tuần của từng môn ở các cột Khối). Các sheet, các cột khác đã có sẵn giá trị mặc định: để nguyên nếu trường không cần.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ: Họ và Tên</t>
+          <t>BẮT ĐẦU NHANH: Chức Vụ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Tên giáo viên; người chưa tuyển được ghi "chưa có".</t>
+          <t>Chủ Nhiệm (ghi lớp ở cột Lớp, vd 1/1), Bộ Môn, Quản Lý, hoặc tên môn GV chuyên dạy (vd Tiếng Anh). Không ghi số thứ tự.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ: Chức Vụ</t>
+          <t>BẮT ĐẦU NHANH: lưu ý</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Chủ Nhiệm, Bộ Môn, Quản Lý, một chức vụ của sheet CHỨC VỤ hoặc tên một môn trong sheet CHƯƠNG TRÌNH HỌC (GV chuyên biệt). Không ghi số thứ tự: chương trình tự đánh số theo thứ tự dòng.</t>
+          <t>Giữ nguyên tên sheet và tên cột. Người đã nghỉ thì xóa hẳn dòng (dòng ẩn vẫn được tính). Ô Có/Không ghi Có hoặc để trống. Lưu file dạng Excel .xlsx.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="25" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ: Lớp</t>
+          <t>BẮT ĐẦU NHANH: không cần Excel</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Chỉ ghi cho Chủ Nhiệm: một lớp của sheet LỚP; sheet LỚP trống thì ghi dạng khối/số thứ tự (vd 1/1) hoặc khối rồi tên lớp (vd 1D15). Mỗi lớp nhiều nhất một Chủ Nhiệm.</t>
+          <t>Mở trang nhập liệu (TKB.exe hoặc giao_dien.py), chọn Soạn mới, rồi dán danh sách giáo viên chép từ Excel (nút Dán từ Excel… ở bước Giáo viên).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="25" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ: Số Tiết/Tuần</t>
+          <t>NHÂN SỰ</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Số tiết tối đa mỗi tuần (số nguyên).</t>
+          <t>Mỗi giáo viên một dòng. Tám cột Thai Sản, Hợp Đồng, Cơ sở 2, Lớp Đang Dạy, Buổi Nghỉ, Chức Vụ Thêm, Nhãn, Thứ Tự Bù không bắt buộc (để trống hoặc xóa cột).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="25" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ: Thai Sản</t>
+          <t>NHÂN SỰ: Họ và Tên</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Ghi Có nếu đang hưởng chế độ thai sản: không dạy bù, chỉ dạy các lớp ở cơ sở 2.</t>
+          <t>Tên giáo viên; người chưa tuyển được ghi "chưa có".</t>
         </is>
       </c>
     </row>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ: Hợp Đồng</t>
+          <t>NHÂN SỰ: Chức Vụ</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Ghi Có nếu là GV hợp đồng: khi phải bù, GVCN hợp đồng bù trước GVCN khác, bộ môn hợp đồng bù trước bộ môn khác.</t>
+          <t>Chủ Nhiệm, Bộ Môn, Quản Lý, một chức vụ của sheet CHỨC VỤ hoặc tên một môn trong sheet CHƯƠNG TRÌNH HỌC (GV chuyên biệt). Không ghi số thứ tự: chương trình tự đánh số theo thứ tự dòng.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="25" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ: Cơ sở 2</t>
+          <t>NHÂN SỰ: Lớp</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Dòng Chủ Nhiệm: ghi Có nếu lớp học ở cơ sở 2 (hoặc ghi ở sheet LỚP). Dòng khác: ghi Có nếu GV chỉ dạy ở cơ sở 2. Mỗi buổi, một GV chỉ dạy ở một cơ sở.</t>
+          <t>Chỉ ghi cho Chủ Nhiệm: một lớp của sheet LỚP; sheet LỚP trống thì ghi dạng khối/số thứ tự (vd 1/1) hoặc khối rồi tên lớp (vd 1D15). Mỗi lớp nhiều nhất một Chủ Nhiệm.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="25" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ: Lớp Đang Dạy</t>
+          <t>NHÂN SỰ: Số Tiết/Tuần</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>GV bộ môn, chuyên biệt: các lớp đang dạy trong TKB cũ, cách nhau bằng dấu phẩy (vd 3D17, 3D18). TKB mới ưu tiên giữ khối, rồi giữ lớp.</t>
+          <t>Số tiết tối đa mỗi tuần (số nguyên).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="25" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ: Buổi Nghỉ</t>
+          <t>NHÂN SỰ: Thai Sản</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Buổi không xếp tiết: buổi cố định (vd Chiều T5, Sáng T6) hoặc số buổi bất kỳ (vd 2 buổi chiều), cách nhau bằng dấu phẩy. GVCN không nghỉ được buổi có tiết Luôn do GVCN dạy (sheet QUY ĐỊNH).</t>
+          <t>Ghi Có nếu đang hưởng chế độ thai sản: không dạy bù, chỉ dạy các lớp ở cơ sở 2.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="25" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ: Chức Vụ Thêm</t>
+          <t>NHÂN SỰ: Hợp Đồng</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Các chức vụ khác người này cũng giữ, cách nhau bằng dấu phẩy: Bộ Môn hoặc chức vụ GV chuyên biệt (vd Tiếng Anh). Người đó dạy được cả các môn của các chức vụ này, ở mọi lớp, trong định mức; vd Chủ Nhiệm ghi Bộ Môn thì dạy được cả các lớp khác. Chủ Nhiệm có chức vụ thêm dạy phần GVCN nhận trọn của lớp mình (không nhận thêm cho đủ định mức), phần định mức còn lại dùng cho chức vụ thêm. Mã GV theo chức vụ chính (cột Chức Vụ).</t>
+          <t>Ghi Có nếu là GV hợp đồng: khi phải bù, GVCN hợp đồng bù trước GVCN khác, bộ môn hợp đồng bù trước bộ môn khác.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="25" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ: Nhãn</t>
+          <t>NHÂN SỰ: Cơ sở 2</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Các nhãn tự đặt, cách nhau bằng dấu phẩy (vd Bán thời gian, Tổ Toán). Cột Giáo viên của sheet LUẬT ghi một nhãn là mọi GV có nhãn đó, vd luật Bán thời gian không dạy buổi chiều. Thai Sản, Hợp Đồng, Cơ sở 2 ghi Có cũng là nhãn cùng tên.</t>
+          <t>Dòng Chủ Nhiệm: ghi Có nếu lớp học ở cơ sở 2 (hoặc ghi ở sheet LỚP). Dòng khác: ghi Có nếu GV chỉ dạy ở cơ sở 2. Mỗi buổi, một GV chỉ dạy ở một cơ sở.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="25" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>NHÂN SỰ: Thứ Tự Bù</t>
+          <t>NHÂN SỰ: Lớp Đang Dạy</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Ai dạy bù trước khi phải bù giờ: số nguyên dương, 1 là bù trước nhất; người cùng số bù ngang nhau. Để trống: GVCN hợp đồng 1, GVCN 2, bộ môn hợp đồng 3, bộ môn 4. Chỉ có tác dụng với người được dạy bù (sheet QUY ĐỊNH, không thai sản).</t>
+          <t>GV bộ môn, chuyên biệt: các lớp đang dạy trong TKB cũ, cách nhau bằng dấu phẩy (vd 3D17, 3D18). TKB mới ưu tiên giữ khối, rồi giữ lớp.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="25" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC</t>
+          <t>NHÂN SỰ: Buổi Nghỉ</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Mỗi môn một dòng: cột Môn học ghi tên môn (dùng đúng tên này ở sheet CHỨC VỤ, hoặc ở cột Chức Vụ của GV chuyên biệt chỉ dạy môn này), cột Khối &lt;tên&gt; ghi số tiết/tuần của môn ở khối đó (0 hoặc để trống: khối đó không học), các cột sau là quy định của môn. Tên khối tùy ý, vd Khối 1, Khối Lá; thêm khối thì thêm cột.</t>
+          <t>Buổi không xếp tiết: buổi cố định (vd Chiều T5, Sáng T6) hoặc số buổi bất kỳ (vd 2 buổi chiều), cách nhau bằng dấu phẩy. GVCN không nghỉ được buổi có tiết Luôn do GVCN dạy (sheet QUY ĐỊNH).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="25" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Quy ước các ô quy định</t>
+          <t>NHÂN SỰ: Chức Vụ Thêm</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Mỗi quy định là một cột (bảng Quy định chung: một dòng). Mỗi ô chỉ ghi Có, Không hoặc một số nguyên dương; ô trống là Không. Riêng cột Tên trong TKB ghi chữ. Xóa một cột (một dòng của bảng chung, một bảng, hoặc cả sheet QUY ĐỊNH) thì quy định đó dùng giá trị mặc định của chương trình.</t>
+          <t>Các chức vụ khác người này cũng giữ, cách nhau bằng dấu phẩy: Bộ Môn hoặc chức vụ GV chuyên biệt (vd Tiếng Anh). Người đó dạy được cả các môn của các chức vụ này, ở mọi lớp, trong định mức; vd Chủ Nhiệm ghi Bộ Môn thì dạy được cả các lớp khác. Chủ Nhiệm có chức vụ thêm dạy phần GVCN nhận trọn của lớp mình (không nhận thêm cho đủ định mức), phần định mức còn lại dùng cho chức vụ thêm. Mã GV theo chức vụ chính (cột Chức Vụ).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="25" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH</t>
+          <t>NHÂN SỰ: Nhãn</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Ba bảng cách nhau một dòng trống: Quy định | Giá trị; Ngày (mỗi dòng một ngày học, mỗi cột Buổi &lt;tên&gt; ghi số tiết của buổi đó); Tiết (đánh số liên tục trong ngày: sáng 4 tiết thì chiều từ tiết 5; ngày dài nhất có bao nhiêu tiết thì bấy nhiêu dòng).</t>
+          <t>Các nhãn tự đặt, cách nhau bằng dấu phẩy (vd Bán thời gian, Tổ Toán). Cột Giáo viên của sheet LUẬT ghi một nhãn là mọi GV có nhãn đó, vd luật Bán thời gian không dạy buổi chiều. Thai Sản, Hợp Đồng, Cơ sở 2 ghi Có cũng là nhãn cùng tên.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="25" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Tên trong TKB</t>
+          <t>NHÂN SỰ: Thứ Tự Bù</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Chữ ghi trong ô TKB (cột duy nhất ghi chữ); trống: ghi đúng tên môn.</t>
+          <t>Ai dạy bù trước khi phải bù giờ: số nguyên dương, 1 là bù trước nhất; người cùng số bù ngang nhau. Để trống: GVCN hợp đồng 1, GVCN 2, bộ môn hợp đồng 3, bộ môn 4. Chỉ có tác dụng với người được dạy bù (sheet QUY ĐỊNH, không thai sản).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="25" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Môn HĐTN</t>
+          <t>CHƯƠNG TRÌNH HỌC</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Có ở một môn: môn chào cờ, sinh hoạt lớp, có tiết cố định ở bảng ngày của sheet QUY ĐỊNH.</t>
+          <t>Mỗi môn một dòng: cột Môn học ghi tên môn (dùng đúng tên này ở sheet CHỨC VỤ, hoặc ở cột Chức Vụ của GV chuyên biệt chỉ dạy môn này), cột Khối &lt;tên&gt; ghi số tiết/tuần của môn ở khối đó (0 hoặc để trống: khối đó không học), các cột sau là quy định của môn. Tên khối tùy ý, vd Khối 1, Khối Lá; thêm khối thì thêm cột.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận trọn</t>
+          <t>Quy ước các ô quy định</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>GVCN nhận hết các môn này của lớp mình; luật cứng: môn nào phải chia cho người khác thì tiết đầu tiên trong tuần do GVCN dạy.</t>
+          <t>Mỗi quy định là một cột (bảng Quy định chung: một dòng). Mỗi ô chỉ ghi Có, Không hoặc một số nguyên dương; ô trống là Không. Riêng cột Tên trong TKB ghi chữ. Xóa một cột (một dòng của bảng chung, một bảng, hoặc cả sheet QUY ĐỊNH) thì quy định đó dùng giá trị mặc định của chương trình.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN cắt bớt</t>
+          <t>QUY ĐỊNH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Số thứ tự 1, 2...: môn cắt trước khi các môn nhận trọn vượt định mức GVCN; mỗi môn GVCN giữ ít nhất 1 tiết.</t>
+          <t>Ba bảng cách nhau một dòng trống: Quy định | Giá trị; Ngày (mỗi dòng một ngày học, mỗi cột Buổi &lt;tên&gt; ghi số tiết của buổi đó); Tiết (đánh số liên tục trong ngày: sáng 4 tiết thì chiều từ tiết 5; ngày dài nhất có bao nhiêu tiết thì bấy nhiêu dòng).</t>
         </is>
       </c>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận thêm</t>
+          <t>CHƯƠNG TRÌNH HỌC: Tên trong TKB</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Số thứ tự 1, 2...: môn GVCN nhận thêm trước cho đủ định mức (không nhận môn của GV chuyên biệt).</t>
+          <t>Chữ ghi trong ô TKB (cột duy nhất ghi chữ); trống: ghi đúng tên môn.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="25" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Chỉ GVCN dạy</t>
+          <t>CHƯƠNG TRÌNH HỌC: Môn HĐTN</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: chỉ GVCN của lớp được dạy.</t>
+          <t>Có ở một môn: môn chào cờ, sinh hoạt lớp, có tiết cố định ở bảng ngày của sheet QUY ĐỊNH.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="25" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Bộ Môn không dạy</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận trọn</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>GV bộ môn không dạy môn này; trường chưa có GV chuyên biệt của môn thì chương trình tuyển thêm. Ghi theo ngoại lệ để môn mới (ô trống) mặc nhiên bộ môn dạy được.</t>
+          <t>GVCN nhận hết các môn này của lớp mình; luật cứng: môn nào phải chia cho người khác thì tiết đầu tiên trong tuần do GVCN dạy.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="25" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Quản lý dạy khối</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN cắt bớt</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Khối mà Quản Lý được dạy môn này (tên khối như ở cột Khối &lt;tên&gt;), vd Kỹ năng sống: 4.</t>
+          <t>Số thứ tự 1, 2...: môn cắt trước khi các môn nhận trọn vượt định mức GVCN; mỗi môn GVCN giữ ít nhất 1 tiết.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="25" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: GVCN bù môn chuyên biệt</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN nhận thêm</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Môn có GV chuyên biệt mà GVCN vẫn được dạy bù ở lớp mình (nhận sau cùng).</t>
+          <t>Số thứ tự 1, 2...: môn GVCN nhận thêm trước cho đủ định mức (không nhận môn của GV chuyên biệt).</t>
         </is>
       </c>
     </row>
     <row r="27" ht="25" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Nhóm môn</t>
+          <t>CHƯƠNG TRÌNH HỌC: Chỉ GVCN dạy</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Môn chính và các môn tăng cường của nó ghi cùng một số, vd Tiếng Việt và Tiếng Việt tăng cường: 1.</t>
+          <t>Luật cứng: chỉ GVCN của lớp được dạy.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="25" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Môn tăng cường</t>
+          <t>CHƯƠNG TRÌNH HỌC: Bộ Môn không dạy</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Có ở môn tăng cường của nhóm; luật cứng: tiết tăng cường đứng sau mọi tiết môn chính trong ngày và ngày đó phải có tiết môn chính; cả nhóm tính chung cho giới hạn mỗi buổi và ghép cặp.</t>
+          <t>GV bộ môn không dạy môn này; trường chưa có GV chuyên biệt của môn thì chương trình tuyển thêm. Ghi theo ngoại lệ để môn mới (ô trống) mặc nhiên bộ môn dạy được.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="25" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Không ghép cặp</t>
+          <t>CHƯƠNG TRÌNH HỌC: Quản lý dạy khối</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Nhóm môn (ghi ở môn chính) không xếp thành cặp 2 tiết liền. Ghi theo ngoại lệ như cột Bộ Môn không dạy.</t>
+          <t>Khối mà Quản Lý được dạy môn này (tên khối như ở cột Khối &lt;tên&gt;), vd Kỹ năng sống: 4.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="25" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Môn nặng</t>
+          <t>CHƯƠNG TRÌNH HỌC: GVCN bù môn chuyên biệt</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu mềm: hạn chế xếp vào các tiết Hạn chế môn nặng (sheet QUY ĐỊNH).</t>
+          <t>Môn có GV chuyên biệt mà GVCN vẫn được dạy bù ở lớp mình (nhận sau cùng).</t>
         </is>
       </c>
     </row>
     <row r="31" ht="25" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CHƯƠNG TRÌNH HỌC: Ưu tiên buổi sáng</t>
+          <t>CHƯƠNG TRÌNH HỌC: Nhóm môn</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu mềm: mỗi tiết ở buổi chiều bị trừ điểm, và môn được rải đều hơn trong tuần.</t>
+          <t>Môn chính và các môn tăng cường của nó ghi cùng một số, vd Tiếng Việt và Tiếng Việt tăng cường: 1.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="25" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Chủ Nhiệm được dạy bù</t>
+          <t>CHƯƠNG TRÌNH HỌC: Môn tăng cường</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>GVCN chỉ bù ở lớp mình và bù trước bộ môn.</t>
+          <t>Có ở môn tăng cường của nhóm; luật cứng: tiết tăng cường đứng sau mọi tiết môn chính trong ngày và ngày đó phải có tiết môn chính; cả nhóm tính chung cho giới hạn mỗi buổi và ghép cặp.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="25" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Bộ Môn được dạy bù</t>
+          <t>CHƯƠNG TRÌNH HỌC: Không ghép cặp</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Bộ môn bù khi GVCN đã bù hết mức.</t>
+          <t>Nhóm môn (ghi ở môn chính) không xếp thành cặp 2 tiết liền. Ghi theo ngoại lệ như cột Bộ Môn không dạy.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="25" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Ngày, Buổi &lt;tên buổi&gt;</t>
+          <t>CHƯƠNG TRÌNH HỌC: Môn nặng</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Bảng Ngày: mỗi dòng một ngày học, tên tùy ý (vd Thứ 2, Thứ 7, Chủ nhật), theo thứ tự trong tuần. Mỗi cột Buổi &lt;tên buổi&gt; (vd Buổi Sáng, Buổi Chiều, Buổi Tối) ghi số tiết của buổi đó trong ngày; ô trống là ngày đó không học buổi đó. Mỗi ngày một số tiết riêng được (vd chiều Thứ 5 có 4 tiết). Thêm buổi thì thêm cột, thêm ngày học thì thêm dòng; ngày không có tiết nào không phải ngày học. Tiết đánh số liên tục trong ngày theo thứ tự các cột buổi: sáng 4 tiết thì chiều bắt đầu từ tiết 5.</t>
+          <t>Mục tiêu mềm: hạn chế xếp vào các tiết Hạn chế môn nặng (sheet QUY ĐỊNH).</t>
         </is>
       </c>
     </row>
     <row r="35" ht="25" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Tiết HĐTN cố định</t>
+          <t>CHƯƠNG TRÌNH HỌC: Ưu tiên buổi sáng</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: tiết môn HĐTN cố định của ngày đó ở mọi lớp, vd Thứ 2: 1, Thứ 6: 4.</t>
+          <t>Mục tiêu mềm: mỗi tiết ở buổi chiều bị trừ điểm, và môn được rải đều hơn trong tuần.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="25" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Xếp tiết HĐTN còn lại</t>
+          <t>QUY ĐỊNH: Chủ Nhiệm được dạy bù</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: các tiết HĐTN còn lại chỉ xếp vào các ngày này (mục tiêu mềm: gần cuối buổi).</t>
+          <t>GVCN chỉ bù ở lớp mình và bù trước bộ môn.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="25" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Luôn do GVCN dạy</t>
+          <t>QUY ĐỊNH: Bộ Môn được dạy bù</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Luật cứng: tiết này ở mọi ngày do GVCN của lớp dạy.</t>
+          <t>Bộ môn bù khi GVCN đã bù hết mức.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="25" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>QUY ĐỊNH: Hạn chế môn nặng</t>
+          <t>QUY ĐỊNH: Ngày, Buổi &lt;tên buổi&gt;</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu mềm: mỗi tiết môn nặng ở tiết này bị trừ điểm.</t>
+          <t>Bảng Ngày: mỗi dòng một ngày học, tên tùy ý (vd Thứ 2, Thứ 7, Chủ nhật), theo thứ tự trong tuần. Mỗi cột Buổi &lt;tên buổi&gt; (vd Buổi Sáng, Buổi Chiều, Buổi Tối) ghi số tiết của buổi đó trong ngày; ô trống là ngày đó không học buổi đó. Mỗi ngày một số tiết riêng được (vd chiều Thứ 5 có 4 tiết). Thêm buổi thì thêm cột, thêm ngày học thì thêm dòng; ngày không có tiết nào không phải ngày học. Tiết đánh số liên tục trong ngày theo thứ tự các cột buổi: sáng 4 tiết thì chiều bắt đầu từ tiết 5.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="25" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>CHỨC VỤ</t>
+          <t>QUY ĐỊNH: Tiết HĐTN cố định</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Không bắt buộc. Mỗi dòng một chức vụ GV chuyên biệt nhà trường tự đặt: cột Chức vụ ghi tên (không ghi số, không trùng Chủ Nhiệm, Bộ Môn, Quản Lý), cột Môn được dạy ghi các môn chức vụ đó dạy, cách nhau bằng dấu phẩy, đúng tên trong sheet CHƯƠNG TRÌNH HỌC, vd GV Nghệ thuật: Âm nhạc, Mỹ thuật. Ở sheet NHÂN SỰ, GV có Chức Vụ là tên đó chỉ dạy các môn này. Chức vụ không ghi ở đây mà trùng tên một môn (vd Tiếng Anh) thì chỉ dạy môn đó. Môn Bộ Môn không dạy mà chưa có GV nào dạy được thì chương trình tuyển thêm chức vụ đầu tiên ở đây dạy môn đó (không có thì chức vụ trùng tên môn).</t>
+          <t>Luật cứng: tiết môn HĐTN cố định của ngày đó ở mọi lớp, vd Thứ 2: 1, Thứ 6: 4.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="25" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>LỚP</t>
+          <t>QUY ĐỊNH: Xếp tiết HĐTN còn lại</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Không bắt buộc. Mỗi dòng một lớp: cột Lớp ghi tên lớp tùy ý (vd 1/1, 1A, Lá 2), cột Khối ghi tên khối như ở các cột Khối &lt;tên&gt; của sheet CHƯƠNG TRÌNH HỌC (vd 1 hoặc Lá; trống: các chữ số đầu tên lớp), cột Cơ sở ghi tên cơ sở (điểm trường) lớp học, tùy ý, bao nhiêu cơ sở cũng được (trống: Cơ sở 1), cột Nhãn ghi các nhãn tự đặt cách nhau dấu phẩy (vd Song ngữ; không trùng tên lớp): cột Lớp của sheet LUẬT ghi nhãn hay tên cơ sở là mọi lớp có nhãn đó, ở cơ sở đó. Có sheet này thì danh sách lớp lấy ở đây: Chủ Nhiệm ghi Lớp là một lớp của sheet, lớp không có Chủ Nhiệm vẫn được xếp (các môn chia cho GV khác; môn Chỉ GVCN dạy, tiết Luôn do GVCN dạy, tiết HĐTN cố định của GVCN không áp dụng cho lớp đó). Không có sheet này (hoặc sheet trống) thì lớp là lớp của các dòng Chủ Nhiệm, ghi dạng khối/số thứ tự (1/1) hoặc khối rồi tên lớp (1A).</t>
+          <t>Luật cứng: các tiết HĐTN còn lại chỉ xếp vào các ngày này (mục tiêu mềm: gần cuối buổi).</t>
         </is>
       </c>
     </row>
     <row r="41" ht="25" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>PHÒNG</t>
+          <t>QUY ĐỊNH: Luôn do GVCN dạy</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Không bắt buộc. Mỗi dòng một phòng học dùng chung (phòng Tin, phòng đa năng, sân trường): cột Phòng ghi tên phòng, cột Cơ sở ghi tên cơ sở như cột Cơ sở của sheet LỚP (trống: Cơ sở 1), cột Môn ghi các môn học ở phòng này cách nhau dấu phẩy (đúng tên trong sheet CHƯƠNG TRÌNH HỌC, hoặc một nhãn môn là tiêu đề một cột Có/Không của sheet đó), cột Khối ghi các khối dùng phòng (trống: mọi khối), cột Sức chứa ghi số lớp học cùng lúc trong phòng (trống: 1; vd sân trường 3). Luật cứng: tiết của môn, khối, cơ sở có phòng ghi ở đây phải học ở một phòng như vậy, mỗi giờ học không quá sức chứa; tên phòng ghi trong TKB và file TKB phòng. Môn không có phòng nào ghi thì học ở lớp.</t>
+          <t>Luật cứng: tiết này ở mọi ngày do GVCN của lớp dạy.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="25" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>LUẬT</t>
+          <t>QUY ĐỊNH: Hạn chế môn nặng</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Mọi luật xếp TKB, mỗi dòng một luật, đọc như một câu: Với mỗi [cột Với mỗi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Mỗi luật trả lời một trong bốn câu hỏi: Ở đâu, Bao nhiêu, Đi cùng nhau, Ai dạy (các kiểu luật và phép đo xếp theo câu hỏi ở dưới). File mẫu ghi sẵn các luật có sẵn của chương trình: sửa số hoặc Điểm để chỉnh, đổi Bắt buộc, xóa dòng để bỏ luật (hoặc ghi Có ở cột Tạm tắt: chương trình bỏ qua dòng đó mà vẫn giữ lại, xóa chữ Có là dùng lại), thêm dòng để có luật mới. Cột Nhóm và Luật đọc là chỉ để đọc (chương trình ghi lại mỗi lần). Kiểu luật: một mẫu hoặc Tự ghép; cột kiểu luật không dùng để trống. Bắt buộc: Có (luật cứng) hoặc Không (ưu tiên); luật ưu tiên ghi Mức Thấp, Vừa, Cao, Rất cao (100, 400, 1500, 5000 điểm) hoặc ghi thẳng Điểm (điểm trừ mỗi lần không theo). Môn, Lớp, Khối, Ngày, Tiết ghi danh sách cách nhau bằng dấu phẩy hoặc khoảng, vd 3, 4 hoặc 3-5; Thứ 2, Thứ 4 hoặc T2-T4; 5-7. Buổi: Sáng hoặc Chiều. Giáo viên: chức vụ (Chủ Nhiệm, Bộ Môn, Quản Lý hoặc chức vụ GV chuyên biệt), 'trừ Chủ Nhiệm' là mọi giáo viên trừ chức vụ đó; hoặc một người: Mã GV (vd Bộ Môn 3, Chủ Nhiệm 1/1, đánh số theo thứ tự dòng của sheet NHÂN SỰ) hay họ tên (hai người trùng tên thì ghi Mã GV), vd giờ bận: Không xếp vào, Giáo viên Bộ Môn 3, Thứ 2, tiết 1 (để trống Môn); ép phân công: Chỉ giáo viên dạy, Môn Tiếng Anh, Lớp 3/1, Giáo viên Tiếng Anh 2. Câu đọc lại ghi Mã GV, không ghi họ tên. Nhãn, Trừ nhãn: tên các cột Có/Không của môn (vd Môn nặng) hoặc của giờ học (ngày, tiết, vd Luôn do GVCN dạy); nhiều nhãn giờ học là giờ có một trong các nhãn. Gồm môn tăng cường: Có thì Môn tính cả các môn tăng cường cùng nhóm. Không có sheet này thì chương trình dùng các luật có sẵn và sheet LUẬT RIÊNG (file của bản trước).</t>
+          <t>Mục tiêu mềm: mỗi tiết môn nặng ở tiết này bị trừ điểm.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="25" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Không xếp vào</t>
+          <t>CHỨC VỤ</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Môn (của các khối ở cột Khối; để trống: mọi khối) không xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục không xếp vào tiết 1; Tin học không xếp vào Thứ 2. Ghi Giáo viên (chức vụ, Mã GV hoặc họ tên) thì chỉ xét tiết của người đó, để trống Môn là mọi môn: giờ bận, vd Bộ Môn 3 không dạy Thứ 2 tiết 1.</t>
+          <t>Không bắt buộc. Mỗi dòng một chức vụ GV chuyên biệt nhà trường tự đặt: cột Chức vụ ghi tên (không ghi số, không trùng Chủ Nhiệm, Bộ Môn, Quản Lý), cột Môn được dạy ghi các môn chức vụ đó dạy, cách nhau bằng dấu phẩy, đúng tên trong sheet CHƯƠNG TRÌNH HỌC, vd GV Nghệ thuật: Âm nhạc, Mỹ thuật. Ở sheet NHÂN SỰ, GV có Chức Vụ là tên đó chỉ dạy các môn này. Chức vụ không ghi ở đây mà trùng tên một môn (vd Tiếng Anh) thì chỉ dạy môn đó. Môn Bộ Môn không dạy mà chưa có GV nào dạy được thì chương trình tuyển thêm chức vụ đầu tiên ở đây dạy môn đó (không có thì chức vụ trùng tên môn).</t>
         </is>
       </c>
     </row>
     <row r="44" ht="25" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Chỉ xếp vào</t>
+          <t>LỚP</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Môn chỉ xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục chỉ xếp vào buổi chiều. Ghi Giáo viên thì chỉ xét tiết của người đó (để trống Môn: mọi môn), vd Bộ Môn 3 chỉ dạy buổi sáng.</t>
+          <t>Không bắt buộc. Mỗi dòng một lớp: cột Lớp ghi tên lớp tùy ý (vd 1/1, 1A, Lá 2), cột Khối ghi tên khối như ở các cột Khối &lt;tên&gt; của sheet CHƯƠNG TRÌNH HỌC (vd 1 hoặc Lá; trống: các chữ số đầu tên lớp), cột Cơ sở ghi tên cơ sở (điểm trường) lớp học, tùy ý, bao nhiêu cơ sở cũng được (trống: Cơ sở 1), cột Nhãn ghi các nhãn tự đặt cách nhau dấu phẩy (vd Song ngữ; không trùng tên lớp): cột Lớp của sheet LUẬT ghi nhãn hay tên cơ sở là mọi lớp có nhãn đó, ở cơ sở đó. Có sheet này thì danh sách lớp lấy ở đây: Chủ Nhiệm ghi Lớp là một lớp của sheet, lớp không có Chủ Nhiệm vẫn được xếp (các môn chia cho GV khác; môn Chỉ GVCN dạy, tiết Luôn do GVCN dạy, tiết HĐTN cố định của GVCN không áp dụng cho lớp đó). Không có sheet này (hoặc sheet trống) thì lớp là lớp của các dòng Chủ Nhiệm, ghi dạng khối/số thứ tự (1/1) hoặc khối rồi tên lớp (1A).</t>
         </is>
       </c>
     </row>
     <row r="45" ht="25" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Cố định vào</t>
+          <t>PHÒNG</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Mỗi lớp (của các khối, lớp ghi ở dòng này) học đúng 1 tiết của Môn ở mỗi giờ ghi ở cột Ngày, Tiết, Buổi, vd Thể dục khối 1 cố định vào Thứ 3 tiết 3.</t>
+          <t>Không bắt buộc. Mỗi dòng một phòng học dùng chung (phòng Tin, phòng đa năng, sân trường): cột Phòng ghi tên phòng, cột Cơ sở ghi tên cơ sở như cột Cơ sở của sheet LỚP (trống: Cơ sở 1), cột Môn ghi các môn học ở phòng này cách nhau dấu phẩy (đúng tên trong sheet CHƯƠNG TRÌNH HỌC, hoặc một nhãn môn là tiêu đề một cột Có/Không của sheet đó), cột Khối ghi các khối dùng phòng (trống: mọi khối), cột Sức chứa ghi số lớp học cùng lúc trong phòng (trống: 1; vd sân trường 3). Luật cứng: tiết của môn, khối, cơ sở có phòng ghi ở đây phải học ở một phòng như vậy, mỗi giờ học không quá sức chứa; tên phòng ghi trong TKB và file TKB phòng. Môn không có phòng nào ghi thì học ở lớp.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="25" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Giáo viên tối đa tiết mỗi ngày</t>
+          <t>LUẬT</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số tiết mỗi ngày.</t>
+          <t>Mọi luật xếp TKB, mỗi dòng một luật, đọc như một câu: Với mỗi [cột Với mỗi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Mỗi luật trả lời một trong bốn câu hỏi: Ở đâu, Bao nhiêu, Đi cùng nhau, Ai dạy (các kiểu luật và phép đo xếp theo câu hỏi ở dưới). File mẫu ghi sẵn các luật có sẵn của chương trình: sửa số hoặc Điểm để chỉnh, đổi Bắt buộc, xóa dòng để bỏ luật (hoặc ghi Có ở cột Tạm tắt: chương trình bỏ qua dòng đó mà vẫn giữ lại, xóa chữ Có là dùng lại), thêm dòng để có luật mới. Cột Nhóm và Luật đọc là chỉ để đọc (chương trình ghi lại mỗi lần). Kiểu luật: một mẫu hoặc Tự ghép; cột kiểu luật không dùng để trống. Bắt buộc: Có (luật cứng) hoặc Không (ưu tiên); luật ưu tiên ghi Mức Thấp, Vừa, Cao, Rất cao (100, 400, 1500, 5000 điểm) hoặc ghi thẳng Điểm (điểm trừ mỗi lần không theo). Môn, Lớp, Khối, Ngày, Tiết ghi danh sách cách nhau bằng dấu phẩy hoặc khoảng, vd 3, 4 hoặc 3-5; Thứ 2, Thứ 4 hoặc T2-T4; 5-7. Buổi: Sáng hoặc Chiều. Giáo viên: chức vụ (Chủ Nhiệm, Bộ Môn, Quản Lý hoặc chức vụ GV chuyên biệt), 'trừ Chủ Nhiệm' là mọi giáo viên trừ chức vụ đó; hoặc một người: Mã GV (vd Bộ Môn 3, Chủ Nhiệm 1/1, đánh số theo thứ tự dòng của sheet NHÂN SỰ) hay họ tên (hai người trùng tên thì ghi Mã GV), vd giờ bận: Không xếp vào, Giáo viên Bộ Môn 3, Thứ 2, tiết 1 (để trống Môn); ép phân công: Chỉ giáo viên dạy, Môn Tiếng Anh, Lớp 3/1, Giáo viên Tiếng Anh 2. Câu đọc lại ghi Mã GV, không ghi họ tên. Nhãn, Trừ nhãn: tên các cột Có/Không của môn (vd Môn nặng) hoặc của giờ học (ngày, tiết, vd Luôn do GVCN dạy); nhiều nhãn giờ học là giờ có một trong các nhãn. Gồm môn tăng cường: Có thì Môn tính cả các môn tăng cường cùng nhóm. Không có sheet này thì chương trình dùng các luật có sẵn và sheet LUẬT RIÊNG (file của bản trước).</t>
         </is>
       </c>
     </row>
     <row r="47" ht="25" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Giáo viên tối đa lớp mỗi ngày</t>
+          <t>LUẬT: Ở đâu · Không xếp vào</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số lớp khác nhau mỗi ngày.</t>
+          <t>Môn (của các khối ở cột Khối; để trống: mọi khối) không xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục không xếp vào tiết 1; Tin học không xếp vào Thứ 2. Ghi Giáo viên (chức vụ, Mã GV hoặc họ tên) thì chỉ xét tiết của người đó, để trống Môn là mọi môn: giờ bận, vd Bộ Môn 3 không dạy Thứ 2 tiết 1.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="25" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Số lớp học cùng lúc tối đa</t>
+          <t>LUẬT: Ở đâu · Chỉ xếp vào</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Môn có tối đa Số lớp học cùng một giờ (cả trường, hoặc các khối ở cột Khối), vd phòng Tin học: 1, sân Thể dục: 2.</t>
+          <t>Môn chỉ xếp vào các ngày, tiết, buổi ghi ở dòng này (ghi ít nhất một trong ba cột), vd Thể dục chỉ xếp vào buổi chiều. Ghi Giáo viên thì chỉ xét tiết của người đó (để trống Môn: mọi môn), vd Bộ Môn 3 chỉ dạy buổi sáng.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="25" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Học ít nhất số ngày</t>
+          <t>LUẬT: Ở đâu · Cố định vào</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Mỗi lớp học Môn ở ít nhất Số ngày khác nhau trong tuần, vd Tiếng Anh ít nhất 3 ngày.</t>
+          <t>Mỗi lớp (của các khối, lớp ghi ở dòng này) học đúng 1 tiết của Môn ở mỗi giờ ghi ở cột Ngày, Tiết, Buổi, vd Thể dục khối 1 cố định vào Thứ 3 tiết 3.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="25" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Học 2 tiết liền</t>
+          <t>LUẬT: Bao nhiêu · Giáo viên tối đa tiết mỗi ngày</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Môn học thành cặp 2 tiết liền, cùng người dạy: mỗi buổi 0 hoặc 2 tiết của môn (tính chung môn tăng cường cùng nhóm), vd Tiếng Anh. Bắt buộc thì số tiết/tuần phải chẵn.</t>
+          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số tiết mỗi ngày.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="25" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Học trước</t>
+          <t>LUẬT: Bao nhiêu · Giáo viên tối đa lớp mỗi ngày</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Trong một buổi có cả hai môn thì Môn học trước Môn thứ hai, vd Tiếng Việt trước Toán.</t>
+          <t>Mỗi giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên; để trống: mọi giáo viên) dạy tối đa Số lớp khác nhau mỗi ngày.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="25" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Học cùng giờ</t>
+          <t>LUẬT: Bao nhiêu · Số lớp học cùng lúc tối đa</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Mỗi lớp (của các khối, lớp ghi ở dòng này) học Môn và các môn ở cột Môn thứ hai cùng giờ, cùng số tiết mỗi tuần, mỗi môn một người dạy, lớp tính một tiết ở giờ đó. Dùng cho lớp chia nhóm, vd nửa lớp học Tin học, nửa lớp học Tiếng Anh; hoặc giáo viên dạy kèm: ghi môn riêng Trợ giảng Tiếng Anh (cùng số tiết, chức vụ Trợ Giảng dạy) học cùng giờ với Tiếng Anh. Chỉ ghi Bắt buộc = Có.</t>
+          <t>Môn có tối đa Số lớp học cùng một giờ (cả trường, hoặc các khối ở cột Khối), vd phòng Tin học: 1, sân Thể dục: 2.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="25" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Ghép lớp</t>
+          <t>LUẬT: Bao nhiêu · Học ít nhất số ngày</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Các lớp ghi ở cột Lớp (hoặc các lớp của khối ở cột Khối) học chung Môn: cùng giờ, cùng số tiết mỗi tuần, một người dạy cả nhóm, người đó tính một tiết ở giờ đó, vd Thể dục lớp 3/1, 3/2 học chung một sân. Ghi Môn thứ hai thì lớp có môn đó học chung với các lớp có Môn (mỗi lớp một môn), vd lớp ghép hai khối. Muốn ghép riêng từng khối: dùng Tự ghép, Với mỗi Khối. Chỉ ghi Bắt buộc = Có.</t>
+          <t>Mỗi lớp học Môn ở ít nhất Số ngày khác nhau trong tuần, vd Tiếng Anh ít nhất 3 ngày.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="25" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Chỉ giáo viên dạy</t>
+          <t>LUẬT: Đi cùng nhau · Học 2 tiết liền</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Các tiết của Môn (ở các khối, lớp, ngày, tiết ghi ở dòng này) chỉ do giáo viên ghi ở cột Giáo viên dạy: chức vụ, vd Tin học khối 3 chỉ GV Tin Học dạy; hoặc một người (Mã GV hay họ tên) để chọn ai dạy lớp nào, vd Tiếng Anh lớp 3/1 chỉ Tiếng Anh 2 dạy.</t>
+          <t>Môn học thành cặp 2 tiết liền, cùng người dạy: mỗi buổi 0 hoặc 2 tiết của môn (tính chung môn tăng cường cùng nhóm), vd Tiếng Anh. Bắt buộc thì số tiết/tuần phải chẵn.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="25" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Buổi nghỉ của giáo viên</t>
+          <t>LUẬT: Đi cùng nhau · Học trước</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Giáo viên không dạy vào các buổi nghỉ ghi ở cột Buổi Nghỉ (sheet NHÂN SỰ) và nghỉ đủ số buổi ghi ở đó. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
+          <t>Trong một buổi có cả hai môn thì Môn học trước Môn thứ hai, vd Tiếng Việt trước Toán.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="25" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Giáo viên chỉ dạy cơ sở 2</t>
+          <t>LUẬT: Đi cùng nhau · Học cùng giờ</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Giáo viên không chủ nhiệm ghi Có ở cột Cơ sở 2 hoặc Thai Sản (sheet NHÂN SỰ) chỉ dạy các lớp ở cơ sở 2. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
+          <t>Mỗi lớp (của các khối, lớp ghi ở dòng này) học Môn và các môn ở cột Môn thứ hai cùng giờ, cùng số tiết mỗi tuần, mỗi môn một người dạy, lớp tính một tiết ở giờ đó. Dùng cho lớp chia nhóm, vd nửa lớp học Tin học, nửa lớp học Tiếng Anh; hoặc giáo viên dạy kèm: ghi môn riêng Trợ giảng Tiếng Anh (cùng số tiết, chức vụ Trợ Giảng dạy) học cùng giờ với Tiếng Anh. Chỉ ghi Bắt buộc = Có.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="25" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép</t>
+          <t>LUẬT: Đi cùng nhau · Ghép lớp</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Tự ghép câu luật: Với mỗi [phạm vi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Xem các phép đo ở dưới.</t>
+          <t>Các lớp ghi ở cột Lớp (hoặc các lớp của khối ở cột Khối) học chung Môn: cùng giờ, cùng số tiết mỗi tuần, một người dạy cả nhóm, người đó tính một tiết ở giờ đó, vd Thể dục lớp 3/1, 3/2 học chung một sân. Ghi Môn thứ hai thì lớp có môn đó học chung với các lớp có Môn (mỗi lớp một môn), vd lớp ghép hai khối. Muốn ghép riêng từng khối: dùng Tự ghép, Với mỗi Khối. Chỉ ghi Bắt buộc = Có.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="25" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Với mỗi</t>
+          <t>LUẬT: Ai dạy · Chỉ giáo viên dạy</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Chia các tiết thành từng nhóm theo các chiều, vd 'Lớp, Ngày': luật áp dụng cho mỗi lớp mỗi ngày. Các chiều: Lớp, Giáo viên, Môn, Nhóm môn, Khối, Ngày, Buổi, Giờ học, Cơ sở. Trống: cả trường cả tuần.</t>
+          <t>Các tiết của Môn (ở các khối, lớp, ngày, tiết ghi ở dòng này) chỉ do giáo viên ghi ở cột Giáo viên dạy: chức vụ, vd Tin học khối 3 chỉ GV Tin Học dạy; hoặc một người (Mã GV hay họ tên) để chọn ai dạy lớp nào, vd Tiếng Anh lớp 3/1 chỉ Tiếng Anh 2 dạy.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="25" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ở đâu · Tự ghép, Phép đo Vị trí</t>
+          <t>LUẬT: Ai dạy · Buổi nghỉ của giáo viên</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Các tiết chỉ xếp vào, hoặc không xếp vào, các ngày, tiết, buổi (hoặc giờ có nhãn) ghi ở dòng này. So sánh: Chỉ trong, Không trong.</t>
+          <t>Giáo viên không dạy vào các buổi nghỉ ghi ở cột Buổi Nghỉ (sheet NHÂN SỰ) và nghỉ đủ số buổi ghi ở đó. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="25" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số tiết</t>
+          <t>LUẬT: Ai dạy · Giáo viên chỉ dạy cơ sở 2</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Đếm số tiết trong mỗi phạm vi, vd mỗi lớp mỗi ngày học tối đa 1 tiết Toán; mỗi giờ học có tối đa 1 tiết Tin học. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số.</t>
+          <t>Giáo viên không chủ nhiệm ghi Có ở cột Cơ sở 2 hoặc Thai Sản (sheet NHÂN SỰ) chỉ dạy các lớp ở cơ sở 2. Chỉ ghi Bắt buộc = Có; muốn bỏ luật thì xóa dòng hoặc ghi Tạm tắt = Có.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="25" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số khác nhau</t>
+          <t>LUẬT: Tự ghép</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Đếm số lớp, ngày, cơ sở… khác nhau (cột Đếm theo), vd mỗi giáo viên mỗi ngày dạy tối đa 3 lớp; mỗi lớp học Tiếng Anh ít nhất 3 ngày. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số. Ghi cột Đếm theo.</t>
+          <t>Tự ghép câu luật: Với mỗi [phạm vi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Xem các phép đo ở dưới.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="25" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Khoảng cách</t>
+          <t>LUẬT: Tự ghép, cột Với mỗi</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Số tiết trống xen giữa các tiết trong buổi (0: không có tiết trống); hoặc số tiết từ tiết đó đến cuối buổi (0: ở tiết cuối buổi). So sánh: Tiết trống tối đa, Cách cuối buổi tối đa. Ghi cột Số.</t>
+          <t>Chia các tiết thành từng nhóm theo các chiều, vd 'Lớp, Ngày': luật áp dụng cho mỗi lớp mỗi ngày. Các chiều: Lớp, Giáo viên, Môn, Nhóm môn, Khối, Ngày, Buổi, Giờ học, Cơ sở. Trống: cả trường cả tuần.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="25" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Liền nhau</t>
+          <t>LUẬT: Ở đâu · Tự ghép, Phép đo Vị trí</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Các tiết trong một buổi (của mỗi lớp hoặc giáo viên) đứng liền nhau, không có tiết khác xen giữa.</t>
+          <t>Các tiết chỉ xếp vào, hoặc không xếp vào, các ngày, tiết, buổi (hoặc giờ có nhãn) ghi ở dòng này. So sánh: Chỉ trong, Không trong.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="25" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Theo cặp 2 tiết</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số tiết</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Mỗi buổi học 0 hoặc 2 tiết, 2 tiết đó liền nhau (ưu tiên: hạn chế tiết lẻ đứng một mình).</t>
+          <t>Đếm số tiết trong mỗi phạm vi, vd mỗi lớp mỗi ngày học tối đa 1 tiết Toán; mỗi giờ học có tối đa 1 tiết Tin học. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="25" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Thứ tự</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Số khác nhau</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Trong một buổi (hoặc ngày, nếu Với mỗi có Ngày) tiết của Môn đứng trước (hoặc sau) tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm. So sánh: Trước, Sau.</t>
+          <t>Đếm số lớp, ngày, cơ sở… khác nhau (cột Đếm theo), vd mỗi giáo viên mỗi ngày dạy tối đa 3 lớp; mỗi lớp học Tiếng Anh ít nhất 3 ngày. So sánh: Tối đa, Tối thiểu, Đúng. Ghi cột Số. Ghi cột Đếm theo.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="25" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Đi kèm</t>
+          <t>LUẬT: Bao nhiêu · Tự ghép, Phép đo Khoảng cách</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Buổi (hoặc ngày) có tiết của Môn thì cũng có tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm.</t>
+          <t>Số tiết trống xen giữa các tiết trong buổi (0: không có tiết trống); hoặc số tiết từ tiết đó đến cuối buổi (0: ở tiết cuối buổi). So sánh: Tiết trống tối đa, Cách cuối buổi tối đa. Ghi cột Số.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="25" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Cùng giờ</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Liền nhau</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Các tiết luôn học cùng giờ, cùng số tiết mỗi tuần; chỉ ghi Bắt buộc. Mỗi môn một người (để trống So sánh): mỗi lớp học Môn và Môn thứ hai cùng giờ, lớp tính một tiết ở giờ đó: lớp chia nhóm (mỗi nhóm học một môn, mỗi môn một người dạy) hoặc giáo viên chính và trợ giảng (ghi trợ giảng thành một môn riêng, vd Trợ giảng Tiếng Anh); Với mỗi là Lớp. Cùng một người: ghép lớp, các lớp (của cả trường, hoặc mỗi khối, mỗi cơ sở ở cột Với mỗi) học Môn (và Môn thứ hai nếu ghi) cùng giờ, một người dạy, người đó tính một tiết ở giờ đó. So sánh: Mỗi môn một người, Cùng một người.</t>
+          <t>Các tiết trong một buổi (của mỗi lớp hoặc giáo viên) đứng liền nhau, không có tiết khác xen giữa.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="25" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Ai dạy · Tự ghép, Phép đo Người dạy</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Theo cặp 2 tiết</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Các tiết do giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên) dạy; hoặc do cùng một người dạy; hoặc hai tiết liền nhau do cùng một người; hoặc tiết đầu tuần do giáo viên đó dạy, tiết của người khác không đứng trước. So sánh: Do, Cùng một người, Liền nhau cùng người, Tiết đầu tuần do.</t>
+          <t>Mỗi buổi học 0 hoặc 2 tiết, 2 tiết đó liền nhau (ưu tiên: hạn chế tiết lẻ đứng một mình).</t>
         </is>
       </c>
     </row>
     <row r="69" ht="25" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Số</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Thứ tự</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Một số nguyên, hoặc (phép đo Số tiết) một ngưỡng theo dữ liệu: tải ngày, tải ngày + 1, số tiết/tuần chia số ngày (tải ngày: định mức của giáo viên chia theo số tiết của ngày).</t>
+          <t>Trong một buổi (hoặc ngày, nếu Với mỗi có Ngày) tiết của Môn đứng trước (hoặc sau) tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm. So sánh: Trước, Sau.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="25" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: Tự ghép, cột Áp dụng khi</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Đi kèm</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Chỉ áp dụng khi số tiết/tuần của các môn ở cột Môn (phạm vi có Môn, Nhóm môn: của từng môn, nhóm môn) ở khối đó thỏa điều kiện, vd '&gt;= 6, chẵn' (từ 6 tiết trở lên và chẵn) hoặc '&lt;= số ngày' (không quá số ngày học).</t>
+          <t>Buổi (hoặc ngày) có tiết của Môn thì cũng có tiết của Môn thứ hai. Để trống Môn thứ hai và Với mỗi có Nhóm môn: các môn khác cùng nhóm.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="25" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>LUẬT: cấu trúc của TKB</t>
+          <t>LUẬT: Đi cùng nhau · Tự ghép, Phép đo Cùng giờ</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Cấu trúc của TKB (không phải luật, luôn có): mỗi lớp mỗi giờ học một tiết; mỗi lớp học đủ số tiết của chương trình học; giáo viên không dạy hai nơi cùng lúc, dạy không quá định mức (cộng số tiết bù tối đa ở chế độ bù giờ), Quản Lý dạy đúng định mức; giáo viên chỉ dạy các môn chức vụ được dạy (sheet CHƯƠNG TRÌNH HỌC, CHỨC VỤ).</t>
+          <t>Các tiết luôn học cùng giờ, cùng số tiết mỗi tuần; chỉ ghi Bắt buộc. Mỗi môn một người (để trống So sánh): mỗi lớp học Môn và Môn thứ hai cùng giờ, lớp tính một tiết ở giờ đó: lớp chia nhóm (mỗi nhóm học một môn, mỗi môn một người dạy) hoặc giáo viên chính và trợ giảng (ghi trợ giảng thành một môn riêng, vd Trợ giảng Tiếng Anh); Với mỗi là Lớp. Cùng một người: ghép lớp, các lớp (của cả trường, hoặc mỗi khối, mỗi cơ sở ở cột Với mỗi) học Môn (và Môn thứ hai nếu ghi) cùng giờ, một người dạy, người đó tính một tiết ở giờ đó. So sánh: Mỗi môn một người, Cùng một người.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="25" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
+          <t>LUẬT: Ai dạy · Tự ghép, Phép đo Người dạy</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Các tiết do giáo viên ghi ở cột Giáo viên (chức vụ, Mã GV hoặc họ tên) dạy; hoặc do cùng một người dạy; hoặc hai tiết liền nhau do cùng một người; hoặc tiết đầu tuần do giáo viên đó dạy, tiết của người khác không đứng trước. So sánh: Do, Cùng một người, Liền nhau cùng người, Tiết đầu tuần do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="25" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>LUẬT: Tự ghép, cột Số</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Một số nguyên, hoặc (phép đo Số tiết) một ngưỡng theo dữ liệu: tải ngày, tải ngày + 1, số tiết/tuần chia số ngày (tải ngày: định mức của giáo viên chia theo số tiết của ngày).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="25" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>LUẬT: Tự ghép, cột Áp dụng khi</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ áp dụng khi số tiết/tuần của các môn ở cột Môn (phạm vi có Môn, Nhóm môn: của từng môn, nhóm môn) ở khối đó thỏa điều kiện, vd '&gt;= 6, chẵn' (từ 6 tiết trở lên và chẵn) hoặc '&lt;= số ngày' (không quá số ngày học).</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="25" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>LUẬT: cấu trúc của TKB</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Cấu trúc của TKB (không phải luật, luôn có): mỗi lớp mỗi giờ học một tiết; mỗi lớp học đủ số tiết của chương trình học; giáo viên không dạy hai nơi cùng lúc, dạy không quá định mức (cộng số tiết bù tối đa ở chế độ bù giờ), Quản Lý dạy đúng định mức; giáo viên chỉ dạy các môn chức vụ được dạy (sheet CHƯƠNG TRÌNH HỌC, CHỨC VỤ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="25" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
           <t>Kiểu chữ</t>
         </is>
       </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>Các file kết quả chép kiểu chữ, cỡ chữ, viền của sheet NHÂN SỰ. Chỉ cần chữ và số: không cần công thức, màu nền, ghi chú trong ô hay danh sách thả xuống.</t>
         </is>

</xml_diff>

<commit_message>
Rules: pick a level instead of points, add rules as fill-in sentences
- Soft rules are written with a level word only; the Điểm column is left out
  of the template and the updated input unless a row has its own points.
  A built-in soft row at its default level keeps its tuned points
  (luat_co_san.tuned on read, plain on write), so rules and result codes
  are unchanged; old files with Điểm still read.
- Rules step: "Thêm luật" opens a list of common sentences; a preset opens
  as a fill-in sentence with the time picker below and optional filters
  folded; built-in rules open with only their free number and the level;
  the level is one select (Bắt buộc or Ưu tiên rất cao/cao/vừa/thấp).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SYSHWKNfUbV9f2WQ9CocTD
</commit_message>
<xml_diff>
--- a/data/Input_Template_V8.xlsx
+++ b/data/Input_Template_V8.xlsx
@@ -5510,7 +5510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X35"/>
+  <dimension ref="A1:W35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5534,8 +5534,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="9" customWidth="1" min="20" max="20"/>
     <col width="6" customWidth="1" min="21" max="21"/>
-    <col width="8" customWidth="1" min="22" max="22"/>
-    <col width="70" customWidth="1" min="23" max="23"/>
+    <col width="70" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -5646,15 +5645,10 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Điểm</t>
+          <t>Tạm tắt</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Tạm tắt</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Luật đọc là</t>
         </is>
@@ -5709,8 +5703,7 @@
       </c>
       <c r="U2" s="3" t="n"/>
       <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>Mỗi buổi, một lớp học tối đa 2 tiết của một môn, tính chung môn chính với môn tăng cường cùng nhóm (bắt buộc)</t>
         </is>
@@ -5773,8 +5766,7 @@
       </c>
       <c r="U3" s="3" t="n"/>
       <c r="V3" s="3" t="n"/>
-      <c r="W3" s="3" t="n"/>
-      <c r="X3" s="2" t="inlineStr">
+      <c r="W3" s="2" t="inlineStr">
         <is>
           <t>Mỗi ngày, một lớp học tối đa 1 tiết Toán, khi số tiết/tuần của môn không quá số ngày học (bắt buộc)</t>
         </is>
@@ -5831,8 +5823,7 @@
       </c>
       <c r="U4" s="3" t="n"/>
       <c r="V4" s="3" t="n"/>
-      <c r="W4" s="3" t="n"/>
-      <c r="X4" s="2" t="inlineStr">
+      <c r="W4" s="2" t="inlineStr">
         <is>
           <t>Môn có từ 6 tiết/tuần trở lên và số tiết chẵn, tính chung môn tăng cường cùng nhóm, học thành cặp 2 tiết liền trong buổi; trừ môn có nhãn Không ghép cặp (bắt buộc)</t>
         </is>
@@ -5881,8 +5872,7 @@
       </c>
       <c r="U5" s="3" t="n"/>
       <c r="V5" s="3" t="n"/>
-      <c r="W5" s="3" t="n"/>
-      <c r="X5" s="2" t="inlineStr">
+      <c r="W5" s="2" t="inlineStr">
         <is>
           <t>Các tiết của một môn trong cùng buổi phải đứng liền nhau (bắt buộc)</t>
         </is>
@@ -5939,8 +5929,7 @@
       </c>
       <c r="U6" s="3" t="n"/>
       <c r="V6" s="3" t="n"/>
-      <c r="W6" s="3" t="n"/>
-      <c r="X6" s="2" t="inlineStr">
+      <c r="W6" s="2" t="inlineStr">
         <is>
           <t>Trong một ngày, tiết môn tăng cường đứng sau các tiết môn chính cùng nhóm (bắt buộc)</t>
         </is>
@@ -5993,8 +5982,7 @@
       </c>
       <c r="U7" s="3" t="n"/>
       <c r="V7" s="3" t="n"/>
-      <c r="W7" s="3" t="n"/>
-      <c r="X7" s="2" t="inlineStr">
+      <c r="W7" s="2" t="inlineStr">
         <is>
           <t>Ngày có tiết môn tăng cường thì cũng có tiết môn chính cùng nhóm (bắt buộc)</t>
         </is>
@@ -6053,8 +6041,7 @@
       </c>
       <c r="U8" s="3" t="n"/>
       <c r="V8" s="3" t="n"/>
-      <c r="W8" s="3" t="n"/>
-      <c r="X8" s="2" t="inlineStr">
+      <c r="W8" s="2" t="inlineStr">
         <is>
           <t>Ở mỗi giờ có nhãn Tiết HĐTN cố định, mỗi lớp học đúng 1 tiết HĐTN (bắt buộc)</t>
         </is>
@@ -6107,8 +6094,7 @@
       </c>
       <c r="U9" s="3" t="n"/>
       <c r="V9" s="3" t="n"/>
-      <c r="W9" s="3" t="n"/>
-      <c r="X9" s="2" t="inlineStr">
+      <c r="W9" s="2" t="inlineStr">
         <is>
           <t>Tiết HĐTN chỉ xếp vào giờ có nhãn Tiết HĐTN cố định hoặc Xếp tiết HĐTN còn lại (bắt buộc)</t>
         </is>
@@ -6169,12 +6155,13 @@
           <t>Không</t>
         </is>
       </c>
-      <c r="U10" s="3" t="n"/>
-      <c r="V10" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="W10" s="3" t="n"/>
-      <c r="X10" s="2" t="inlineStr">
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="V10" s="3" t="n"/>
+      <c r="W10" s="2" t="inlineStr">
         <is>
           <t>Tiết HĐTN còn lại, ngoài giờ cố định, xếp ở tiết cuối buổi (ưu tiên thấp)</t>
         </is>
@@ -6231,8 +6218,7 @@
       </c>
       <c r="U11" s="3" t="n"/>
       <c r="V11" s="3" t="n"/>
-      <c r="W11" s="3" t="n"/>
-      <c r="X11" s="2" t="inlineStr">
+      <c r="W11" s="2" t="inlineStr">
         <is>
           <t>Ở giờ có nhãn Luôn do GVCN dạy, lớp học với GV chủ nhiệm (bắt buộc)</t>
         </is>
@@ -6289,8 +6275,7 @@
       </c>
       <c r="U12" s="3" t="n"/>
       <c r="V12" s="3" t="n"/>
-      <c r="W12" s="3" t="n"/>
-      <c r="X12" s="2" t="inlineStr">
+      <c r="W12" s="2" t="inlineStr">
         <is>
           <t>Môn có nhãn Chỉ GVCN dạy thì chỉ GV chủ nhiệm dạy (bắt buộc)</t>
         </is>
@@ -6343,8 +6328,7 @@
       </c>
       <c r="U13" s="3" t="n"/>
       <c r="V13" s="3" t="n"/>
-      <c r="W13" s="3" t="n"/>
-      <c r="X13" s="2" t="inlineStr">
+      <c r="W13" s="2" t="inlineStr">
         <is>
           <t>Hai tiết liền nhau của một môn (cùng nhóm) trong buổi do cùng một giáo viên dạy (bắt buộc)</t>
         </is>
@@ -6405,8 +6389,7 @@
       </c>
       <c r="U14" s="3" t="n"/>
       <c r="V14" s="3" t="n"/>
-      <c r="W14" s="3" t="n"/>
-      <c r="X14" s="2" t="inlineStr">
+      <c r="W14" s="2" t="inlineStr">
         <is>
           <t>Môn có nhãn GVCN nhận trọn: tiết đầu tuần của lớp do GV chủ nhiệm dạy, tiết của giáo viên khác không đứng trước (bắt buộc)</t>
         </is>
@@ -6447,8 +6430,7 @@
       </c>
       <c r="U15" s="3" t="n"/>
       <c r="V15" s="3" t="n"/>
-      <c r="W15" s="3" t="n"/>
-      <c r="X15" s="2" t="inlineStr">
+      <c r="W15" s="2" t="inlineStr">
         <is>
           <t>Giáo viên không dạy vào buổi nghỉ ghi ở cột Buổi Nghỉ và nghỉ đủ số buổi ghi ở đó (bắt buộc)</t>
         </is>
@@ -6507,8 +6489,7 @@
       </c>
       <c r="U16" s="3" t="n"/>
       <c r="V16" s="3" t="n"/>
-      <c r="W16" s="3" t="n"/>
-      <c r="X16" s="2" t="inlineStr">
+      <c r="W16" s="2" t="inlineStr">
         <is>
           <t>Mỗi buổi, một giáo viên chỉ dạy ở một cơ sở (bắt buộc)</t>
         </is>
@@ -6565,12 +6546,13 @@
           <t>Không</t>
         </is>
       </c>
-      <c r="U17" s="3" t="n"/>
-      <c r="V17" s="3" t="n">
-        <v>10000</v>
-      </c>
-      <c r="W17" s="3" t="n"/>
-      <c r="X17" s="2" t="inlineStr">
+      <c r="U17" s="3" t="inlineStr">
+        <is>
+          <t>Rất cao</t>
+        </is>
+      </c>
+      <c r="V17" s="3" t="n"/>
+      <c r="W17" s="2" t="inlineStr">
         <is>
           <t>Hạn chế để một giáo viên đổi cơ sở trong cùng một ngày (dạy ở hai cơ sở trở lên) (ưu tiên rất cao)</t>
         </is>
@@ -6611,8 +6593,7 @@
       </c>
       <c r="U18" s="3" t="n"/>
       <c r="V18" s="3" t="n"/>
-      <c r="W18" s="3" t="n"/>
-      <c r="X18" s="2" t="inlineStr">
+      <c r="W18" s="2" t="inlineStr">
         <is>
           <t>Giáo viên không chủ nhiệm ghi Cơ sở 2 hoặc Thai Sản chỉ dạy các lớp ở cơ sở 2 (bắt buộc)</t>
         </is>
@@ -6663,12 +6644,13 @@
           <t>Không</t>
         </is>
       </c>
-      <c r="U19" s="3" t="n"/>
-      <c r="V19" s="3" t="n">
-        <v>1200</v>
-      </c>
-      <c r="W19" s="3" t="n"/>
-      <c r="X19" s="2" t="inlineStr">
+      <c r="U19" s="3" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="V19" s="3" t="n"/>
+      <c r="W19" s="2" t="inlineStr">
         <is>
           <t>Tránh xếp môn có nhãn Môn nặng vào giờ có nhãn Hạn chế môn nặng (ưu tiên cao)</t>
         </is>
@@ -6723,12 +6705,13 @@
           <t>Không</t>
         </is>
       </c>
-      <c r="U20" s="3" t="n"/>
-      <c r="V20" s="3" t="n">
-        <v>300</v>
-      </c>
-      <c r="W20" s="3" t="n"/>
-      <c r="X20" s="2" t="inlineStr">
+      <c r="U20" s="3" t="inlineStr">
+        <is>
+          <t>Vừa</t>
+        </is>
+      </c>
+      <c r="V20" s="3" t="n"/>
+      <c r="W20" s="2" t="inlineStr">
         <is>
           <t>Môn có nhãn Ưu tiên buổi sáng xếp vào buổi sáng (ưu tiên vừa)</t>
         </is>
@@ -6783,12 +6766,13 @@
           <t>Không</t>
         </is>
       </c>
-      <c r="U21" s="3" t="n"/>
-      <c r="V21" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="W21" s="3" t="n"/>
-      <c r="X21" s="2" t="inlineStr">
+      <c r="U21" s="3" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="V21" s="3" t="n"/>
+      <c r="W21" s="2" t="inlineStr">
         <is>
           <t>Số tiết mỗi ngày của giáo viên không quá tải ngày, tức số tiết/tuần chia đều cho các ngày (ưu tiên thấp)</t>
         </is>
@@ -6843,12 +6827,13 @@
           <t>Không</t>
         </is>
       </c>
-      <c r="U22" s="3" t="n"/>
-      <c r="V22" s="3" t="n">
-        <v>300</v>
-      </c>
-      <c r="W22" s="3" t="n"/>
-      <c r="X22" s="2" t="inlineStr">
+      <c r="U22" s="3" t="inlineStr">
+        <is>
+          <t>Vừa</t>
+        </is>
+      </c>
+      <c r="V22" s="3" t="n"/>
+      <c r="W22" s="2" t="inlineStr">
         <is>
           <t>Số tiết mỗi ngày của giáo viên không quá tải ngày + 1 tiết (ưu tiên vừa)</t>
         </is>
@@ -6907,12 +6892,13 @@
           <t>Không</t>
         </is>
       </c>
-      <c r="U23" s="3" t="n"/>
-      <c r="V23" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="W23" s="3" t="n"/>
-      <c r="X23" s="2" t="inlineStr">
+      <c r="U23" s="3" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="V23" s="3" t="n"/>
+      <c r="W23" s="2" t="inlineStr">
         <is>
           <t>Mỗi môn, trừ HĐTN và môn ưu tiên buổi sáng, rải đều trong tuần: một ngày không quá số tiết/tuần chia số ngày (ưu tiên thấp)</t>
         </is>
@@ -6975,12 +6961,13 @@
           <t>Không</t>
         </is>
       </c>
-      <c r="U24" s="3" t="n"/>
-      <c r="V24" s="3" t="n">
-        <v>120</v>
-      </c>
-      <c r="W24" s="3" t="n"/>
-      <c r="X24" s="2" t="inlineStr">
+      <c r="U24" s="3" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="V24" s="3" t="n"/>
+      <c r="W24" s="2" t="inlineStr">
         <is>
           <t>Môn ưu tiên buổi sáng rải đều trong tuần: một ngày không quá số tiết/tuần chia số ngày (ưu tiên thấp)</t>
         </is>
@@ -7037,12 +7024,13 @@
           <t>Không</t>
         </is>
       </c>
-      <c r="U25" s="3" t="n"/>
-      <c r="V25" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="W25" s="3" t="n"/>
-      <c r="X25" s="2" t="inlineStr">
+      <c r="U25" s="3" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="V25" s="3" t="n"/>
+      <c r="W25" s="2" t="inlineStr">
         <is>
           <t>Giáo viên, trừ GV chủ nhiệm, không có tiết trống xen giữa các tiết trong buổi (ưu tiên thấp)</t>
         </is>
@@ -7071,8 +7059,7 @@
       <c r="T26" s="3" t="n"/>
       <c r="U26" s="3" t="n"/>
       <c r="V26" s="3" t="n"/>
-      <c r="W26" s="3" t="n"/>
-      <c r="X26" s="2" t="n"/>
+      <c r="W26" s="2" t="n"/>
     </row>
     <row r="27" ht="25" customHeight="1">
       <c r="A27" s="2" t="n"/>
@@ -7097,8 +7084,7 @@
       <c r="T27" s="3" t="n"/>
       <c r="U27" s="3" t="n"/>
       <c r="V27" s="3" t="n"/>
-      <c r="W27" s="3" t="n"/>
-      <c r="X27" s="2" t="n"/>
+      <c r="W27" s="2" t="n"/>
     </row>
     <row r="28" ht="25" customHeight="1">
       <c r="A28" s="2" t="n"/>
@@ -7123,8 +7109,7 @@
       <c r="T28" s="3" t="n"/>
       <c r="U28" s="3" t="n"/>
       <c r="V28" s="3" t="n"/>
-      <c r="W28" s="3" t="n"/>
-      <c r="X28" s="2" t="n"/>
+      <c r="W28" s="2" t="n"/>
     </row>
     <row r="29" ht="25" customHeight="1">
       <c r="A29" s="2" t="n"/>
@@ -7149,8 +7134,7 @@
       <c r="T29" s="3" t="n"/>
       <c r="U29" s="3" t="n"/>
       <c r="V29" s="3" t="n"/>
-      <c r="W29" s="3" t="n"/>
-      <c r="X29" s="2" t="n"/>
+      <c r="W29" s="2" t="n"/>
     </row>
     <row r="30" ht="25" customHeight="1">
       <c r="A30" s="2" t="n"/>
@@ -7175,8 +7159,7 @@
       <c r="T30" s="3" t="n"/>
       <c r="U30" s="3" t="n"/>
       <c r="V30" s="3" t="n"/>
-      <c r="W30" s="3" t="n"/>
-      <c r="X30" s="2" t="n"/>
+      <c r="W30" s="2" t="n"/>
     </row>
     <row r="31" ht="25" customHeight="1">
       <c r="A31" s="2" t="n"/>
@@ -7201,8 +7184,7 @@
       <c r="T31" s="3" t="n"/>
       <c r="U31" s="3" t="n"/>
       <c r="V31" s="3" t="n"/>
-      <c r="W31" s="3" t="n"/>
-      <c r="X31" s="2" t="n"/>
+      <c r="W31" s="2" t="n"/>
     </row>
     <row r="32" ht="25" customHeight="1">
       <c r="A32" s="2" t="n"/>
@@ -7227,8 +7209,7 @@
       <c r="T32" s="3" t="n"/>
       <c r="U32" s="3" t="n"/>
       <c r="V32" s="3" t="n"/>
-      <c r="W32" s="3" t="n"/>
-      <c r="X32" s="2" t="n"/>
+      <c r="W32" s="2" t="n"/>
     </row>
     <row r="33" ht="25" customHeight="1">
       <c r="A33" s="2" t="n"/>
@@ -7253,8 +7234,7 @@
       <c r="T33" s="3" t="n"/>
       <c r="U33" s="3" t="n"/>
       <c r="V33" s="3" t="n"/>
-      <c r="W33" s="3" t="n"/>
-      <c r="X33" s="2" t="n"/>
+      <c r="W33" s="2" t="n"/>
     </row>
     <row r="34" ht="25" customHeight="1">
       <c r="A34" s="2" t="n"/>
@@ -7279,8 +7259,7 @@
       <c r="T34" s="3" t="n"/>
       <c r="U34" s="3" t="n"/>
       <c r="V34" s="3" t="n"/>
-      <c r="W34" s="3" t="n"/>
-      <c r="X34" s="2" t="n"/>
+      <c r="W34" s="2" t="n"/>
     </row>
     <row r="35" ht="25" customHeight="1">
       <c r="A35" s="2" t="n"/>
@@ -7305,8 +7284,7 @@
       <c r="T35" s="3" t="n"/>
       <c r="U35" s="3" t="n"/>
       <c r="V35" s="3" t="n"/>
-      <c r="W35" s="3" t="n"/>
-      <c r="X35" s="2" t="n"/>
+      <c r="W35" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7886,7 +7864,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Mọi luật xếp TKB, mỗi dòng một luật, đọc như một câu: Với mỗi [cột Với mỗi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Mỗi luật trả lời một trong bốn câu hỏi: Ở đâu, Bao nhiêu, Đi cùng nhau, Ai dạy (các kiểu luật và phép đo xếp theo câu hỏi ở dưới). File mẫu ghi sẵn các luật có sẵn của chương trình: sửa số hoặc Điểm để chỉnh, đổi Bắt buộc, xóa dòng để bỏ luật (hoặc ghi Có ở cột Tạm tắt: chương trình bỏ qua dòng đó mà vẫn giữ lại, xóa chữ Có là dùng lại), thêm dòng để có luật mới. Cột Nhóm và Luật đọc là chỉ để đọc (chương trình ghi lại mỗi lần). Kiểu luật: một mẫu hoặc Tự ghép; cột kiểu luật không dùng để trống. Bắt buộc: Có (luật cứng) hoặc Không (ưu tiên); luật ưu tiên ghi Mức Thấp, Vừa, Cao, Rất cao (100, 400, 1500, 5000 điểm) hoặc ghi thẳng Điểm (điểm trừ mỗi lần không theo). Môn, Lớp, Khối, Ngày, Tiết ghi danh sách cách nhau bằng dấu phẩy hoặc khoảng, vd 3, 4 hoặc 3-5; Thứ 2, Thứ 4 hoặc T2-T4; 5-7. Buổi: Sáng hoặc Chiều. Giáo viên: chức vụ (Chủ Nhiệm, Bộ Môn, Quản Lý hoặc chức vụ GV chuyên biệt), 'trừ Chủ Nhiệm' là mọi giáo viên trừ chức vụ đó; hoặc một người: Mã GV (vd Bộ Môn 3, Chủ Nhiệm 1/1, đánh số theo thứ tự dòng của sheet NHÂN SỰ) hay họ tên (hai người trùng tên thì ghi Mã GV), vd giờ bận: Không xếp vào, Giáo viên Bộ Môn 3, Thứ 2, tiết 1 (để trống Môn); ép phân công: Chỉ giáo viên dạy, Môn Tiếng Anh, Lớp 3/1, Giáo viên Tiếng Anh 2. Câu đọc lại ghi Mã GV, không ghi họ tên. Nhãn, Trừ nhãn: tên các cột Có/Không của môn (vd Môn nặng) hoặc của giờ học (ngày, tiết, vd Luôn do GVCN dạy); nhiều nhãn giờ học là giờ có một trong các nhãn. Gồm môn tăng cường: Có thì Môn tính cả các môn tăng cường cùng nhóm. Không có sheet này thì chương trình dùng các luật có sẵn và sheet LUẬT RIÊNG (file của bản trước).</t>
+          <t>Mọi luật xếp TKB, mỗi dòng một luật, đọc như một câu: Với mỗi [cột Với mỗi] · các tiết [Môn, Nhãn, Khối, Lớp, Ngày, Tiết, Buổi, Giáo viên] · thì [Phép đo] [So sánh] [Số] · khi [Áp dụng khi]. Mỗi luật trả lời một trong bốn câu hỏi: Ở đâu, Bao nhiêu, Đi cùng nhau, Ai dạy (các kiểu luật và phép đo xếp theo câu hỏi ở dưới). File mẫu ghi sẵn các luật có sẵn của chương trình: sửa số hoặc Mức để chỉnh, đổi Bắt buộc, xóa dòng để bỏ luật (hoặc ghi Có ở cột Tạm tắt: chương trình bỏ qua dòng đó mà vẫn giữ lại, xóa chữ Có là dùng lại), thêm dòng để có luật mới. Cột Nhóm và Luật đọc là chỉ để đọc (chương trình ghi lại mỗi lần). Kiểu luật: một mẫu hoặc Tự ghép; cột kiểu luật không dùng để trống. Bắt buộc: Có (luật cứng) hoặc Không (ưu tiên); luật ưu tiên chọn Mức Thấp, Vừa, Cao, Rất cao (100, 400, 1500, 5000 điểm trừ mỗi lần không theo; luật có sẵn để nguyên mức mặc định thì dùng điểm đã chỉnh sẵn của luật đó). File cũ có cột Điểm (điểm trừ ghi thẳng) vẫn đọc được. Môn, Lớp, Khối, Ngày, Tiết ghi danh sách cách nhau bằng dấu phẩy hoặc khoảng, vd 3, 4 hoặc 3-5; Thứ 2, Thứ 4 hoặc T2-T4; 5-7. Buổi: Sáng hoặc Chiều. Giáo viên: chức vụ (Chủ Nhiệm, Bộ Môn, Quản Lý hoặc chức vụ GV chuyên biệt), 'trừ Chủ Nhiệm' là mọi giáo viên trừ chức vụ đó; hoặc một người: Mã GV (vd Bộ Môn 3, Chủ Nhiệm 1/1, đánh số theo thứ tự dòng của sheet NHÂN SỰ) hay họ tên (hai người trùng tên thì ghi Mã GV), vd giờ bận: Không xếp vào, Giáo viên Bộ Môn 3, Thứ 2, tiết 1 (để trống Môn); ép phân công: Chỉ giáo viên dạy, Môn Tiếng Anh, Lớp 3/1, Giáo viên Tiếng Anh 2. Câu đọc lại ghi Mã GV, không ghi họ tên. Nhãn, Trừ nhãn: tên các cột Có/Không của môn (vd Môn nặng) hoặc của giờ học (ngày, tiết, vd Luôn do GVCN dạy); nhiều nhãn giờ học là giờ có một trong các nhãn. Gồm môn tăng cường: Có thì Môn tính cả các môn tăng cường cùng nhóm. Không có sheet này thì chương trình dùng các luật có sẵn và sheet LUẬT RIÊNG (file của bản trước).</t>
         </is>
       </c>
     </row>

</xml_diff>